<commit_message>
sheet formation in the final output
</commit_message>
<xml_diff>
--- a/SINGLE HADITH CONTENT/BOOK WISE FINAL UPDATED CONTENT/BN/BN_100 HADITH.xlsx
+++ b/SINGLE HADITH CONTENT/BOOK WISE FINAL UPDATED CONTENT/BN/BN_100 HADITH.xlsx
@@ -460,7 +460,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঘুমের আগে ওজু ও ডান কাতে শোয়ার সুন্নাহ","description":"$book_name$ $hadith_number$ - $chapter_name$. ঘুমের আগে নামাজের মতো ওজু করে ডান কাতে শোয়া রাসূল صلى الله عليه وسلم-এর শেখানো সুন্দর আদব।"},"heading":{"title":"ঘুমের আগে ওজু: ডান কাতে শোয়ার নববী সুন্নাহ","description":"এই হাদিসে ঘুমের আগে ওজু করার সুন্নাহ এবং ডান কাতে শোয়ার আদব শেখানো হয়েছে। নবী করীম সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বারা ইবনে আ’যেব (রাঃ)-কে বলেছেন, যখন শয্যা গ্রহণের ইচ্ছা করবে, তখন নামাজের মতো ওজু করবে এবং ডান কাতে শোবে। এখানে খুব সহজ একটি রাতের আমল বলা হয়েছে। মানুষ ঘুমের আগে দিনের কাজ শেষ করে বিশ্রামে যায়। সেই সময় নিজেকে পবিত্র অবস্থায় রাখা এবং নবীজির শেখানো ভঙ্গিতে শোয়া মুমিনের জীবনে সুন্নাহর ভালো চর্চা। এই হাদিস থেকে বোঝা যায়, ইসলাম শুধু নামাজের সময়ের আদব শেখায় না; ঘুমের মতো সাধারণ কাজেও সুন্দর পথ দেখায়। তাই ঘুমের দোয়া, ওজু করে ঘুমানো এবং ডান কাতে শোয়া—এসব বিষয় মুসলিম জীবনের সহজ কিন্তু মূল্যবান আমল।"},"teachings":["ঘুমের আগে নামাজের মতো ওজু করা নবী صلى الله عليه وسلم-এর শেখানো আদব।","ডান কাতে শোয়া শয্যা গ্রহণের সুন্নতি ভঙ্গি।","দৈনন্দিন কাজেও সুন্নাহ অনুসরণের সুযোগ আছে।","ঘুমের আগে পবিত্রতার প্রতি যত্ন নেওয়া মুমিনের ভালো অভ্যাস।"],"related_hadiths":[{"id":"5017","book_id":"1","label":"Sahih Bukhari"},{"id":"631৮","book_id":"1","label":"Sahih Bukhari"},{"id":"1154","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঘুমের আগে ওজু ও ডান কাতে শোয়ার সুন্নাহ","description":"$book_name$ $hadith_number$ - $chapter_name$. ঘুমের আগে নামাজের মতো ওজু করে ডান কাতে শোয়া রাসূল صلى الله عليه وسلم-এর শেখানো সুন্দর আদব।"},"heading":{"title":"ঘুমের আগে ওজু: ডান কাতে শোয়ার নববী সুন্নাহ","description":"এই হাদিসে ঘুমের আগে ওজু করার সুন্নাহ এবং ডান কাতে শোয়ার আদব শেখানো হয়েছে। নবী করীম সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বারা ইবনে আ’যেব (রাঃ)-কে বলেছেন, যখন শয্যা গ্রহণের ইচ্ছা করবে, তখন নামাজের মতো ওজু করবে এবং ডান কাতে শোবে। এখানে খুব সহজ একটি রাতের আমল বলা হয়েছে। মানুষ ঘুমের আগে দিনের কাজ শেষ করে বিশ্রামে যায়। সেই সময় নিজেকে পবিত্র অবস্থায় রাখা এবং নবীজির শেখানো ভঙ্গিতে শোয়া মুমিনের জীবনে সুন্নাহর ভালো চর্চা। এই হাদিস থেকে বোঝা যায়, ইসলাম শুধু নামাজের সময়ের আদব শেখায় না; ঘুমের মতো সাধারণ কাজেও সুন্দর পথ দেখায়। তাই ঘুমের দোয়া, ওজু করে ঘুমানো এবং ডান কাতে শোয়া—এসব বিষয় মুসলিম জীবনের সহজ কিন্তু মূল্যবান আমল।"},"teachings":["ঘুমের আগে নামাজের মতো ওজু করা নবী صلى الله عليه وسلم-এর শেখানো আদব।","ডান কাতে শোয়া শয্যা গ্রহণের সুন্নতি ভঙ্গি।","দৈনন্দিন কাজেও সুন্নাহ অনুসরণের সুযোগ আছে।","ঘুমের আগে পবিত্রতার প্রতি যত্ন নেওয়া মুমিনের ভালো অভ্যাস।"],"related_hadiths":[{"id":"5017","book_id":"1","label":"Sahih Bukhari"},{"id":"6318","book_id":"1","label":"Sahih Bukhari"},{"id":"1154","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | অল্প হলেও নিয়মিত আমলের মর্যাদা","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহর কাছে প্রিয় আমল হলো যা অব্যাহত রাখা হয়, যদিও তা পরিমাণে অল্প হয়।"},"heading":{"title":"নিয়মিত আমল: অল্প হলেও অব্যাহত রাখার হাদিস","description":"এই হাদিসে আমলের ধারাবাহিকতার গুরুত্ব এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামকে জিজ্ঞেস করা হলো, কোন আমল আল্লাহর কাছে বেশি প্রিয়। তিনি বললেন, যে আমল অব্যাহত রাখা হয়, যদিও তা অল্প হয়। এখানে শিক্ষা খুব বাস্তব। অনেক মানুষ বড় আমল শুরু করে, কিন্তু ধরে রাখতে পারে না। হাদিস শেখায়, কম হলেও নিয়মিত আমল আল্লাহর কাছে প্রিয় হতে পারে। নিয়মিত আমল হাদিস, অল্প আমল এবং ধারাবাহিক ইবাদত—এই বিষয়গুলো এখানে প্রধান। এতে অলসতা বা অতিরিক্ত চাপ দুই দিক থেকেই ভারসাম্য শেখা যায়। একজন মুসলিম নিজের সামর্থ্য অনুযায়ী এমন আমল বেছে নিতে পারে, যা সে ধারাবাহিকভাবে করতে পারে। স্থায়ী অভ্যাস গড়াই এখানে মূল শিক্ষা।"},"teachings":["অল্প আমল হলেও নিয়মিত রাখা গুরুত্বপূর্ণ।","আল্লাহর কাছে প্রিয় আমলের একটি গুণ হলো ধারাবাহিকতা।","নিজের সামর্থ্য অনুযায়ী আমল বেছে নেওয়া উচিত।","বড় শুরু করে ছেড়ে দেওয়ার চেয়ে ছোট আমল ধরে রাখা ভালো হতে পারে।"],"related_hadiths":[{"id":"6464","book_id":"1","label":"Sahih Bukhari"},{"id":"7৮2","book_id":"2","label":"Sahih Muslim"},{"id":"43","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | অল্প হলেও নিয়মিত আমলের মর্যাদা","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহর কাছে প্রিয় আমল হলো যা অব্যাহত রাখা হয়, যদিও তা পরিমাণে অল্প হয়।"},"heading":{"title":"নিয়মিত আমল: অল্প হলেও অব্যাহত রাখার হাদিস","description":"এই হাদিসে আমলের ধারাবাহিকতার গুরুত্ব এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামকে জিজ্ঞেস করা হলো, কোন আমল আল্লাহর কাছে বেশি প্রিয়। তিনি বললেন, যে আমল অব্যাহত রাখা হয়, যদিও তা অল্প হয়। এখানে শিক্ষা খুব বাস্তব। অনেক মানুষ বড় আমল শুরু করে, কিন্তু ধরে রাখতে পারে না। হাদিস শেখায়, কম হলেও নিয়মিত আমল আল্লাহর কাছে প্রিয় হতে পারে। নিয়মিত আমল হাদিস, অল্প আমল এবং ধারাবাহিক ইবাদত—এই বিষয়গুলো এখানে প্রধান। এতে অলসতা বা অতিরিক্ত চাপ দুই দিক থেকেই ভারসাম্য শেখা যায়। একজন মুসলিম নিজের সামর্থ্য অনুযায়ী এমন আমল বেছে নিতে পারে, যা সে ধারাবাহিকভাবে করতে পারে। স্থায়ী অভ্যাস গড়াই এখানে মূল শিক্ষা।"},"teachings":["অল্প আমল হলেও নিয়মিত রাখা গুরুত্বপূর্ণ।","আল্লাহর কাছে প্রিয় আমলের একটি গুণ হলো ধারাবাহিকতা।","নিজের সামর্থ্য অনুযায়ী আমল বেছে নেওয়া উচিত।","বড় শুরু করে ছেড়ে দেওয়ার চেয়ে ছোট আমল ধরে রাখা ভালো হতে পারে।"],"related_hadiths":[{"id":"6464","book_id":"1","label":"Sahih Bukhari"},{"id":"782","book_id":"2","label":"Sahih Muslim"},{"id":"43","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আল্লাহর নৈকট্য লাভের পথ","description":"$book_name$ $hadith_number$ - $chapter_name$. ফরয আমল ও নফল ইবাদতের মাধ্যমে আল্লাহর নৈকট্য, ভালোবাসা ও আশ্রয় লাভের গুরুত্বপূর্ণ শিক্ষা।"},"heading":{"title":"আল্লাহর নৈকট্য লাভ: ফরয ও নফল ইবাদতের গুরুত্ব","description":"এই হাদিসে আল্লাহর নৈকট্য লাভের পথ খুব স্পষ্টভাবে বলা হয়েছে। প্রথম শিক্ষা হলো, আল্লাহর অলীর সঙ্গে শত্রুতা করা ভয়াবহ বিষয়। আল্লাহ তা’আলা নিজেই বলেন, যে তাঁর অলীর সঙ্গে শত্রুতা করে, তার বিরুদ্ধে তিনি যুদ্ধ ঘোষণা করেন। এরপর হাদিসে বান্দার আমলের ধারাও পরিষ্কার করা হয়েছে। বান্দা আল্লাহর কাছে সবচেয়ে বেশি নিকটবর্তী হয় সেই ফরয আমলগুলোর মাধ্যমে, যা আল্লাহ তার ওপর ফরয করেছেন। তাই নামাজ, রোজা ও অন্যান্য ফরয ইবাদতকে অবহেলা করা যাবে না। এরপর নফল ইবাদত বান্দাকে আরও কাছে নিয়ে যায়। নফল কাজ করতে করতে বান্দা আল্লাহর ভালোবাসা লাভের পথে এগোয়। হাদিসে আরও বলা হয়েছে, আল্লাহ যখন বান্দাকে ভালোবাসেন, তখন তার শোনা, দেখা, ধরা ও চলার কাজে বিশেষ হিদায়াত ও সাহায্য দেন। বান্দা চাইলে তিনি দেন, আশ্রয় চাইলে আশ্রয় দেন। তাই এই হাদিস আমাদের শেখায়—ফরয আমল ঠিক রাখা, নফল ইবাদতে আগ্রহী হওয়া এবং আল্লাহর প্রিয় বান্দাদের সম্মান করা মুমিনের জীবনের বড় শিক্ষা।"},"teachings":["আল্লাহর অলীর সঙ্গে শত্রুতা করা খুব গুরুতর বিষয়।","আল্লাহর নৈকট্য লাভের প্রধান পথ হলো ফরয আমল ঠিকভাবে পালন করা।","নফল ইবাদত বান্দাকে আল্লাহর ভালোবাসার দিকে এগিয়ে নেয়।","আল্লাহর কাছে দোয়া করা ও আশ্রয় চাওয়া মুমিনের জন্য বড় ভরসার বিষয়।"],"related_hadiths":[{"id":"320৯","book_id":"1","label":"Sahih Bukhari"},{"id":"6507","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আল্লাহর নৈকট্য লাভের পথ","description":"$book_name$ $hadith_number$ - $chapter_name$. ফরয আমল ও নফল ইবাদতের মাধ্যমে আল্লাহর নৈকট্য, ভালোবাসা ও আশ্রয় লাভের গুরুত্বপূর্ণ শিক্ষা।"},"heading":{"title":"আল্লাহর নৈকট্য লাভ: ফরয ও নফল ইবাদতের গুরুত্ব","description":"এই হাদিসে আল্লাহর নৈকট্য লাভের পথ খুব স্পষ্টভাবে বলা হয়েছে। প্রথম শিক্ষা হলো, আল্লাহর অলীর সঙ্গে শত্রুতা করা ভয়াবহ বিষয়। আল্লাহ তা’আলা নিজেই বলেন, যে তাঁর অলীর সঙ্গে শত্রুতা করে, তার বিরুদ্ধে তিনি যুদ্ধ ঘোষণা করেন। এরপর হাদিসে বান্দার আমলের ধারাও পরিষ্কার করা হয়েছে। বান্দা আল্লাহর কাছে সবচেয়ে বেশি নিকটবর্তী হয় সেই ফরয আমলগুলোর মাধ্যমে, যা আল্লাহ তার ওপর ফরয করেছেন। তাই নামাজ, রোজা ও অন্যান্য ফরয ইবাদতকে অবহেলা করা যাবে না। এরপর নফল ইবাদত বান্দাকে আরও কাছে নিয়ে যায়। নফল কাজ করতে করতে বান্দা আল্লাহর ভালোবাসা লাভের পথে এগোয়। হাদিসে আরও বলা হয়েছে, আল্লাহ যখন বান্দাকে ভালোবাসেন, তখন তার শোনা, দেখা, ধরা ও চলার কাজে বিশেষ হিদায়াত ও সাহায্য দেন। বান্দা চাইলে তিনি দেন, আশ্রয় চাইলে আশ্রয় দেন। তাই এই হাদিস আমাদের শেখায়—ফরয আমল ঠিক রাখা, নফল ইবাদতে আগ্রহী হওয়া এবং আল্লাহর প্রিয় বান্দাদের সম্মান করা মুমিনের জীবনের বড় শিক্ষা।"},"teachings":["আল্লাহর অলীর সঙ্গে শত্রুতা করা খুব গুরুতর বিষয়।","আল্লাহর নৈকট্য লাভের প্রধান পথ হলো ফরয আমল ঠিকভাবে পালন করা।","নফল ইবাদত বান্দাকে আল্লাহর ভালোবাসার দিকে এগিয়ে নেয়।","আল্লাহর কাছে দোয়া করা ও আশ্রয় চাওয়া মুমিনের জন্য বড় ভরসার বিষয়।"],"related_hadiths":[{"id":"3209","book_id":"1","label":"Sahih Bukhari"},{"id":"6507","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আযানের জবাব, দরূদ ও দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. আযান শুনে জবাব দেওয়া, নবী صلى الله عليه وسلم-এর ওপর দরূদ পড়া ও নির্দিষ্ট দোয়ার ফজিলত।"},"heading":{"title":"আযানের জবাব: দরূদ ও দোয়ার সহজ সুন্নাহ","description":"এই হাদিসে আযান শুনলে কী করতে হবে, তা শেখানো হয়েছে। নবী করীম সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, যখন তোমরা মুআযযিনের আযান শুনবে, তখন তার মতো বলবে। এরপর তাঁর ওপর দরূদ পাঠ করবে। কারণ, যে ব্যক্তি নবী صلى الله عليه وسلم-এর ওপর একবার দরূদ পাঠ করে, তার ওপর আল্লাহ দশটি রহমত বর্ষণ করেন। এরপর আযানের পরের দোয়াও এসেছে, যেখানে আল্লাহর কাছে নবী মুহাম্মাদ صلى الله عليه وسلم-এর জন্য সম্মান, উচ্চ মর্যাদা এবং মাকামে মাহমুদ চাওয়া হয়। হাদিসে আরও বলা হয়েছে, যে ব্যক্তি এই দোয়া পড়বে, তার জন্য নবী صلى الله عليه وسلم-এর সুপারিশ ওয়াজিব হয়ে যাবে। আযানের জবাব, দরূদ শরীফ এবং আযানের পর দোয়া—এই তিনটি আমল এখানে খুব সুন্দরভাবে একসঙ্গে এসেছে।"},"teachings":["আযান শুনে মুআযযিনের কথার মতো জবাব দেওয়া উচিত।","আযানের পর নবী صلى الله عليه وسلم-এর ওপর দরূদ পাঠ করার শিক্ষা আছে।","একবার দরূদ পাঠে আল্লাহর দশ রহমতের কথা হাদিসে এসেছে।","আযানের পর নির্দিষ্ট দোয়া পড়ার ফজিলত বর্ণিত হয়েছে।"],"related_hadiths":[{"id":"611","book_id":"1","label":"Sahih Bukhari"},{"id":"614","book_id":"1","label":"Sahih Bukhari"},{"id":"3৮5","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আযানের জবাব, দরূদ ও দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. আযান শুনে জবাব দেওয়া, নবী صلى الله عليه وسلم-এর ওপর দরূদ পড়া ও নির্দিষ্ট দোয়ার ফজিলত।"},"heading":{"title":"আযানের জবাব: দরূদ ও দোয়ার সহজ সুন্নাহ","description":"এই হাদিসে আযান শুনলে কী করতে হবে, তা শেখানো হয়েছে। নবী করীম সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, যখন তোমরা মুআযযিনের আযান শুনবে, তখন তার মতো বলবে। এরপর তাঁর ওপর দরূদ পাঠ করবে। কারণ, যে ব্যক্তি নবী صلى الله عليه وسلم-এর ওপর একবার দরূদ পাঠ করে, তার ওপর আল্লাহ দশটি রহমত বর্ষণ করেন। এরপর আযানের পরের দোয়াও এসেছে, যেখানে আল্লাহর কাছে নবী মুহাম্মাদ صلى الله عليه وسلم-এর জন্য সম্মান, উচ্চ মর্যাদা এবং মাকামে মাহমুদ চাওয়া হয়। হাদিসে আরও বলা হয়েছে, যে ব্যক্তি এই দোয়া পড়বে, তার জন্য নবী صلى الله عليه وسلم-এর সুপারিশ ওয়াজিব হয়ে যাবে। আযানের জবাব, দরূদ শরীফ এবং আযানের পর দোয়া—এই তিনটি আমল এখানে খুব সুন্দরভাবে একসঙ্গে এসেছে।"},"teachings":["আযান শুনে মুআযযিনের কথার মতো জবাব দেওয়া উচিত।","আযানের পর নবী صلى الله عليه وسلم-এর ওপর দরূদ পাঠ করার শিক্ষা আছে।","একবার দরূদ পাঠে আল্লাহর দশ রহমতের কথা হাদিসে এসেছে।","আযানের পর নির্দিষ্ট দোয়া পড়ার ফজিলত বর্ণিত হয়েছে।"],"related_hadiths":[{"id":"611","book_id":"1","label":"Sahih Bukhari"},{"id":"614","book_id":"1","label":"Sahih Bukhari"},{"id":"385","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আগে আগে নামাজে আসার ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. নামাজে আগে আসার ফজিলত জানা থাকলে মানুষ আগেভাগে মসজিদে আসতে আগ্রহী হতো।"},"heading":{"title":"আগে আগে নামাজে আসা: জামাতের প্রতি আগ্রহের শিক্ষা","description":"এই হাদিসে নামাজে আগে আগে আসার ফজিলত সম্পর্কে বলা হয়েছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, মানুষ যদি অগ্রিম নামাজে আসার ফজিলত কত বেশি জানত, তাহলে অবশ্যই তারা আগেই নামাজের জন্য আসত। এখানে নামাজের সময় উপস্থিত হওয়ার আগ্রহ বাড়ানোর শিক্ষা আছে। নামাজ শুরু হওয়ার ঠিক আগে তাড়াহুড়া করা নয়; বরং আগেভাগে প্রস্তুত হয়ে আসা মুমিনের সুন্দর অভ্যাস। এই হাদিসে নির্দিষ্ট কোনো অতিরিক্ত কাজের কথা নেই; মূল কথা হলো, নামাজের জন্য আগে আসার মর্যাদা। যারা জামাতে নামাজ, মসজিদে আগে আসা এবং নামাজের ফজিলত জানতে চান, তাদের জন্য এই হাদিস খুব প্রাসঙ্গিক। এটি আমাদের শেখায়, নামাজকে দিনের কাজের শেষে রাখা নয়; বরং গুরুত্ব দিয়ে আগে থেকে প্রস্তুত হওয়া দরকার।"},"teachings":["নামাজের জন্য আগে আসার ফজিলত হাদিসে উল্লেখ আছে।","জামাতে নামাজের প্রতি আগ্রহী হওয়া উচিত।","নামাজকে গুরুত্ব দিয়ে আগে থেকে প্রস্তুতি নেওয়া ভালো।","ফজিলত জানা মানুষকে ভালো আমলে উৎসাহিত করে।"],"related_hadiths":[{"id":"251","book_id":"2","label":"Sahih Muslim"},{"id":"৯0৮","book_id":"1","label":"Sahih Bukhari"},{"id":"602","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আগে আগে নামাজে আসার ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. নামাজে আগে আসার ফজিলত জানা থাকলে মানুষ আগেভাগে মসজিদে আসতে আগ্রহী হতো।"},"heading":{"title":"আগে আগে নামাজে আসা: জামাতের প্রতি আগ্রহের শিক্ষা","description":"এই হাদিসে নামাজে আগে আগে আসার ফজিলত সম্পর্কে বলা হয়েছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, মানুষ যদি অগ্রিম নামাজে আসার ফজিলত কত বেশি জানত, তাহলে অবশ্যই তারা আগেই নামাজের জন্য আসত। এখানে নামাজের সময় উপস্থিত হওয়ার আগ্রহ বাড়ানোর শিক্ষা আছে। নামাজ শুরু হওয়ার ঠিক আগে তাড়াহুড়া করা নয়; বরং আগেভাগে প্রস্তুত হয়ে আসা মুমিনের সুন্দর অভ্যাস। এই হাদিসে নির্দিষ্ট কোনো অতিরিক্ত কাজের কথা নেই; মূল কথা হলো, নামাজের জন্য আগে আসার মর্যাদা। যারা জামাতে নামাজ, মসজিদে আগে আসা এবং নামাজের ফজিলত জানতে চান, তাদের জন্য এই হাদিস খুব প্রাসঙ্গিক। এটি আমাদের শেখায়, নামাজকে দিনের কাজের শেষে রাখা নয়; বরং গুরুত্ব দিয়ে আগে থেকে প্রস্তুত হওয়া দরকার।"},"teachings":["নামাজের জন্য আগে আসার ফজিলত হাদিসে উল্লেখ আছে।","জামাতে নামাজের প্রতি আগ্রহী হওয়া উচিত।","নামাজকে গুরুত্ব দিয়ে আগে থেকে প্রস্তুতি নেওয়া ভালো।","ফজিলত জানা মানুষকে ভালো আমলে উৎসাহিত করে।"],"related_hadiths":[{"id":"251","book_id":"2","label":"Sahih Muslim"},{"id":"908","book_id":"1","label":"Sahih Bukhari"},{"id":"602","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সুন্দর ওজু, মসজিদে পদচারণা ও নামাজের অপেক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. কষ্টের সময় সুন্দর ওজু, মসজিদে যাওয়া ও নামাজের অপেক্ষা গোনাহ মাফের কারণ।"},"heading":{"title":"সুন্দর ওজু ও মসজিদে যাওয়া: মর্যাদা বৃদ্ধির আমল","description":"এই হাদিসে তিনটি সহজ কিন্তু মূল্যবান আমলের কথা এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম সাহাবাদের জিজ্ঞেস করলেন, তিনি কি এমন বিষয় জানাবেন যার দ্বারা আল্লাহ গোনাহ মাফ করেন এবং মর্যাদা উন্নত করেন? এরপর তিনি বললেন, কষ্টের সময় সুন্দরভাবে ওজু করা, মসজিদের দিকে বেশি বেশি পদচারণা করা এবং এক নামাজের পর আরেক নামাজের জন্য অপেক্ষা করা। শেষে তিনি বললেন, এটি জিহাদে প্রতিরক্ষার কাজের ন্যায়। এখানে ওজুর ফজিলত, মসজিদে যাওয়ার ফজিলত এবং নামাজের অপেক্ষার গুরুত্ব একসঙ্গে এসেছে। কষ্টের সময়ও ওজু ঠিকভাবে করা এবং নামাজের সঙ্গে হৃদয়কে যুক্ত রাখা মুমিনের দৃঢ়তা দেখায়। এই হাদিস মানুষকে নামাজকেন্দ্রিক জীবন গড়তে উৎসাহ দেয়।"},"teachings":["কষ্টের সময় সুন্দরভাবে ওজু করা গোনাহ মাফের কারণ হিসেবে এসেছে।","মসজিদের দিকে বেশি পদচারণার ফজিলত আছে।","এক নামাজের পর আরেক নামাজের অপেক্ষা মর্যাদা বৃদ্ধির আমল।","নামাজকেন্দ্রিক জীবন মুমিনের জন্য মূল্যবান পথ।"],"related_hadiths":[{"id":"15৯","book_id":"1","label":"Sahih Bukhari"},{"id":"234","book_id":"2","label":"Sahih Muslim"},{"id":"615","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সুন্দর ওজু, মসজিদে পদচারণা ও নামাজের অপেক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. কষ্টের সময় সুন্দর ওজু, মসজিদে যাওয়া ও নামাজের অপেক্ষা গোনাহ মাফের কারণ।"},"heading":{"title":"সুন্দর ওজু ও মসজিদে যাওয়া: মর্যাদা বৃদ্ধির আমল","description":"এই হাদিসে তিনটি সহজ কিন্তু মূল্যবান আমলের কথা এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম সাহাবাদের জিজ্ঞেস করলেন, তিনি কি এমন বিষয় জানাবেন যার দ্বারা আল্লাহ গোনাহ মাফ করেন এবং মর্যাদা উন্নত করেন? এরপর তিনি বললেন, কষ্টের সময় সুন্দরভাবে ওজু করা, মসজিদের দিকে বেশি বেশি পদচারণা করা এবং এক নামাজের পর আরেক নামাজের জন্য অপেক্ষা করা। শেষে তিনি বললেন, এটি জিহাদে প্রতিরক্ষার কাজের ন্যায়। এখানে ওজুর ফজিলত, মসজিদে যাওয়ার ফজিলত এবং নামাজের অপেক্ষার গুরুত্ব একসঙ্গে এসেছে। কষ্টের সময়ও ওজু ঠিকভাবে করা এবং নামাজের সঙ্গে হৃদয়কে যুক্ত রাখা মুমিনের দৃঢ়তা দেখায়। এই হাদিস মানুষকে নামাজকেন্দ্রিক জীবন গড়তে উৎসাহ দেয়।"},"teachings":["কষ্টের সময় সুন্দরভাবে ওজু করা গোনাহ মাফের কারণ হিসেবে এসেছে।","মসজিদের দিকে বেশি পদচারণার ফজিলত আছে।","এক নামাজের পর আরেক নামাজের অপেক্ষা মর্যাদা বৃদ্ধির আমল।","নামাজকেন্দ্রিক জীবন মুমিনের জন্য মূল্যবান পথ।"],"related_hadiths":[{"id":"159","book_id":"1","label":"Sahih Bukhari"},{"id":"234","book_id":"2","label":"Sahih Muslim"},{"id":"615","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মসজিদে প্রবেশ ও বের হওয়ার দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. মসজিদে ঢোকার সময় রহমত আর বের হওয়ার সময় আল্লাহর অনুগ্রহ চাওয়ার দোয়া।"},"heading":{"title":"মসজিদে প্রবেশের দোয়া: রহমত ও অনুগ্রহ চাওয়ার সুন্নাহ","description":"এই হাদিসে মসজিদে প্রবেশ ও বের হওয়ার দোয়া শেখানো হয়েছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, তোমাদের কেউ যখন মসজিদে প্রবেশ করে, তখন যেন বলে, “আল্লাহুম্মাফ তাহলী আবওয়াবা রাহমাতিক”—অর্থাৎ, হে আল্লাহ, আমার জন্য তোমার রহমতের দরজাসমূহ খুলে দাও। আর যখন বের হয়, তখন যেন বলে, “আল্লাহুম্মা ইন্নি আসআলুকা মিন ফাযলিকা”—অর্থাৎ, হে আল্লাহ, আমি তোমার অনুগ্রহ কামনা করছি। এই হাদিসে মসজিদকে রহমতের জায়গা হিসেবে দেখা যায় এবং বাইরে বের হওয়ার সময় আল্লাহর অনুগ্রহ চাওয়ার শিক্ষা আছে। মসজিদে প্রবেশের দোয়া, মসজিদ থেকে বের হওয়ার দোয়া এবং নামাজের আদব জানতে চাইলে এই হাদিস খুব সহজ নির্দেশনা দেয়।"},"teachings":["মসজিদে প্রবেশের সময় আল্লাহর রহমত চাওয়া উচিত।","মসজিদ থেকে বের হলে আল্লাহর অনুগ্রহ চাওয়ার দোয়া আছে।","মসজিদে যাতায়াতেও দোয়ার আদব শেখানো হয়েছে।","ছোট দোয়াগুলো দৈনন্দিন ইবাদতকে সুন্দর করে।"],"related_hadiths":[{"id":"251","book_id":"2","label":"Sahih Muslim"},{"id":"615","book_id":"1","label":"Sahih Bukhari"},{"id":"৯0৮","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মসজিদে প্রবেশ ও বের হওয়ার দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. মসজিদে ঢোকার সময় রহমত আর বের হওয়ার সময় আল্লাহর অনুগ্রহ চাওয়ার দোয়া।"},"heading":{"title":"মসজিদে প্রবেশের দোয়া: রহমত ও অনুগ্রহ চাওয়ার সুন্নাহ","description":"এই হাদিসে মসজিদে প্রবেশ ও বের হওয়ার দোয়া শেখানো হয়েছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, তোমাদের কেউ যখন মসজিদে প্রবেশ করে, তখন যেন বলে, “আল্লাহুম্মাফ তাহলী আবওয়াবা রাহমাতিক”—অর্থাৎ, হে আল্লাহ, আমার জন্য তোমার রহমতের দরজাসমূহ খুলে দাও। আর যখন বের হয়, তখন যেন বলে, “আল্লাহুম্মা ইন্নি আসআলুকা মিন ফাযলিকা”—অর্থাৎ, হে আল্লাহ, আমি তোমার অনুগ্রহ কামনা করছি। এই হাদিসে মসজিদকে রহমতের জায়গা হিসেবে দেখা যায় এবং বাইরে বের হওয়ার সময় আল্লাহর অনুগ্রহ চাওয়ার শিক্ষা আছে। মসজিদে প্রবেশের দোয়া, মসজিদ থেকে বের হওয়ার দোয়া এবং নামাজের আদব জানতে চাইলে এই হাদিস খুব সহজ নির্দেশনা দেয়।"},"teachings":["মসজিদে প্রবেশের সময় আল্লাহর রহমত চাওয়া উচিত।","মসজিদ থেকে বের হলে আল্লাহর অনুগ্রহ চাওয়ার দোয়া আছে।","মসজিদে যাতায়াতেও দোয়ার আদব শেখানো হয়েছে।","ছোট দোয়াগুলো দৈনন্দিন ইবাদতকে সুন্দর করে।"],"related_hadiths":[{"id":"251","book_id":"2","label":"Sahih Muslim"},{"id":"615","book_id":"1","label":"Sahih Bukhari"},{"id":"908","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নামাজে সুতরা রাখার বিধান","description":"$book_name$ $hadith_number$ - $chapter_name$. সামনে সুতরা রেখে নামাজ পড়লে সামনে দিয়ে অতিক্রমকারী নিয়ে চিন্তার প্রয়োজন নেই।"},"heading":{"title":"নামাজে সুতরা: সামনে আড়াল রেখে নামাজ পড়ার শিক্ষা","description":"এই হাদিসে নামাজে সুতরা রাখার বিষয়টি এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, তোমাদের কেউ নিজের সামনে বাহনের জিনের পিছনের কাঠের মতো কিছু রেখে নামাজ পড়লে, তার সামনে দিয়ে কেউ অতিক্রম করলে সে বিষয় নিয়ে পরোয়া করার দরকার নেই। এখানে মূল কথা হলো, নামাজের সামনে একটি চিহ্ন বা আড়াল রাখা। এতে নামাজ পড়া ব্যক্তি নিজের মনোযোগ ধরে রাখতে পারে এবং সামনে দিয়ে চলাচলের বিষয়টি আলাদা হয়ে যায়। হাদিসে কোনো বড় আয়োজনের কথা নেই; বাহনের জিনের পিছনের কাঠের মতো কিছুর উদাহরণ দেওয়া হয়েছে। নামাজে সুতরা, সামনে দিয়ে যাওয়া এবং নামাজের আদব—এই বিষয়গুলো এই হাদিসে সরাসরি এসেছে।"},"teachings":["নামাজের সামনে সুতরা রাখা হাদিসে বর্ণিত।","সুতরা থাকলে সামনে দিয়ে অতিক্রমকারী নিয়ে পরোয়া না করার কথা এসেছে।","নামাজে মনোযোগ রক্ষায় সামনে আড়াল রাখা উপকারী।","সুতরার জন্য খুব বড় কিছু দরকার—এমন কথা হাদিসে নেই।"],"related_hadiths":[{"id":"50৯","book_id":"1","label":"Sahih Bukhari"},{"id":"510","book_id":"1","label":"Sahih Bukhari"},{"id":"501","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নামাজে সুতরা রাখার বিধান","description":"$book_name$ $hadith_number$ - $chapter_name$. সামনে সুতরা রেখে নামাজ পড়লে সামনে দিয়ে অতিক্রমকারী নিয়ে চিন্তার প্রয়োজন নেই।"},"heading":{"title":"নামাজে সুতরা: সামনে আড়াল রেখে নামাজ পড়ার শিক্ষা","description":"এই হাদিসে নামাজে সুতরা রাখার বিষয়টি এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, তোমাদের কেউ নিজের সামনে বাহনের জিনের পিছনের কাঠের মতো কিছু রেখে নামাজ পড়লে, তার সামনে দিয়ে কেউ অতিক্রম করলে সে বিষয় নিয়ে পরোয়া করার দরকার নেই। এখানে মূল কথা হলো, নামাজের সামনে একটি চিহ্ন বা আড়াল রাখা। এতে নামাজ পড়া ব্যক্তি নিজের মনোযোগ ধরে রাখতে পারে এবং সামনে দিয়ে চলাচলের বিষয়টি আলাদা হয়ে যায়। হাদিসে কোনো বড় আয়োজনের কথা নেই; বাহনের জিনের পিছনের কাঠের মতো কিছুর উদাহরণ দেওয়া হয়েছে। নামাজে সুতরা, সামনে দিয়ে যাওয়া এবং নামাজের আদব—এই বিষয়গুলো এই হাদিসে সরাসরি এসেছে।"},"teachings":["নামাজের সামনে সুতরা রাখা হাদিসে বর্ণিত।","সুতরা থাকলে সামনে দিয়ে অতিক্রমকারী নিয়ে পরোয়া না করার কথা এসেছে।","নামাজে মনোযোগ রক্ষায় সামনে আড়াল রাখা উপকারী।","সুতরার জন্য খুব বড় কিছু দরকার—এমন কথা হাদিসে নেই।"],"related_hadiths":[{"id":"509","book_id":"1","label":"Sahih Bukhari"},{"id":"510","book_id":"1","label":"Sahih Bukhari"},{"id":"501","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নামাজে ইকআ ভঙ্গিতে বসা","description":"$book_name$ $hadith_number$ - $chapter_name$. ইবনে আব্বাস (রাঃ) ইকআ ভঙ্গিতে বসাকে নবী صلى الله عليه وسلم-এর সুন্নাহ বলেছেন।"},"heading":{"title":"ইকআ ভঙ্গিতে বসা: নামাজে নবী صلى الله عليه وسلم-এর সুন্নাহর শিক্ষা","description":"এই হাদিসে নামাজে ইকআ ভঙ্গিতে বসার বিষয়টি এসেছে। ত্বাউস বলেন, তারা ইবনে আব্বাস (রাঃ)-কে দুই পায়ের ওপর ইকআ নিয়মে বসা সম্পর্কে জিজ্ঞাসা করেছিলেন। তিনি বললেন, এটা সুন্নত। তারা বললেন, এতে তো পায়ের প্রতি কষ্ট বা যুলুম হয়। তখন ইবনে আব্বাস (রাঃ) বললেন, বরং এটি তোমার নবীর সুন্নত। হাদিসটি দেখায়, কোনো আমল সম্পর্কে নিজের ধারণা থাকলেও সাহাবীদের কাছে সুন্নাহর গুরুত্ব ছিল বেশি। এখানে ইকআ বসার পদ্ধতির পূর্ণ বিস্তারিত নেই; শুধু এটিকে সুন্নাহ বলা হয়েছে। তাই নামাজে বসার সুন্নাহ, ইকআ ভঙ্গি এবং সাহাবীদের সুন্নাহ মানার মনোভাব—এসব শিক্ষা এই হাদিসে সরাসরি পাওয়া যায়।"},"teachings":["ইকআ ভঙ্গিতে বসাকে ইবনে আব্বাস (রাঃ) সুন্নত বলেছেন।","সুন্নাহর সামনে ব্যক্তিগত ধারণাকে অগ্রাধিকার দেওয়া উচিত নয়।","সাহাবীরা নামাজের ছোট বিষয়েও নবী صلى الله عليه وسلم-এর আমল জানতে চাইতেন।","নামাজের বসার ভঙ্গিও সুন্নাহর অংশ হতে পারে।"],"related_hadiths":[{"id":"৮2৮","book_id":"1","label":"Sahih Bukhari"},{"id":"৮35","book_id":"1","label":"Sahih Bukhari"},{"id":"4৯৮","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নামাজে ইকআ ভঙ্গিতে বসা","description":"$book_name$ $hadith_number$ - $chapter_name$. ইবনে আব্বাস (রাঃ) ইকআ ভঙ্গিতে বসাকে নবী صلى الله عليه وسلم-এর সুন্নাহ বলেছেন।"},"heading":{"title":"ইকআ ভঙ্গিতে বসা: নামাজে নবী صلى الله عليه وسلم-এর সুন্নাহর শিক্ষা","description":"এই হাদিসে নামাজে ইকআ ভঙ্গিতে বসার বিষয়টি এসেছে। ত্বাউস বলেন, তারা ইবনে আব্বাস (রাঃ)-কে দুই পায়ের ওপর ইকআ নিয়মে বসা সম্পর্কে জিজ্ঞাসা করেছিলেন। তিনি বললেন, এটা সুন্নত। তারা বললেন, এতে তো পায়ের প্রতি কষ্ট বা যুলুম হয়। তখন ইবনে আব্বাস (রাঃ) বললেন, বরং এটি তোমার নবীর সুন্নত। হাদিসটি দেখায়, কোনো আমল সম্পর্কে নিজের ধারণা থাকলেও সাহাবীদের কাছে সুন্নাহর গুরুত্ব ছিল বেশি। এখানে ইকআ বসার পদ্ধতির পূর্ণ বিস্তারিত নেই; শুধু এটিকে সুন্নাহ বলা হয়েছে। তাই নামাজে বসার সুন্নাহ, ইকআ ভঙ্গি এবং সাহাবীদের সুন্নাহ মানার মনোভাব—এসব শিক্ষা এই হাদিসে সরাসরি পাওয়া যায়।"},"teachings":["ইকআ ভঙ্গিতে বসাকে ইবনে আব্বাস (রাঃ) সুন্নত বলেছেন।","সুন্নাহর সামনে ব্যক্তিগত ধারণাকে অগ্রাধিকার দেওয়া উচিত নয়।","সাহাবীরা নামাজের ছোট বিষয়েও নবী صلى الله عليه وسلم-এর আমল জানতে চাইতেন।","নামাজের বসার ভঙ্গিও সুন্নাহর অংশ হতে পারে।"],"related_hadiths":[{"id":"828","book_id":"1","label":"Sahih Bukhari"},{"id":"835","book_id":"1","label":"Sahih Bukhari"},{"id":"498","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -702,7 +702,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শেষ রাকআতে বসার সুন্নতি পদ্ধতি","description":"$book_name$ $hadith_number$ - $chapter_name$. শেষ রাকআতে বাম পা এগিয়ে, ডান পা খাড়া করে নিতম্বের ওপর বসার বর্ণনা।"},"heading":{"title":"শেষ রাকআতে বসা: তাশাহহুদের সুন্নতি ভঙ্গি","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর শেষ রাকআতে বসার ভঙ্গি বর্ণিত হয়েছে। বলা হয়েছে, তিনি যখন শেষ রাকআতে বসতেন, তখন বাম পা এগিয়ে দিতেন, ডান পা খাড়া রাখতেন এবং নিতম্বের ওপর বসতেন। নামাজে বসার ভঙ্গি নিয়ে অনেকের প্রশ্ন থাকে। এই হাদিস সেই বিষয়ে একটি সরাসরি বর্ণনা দেয়। এখানে মূল শিক্ষা হলো, নামাজের ভেতরের অঙ্গভঙ্গিতেও নবীজির পদ্ধতি অনুসরণ করার চেষ্টা করা। শেষ রাকআতে বসা, তাশাহহুদের ভঙ্গি এবং নামাজের সুন্নাহ—এই বিষয়গুলো এই হাদিসে পরিষ্কারভাবে এসেছে। হাদিসে যতটুকু বর্ণিত হয়েছে, ততটুকুই বলা উচিত; এর বাইরে অতিরিক্ত দাবি করার দরকার নেই।"},"teachings":["শেষ রাকআতে নবী صلى الله عليه وسلم-এর বসার ভঙ্গি বর্ণিত হয়েছে।","বাম পা এগিয়ে ও ডান পা খাড়া রাখার কথা এসেছে।","নামাজের অঙ্গভঙ্গিতেও সুন্নাহ অনুসরণ গুরুত্বপূর্ণ।","তাশাহহুদের বসা সম্পর্কে হাদিসভিত্তিক জ্ঞান নেওয়া দরকার।"],"related_hadiths":[{"id":"536","book_id":"2","label":"Sahih Muslim"},{"id":"৮35","book_id":"1","label":"Sahih Bukhari"},{"id":"4৯৮","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শেষ রাকআতে বসার সুন্নতি পদ্ধতি","description":"$book_name$ $hadith_number$ - $chapter_name$. শেষ রাকআতে বাম পা এগিয়ে, ডান পা খাড়া করে নিতম্বের ওপর বসার বর্ণনা।"},"heading":{"title":"শেষ রাকআতে বসা: তাশাহহুদের সুন্নতি ভঙ্গি","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর শেষ রাকআতে বসার ভঙ্গি বর্ণিত হয়েছে। বলা হয়েছে, তিনি যখন শেষ রাকআতে বসতেন, তখন বাম পা এগিয়ে দিতেন, ডান পা খাড়া রাখতেন এবং নিতম্বের ওপর বসতেন। নামাজে বসার ভঙ্গি নিয়ে অনেকের প্রশ্ন থাকে। এই হাদিস সেই বিষয়ে একটি সরাসরি বর্ণনা দেয়। এখানে মূল শিক্ষা হলো, নামাজের ভেতরের অঙ্গভঙ্গিতেও নবীজির পদ্ধতি অনুসরণ করার চেষ্টা করা। শেষ রাকআতে বসা, তাশাহহুদের ভঙ্গি এবং নামাজের সুন্নাহ—এই বিষয়গুলো এই হাদিসে পরিষ্কারভাবে এসেছে। হাদিসে যতটুকু বর্ণিত হয়েছে, ততটুকুই বলা উচিত; এর বাইরে অতিরিক্ত দাবি করার দরকার নেই।"},"teachings":["শেষ রাকআতে নবী صلى الله عليه وسلم-এর বসার ভঙ্গি বর্ণিত হয়েছে।","বাম পা এগিয়ে ও ডান পা খাড়া রাখার কথা এসেছে।","নামাজের অঙ্গভঙ্গিতেও সুন্নাহ অনুসরণ গুরুত্বপূর্ণ।","তাশাহহুদের বসা সম্পর্কে হাদিসভিত্তিক জ্ঞান নেওয়া দরকার।"],"related_hadiths":[{"id":"536","book_id":"2","label":"Sahih Muslim"},{"id":"835","book_id":"1","label":"Sahih Bukhari"},{"id":"498","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঘুমের আগে তিন কুল পড়ার আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. শয্যার সময় সূরা ইখলাস, ফালাক ও নাস পড়ে শরীরে হাত বুলানো নবী صلى الله عليه وسلم-এর রাতের আমল।"},"heading":{"title":"ঘুমের আগে তিন কুল: রাতের সুরক্ষাময় সুন্নতি আমল","description":"এই হাদিসে ঘুমের আগে তিন কুল পড়ার আমল বর্ণিত হয়েছে। নবী করীম সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম প্রতি রাতে শয্যা গ্রহণের সময় দুই হাতের তালু এক করতেন। তারপর সূরা ইখলাস, সূরা ফালাক ও সূরা নাস পড়ে তাতে ফুঁ দিতেন। এরপর হাত দিয়ে শরীরের যতদূর সম্ভব বুলিয়ে নিতেন। তিনি মাথা, চেহারা এবং শরীরের সামনের দিক থেকে শুরু করতেন এবং এভাবে তিনবার করতেন। এই হাদিস থেকে বোঝা যায়, ঘুমের আগে কুরআনের ছোট সূরাগুলো পড়া একটি সুন্দর সুন্নাহ। এটি খুব সহজ আমল, কিন্তু নিয়মিত করলে রাতের শুরুটা আল্লাহর স্মরণ দিয়ে হয়। ঘুমের দোয়া ও ঘুমের আগে আমল খোঁজেন এমন মানুষের জন্য এই হাদিস সরাসরি একটি পরিষ্কার নির্দেশনা দেয়।"},"teachings":["ঘুমের আগে সূরা ইখলাস, ফালাক ও নাস পড়া নবী صلى الله عليه وسلم-এর আমল।","তালুতে ফুঁ দিয়ে শরীরে হাত বুলানো হাদিসে বর্ণিত পদ্ধতি।","এই আমল তিনবার করা নবী صلى الله عليه وسلم থেকে প্রমাণিত।","রাতের শুরুতে কুরআন তিলাওয়াত মুসলিমের সুন্দর অভ্যাস হতে পারে।"],"related_hadiths":[{"id":"6311","book_id":"1","label":"Sahih Bukhari"},{"id":"631৮","book_id":"1","label":"Sahih Bukhari"},{"id":"1154","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঘুমের আগে তিন কুল পড়ার আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. শয্যার সময় সূরা ইখলাস, ফালাক ও নাস পড়ে শরীরে হাত বুলানো নবী صلى الله عليه وسلم-এর রাতের আমল।"},"heading":{"title":"ঘুমের আগে তিন কুল: রাতের সুরক্ষাময় সুন্নতি আমল","description":"এই হাদিসে ঘুমের আগে তিন কুল পড়ার আমল বর্ণিত হয়েছে। নবী করীম সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম প্রতি রাতে শয্যা গ্রহণের সময় দুই হাতের তালু এক করতেন। তারপর সূরা ইখলাস, সূরা ফালাক ও সূরা নাস পড়ে তাতে ফুঁ দিতেন। এরপর হাত দিয়ে শরীরের যতদূর সম্ভব বুলিয়ে নিতেন। তিনি মাথা, চেহারা এবং শরীরের সামনের দিক থেকে শুরু করতেন এবং এভাবে তিনবার করতেন। এই হাদিস থেকে বোঝা যায়, ঘুমের আগে কুরআনের ছোট সূরাগুলো পড়া একটি সুন্দর সুন্নাহ। এটি খুব সহজ আমল, কিন্তু নিয়মিত করলে রাতের শুরুটা আল্লাহর স্মরণ দিয়ে হয়। ঘুমের দোয়া ও ঘুমের আগে আমল খোঁজেন এমন মানুষের জন্য এই হাদিস সরাসরি একটি পরিষ্কার নির্দেশনা দেয়।"},"teachings":["ঘুমের আগে সূরা ইখলাস, ফালাক ও নাস পড়া নবী صلى الله عليه وسلم-এর আমল।","তালুতে ফুঁ দিয়ে শরীরে হাত বুলানো হাদিসে বর্ণিত পদ্ধতি।","এই আমল তিনবার করা নবী صلى الله عليه وسلم থেকে প্রমাণিত।","রাতের শুরুতে কুরআন তিলাওয়াত মুসলিমের সুন্দর অভ্যাস হতে পারে।"],"related_hadiths":[{"id":"6311","book_id":"1","label":"Sahih Bukhari"},{"id":"6318","book_id":"1","label":"Sahih Bukhari"},{"id":"1154","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | তাশাহহুদের পর দোয়া করার শিক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. তাশাহহুদ ও দরূদের পর নিজের পছন্দমতো দোয়া বেছে নেওয়ার শিক্ষা।"},"heading":{"title":"তাশাহহুদের পর দোয়া: নামাজে নিজের প্রয়োজন চাওয়ার সুযোগ","description":"এই হাদিসে নামাজের শেষ অংশে দোয়া করার শিক্ষা এসেছে। বর্ণনাকারী বলেন, তারা যখন নবী করীম সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর পিছনে নামাজ পড়তেন, তখন শেষে বলা হয়েছে—তাশাহহুদ ও দরূদের পর প্রত্যেকে নিজের পছন্দমতো দোয়া বেছে নিয়ে দোয়া করবে। এখানে নামাজের ভেতরে দোয়ার একটি সুন্দর স্থান বোঝানো হয়েছে। তাশাহহুদ ও দরূদ পড়ার পর বান্দা নিজের প্রয়োজন, ক্ষমা, কল্যাণ ও আল্লাহর সাহায্য চাইতে পারে। হাদিসে নির্দিষ্ট কোনো দোয়ার তালিকা দেওয়া হয়নি; বরং নিজের পছন্দমতো দোয়া করার কথা এসেছে। তাই তাশাহহুদের পর দোয়া, নামাজের দোয়া এবং দরূদের পর চাওয়ার আদব—এই বিষয়গুলো এই হাদিসে সহজভাবে শেখানো হয়েছে।"},"teachings":["তাশাহহুদ ও দরূদের পর দোয়া করার শিক্ষা আছে।","নামাজের শেষ অংশে নিজের পছন্দমতো দোয়া বেছে নেওয়া যায়।","দরূদের পর আল্লাহর কাছে প্রয়োজন চাওয়া সুন্দর আমল।","নামাজ শুধু তিলাওয়াত নয়; এতে দোয়ার সুযোগও আছে।"],"related_hadiths":[{"id":"৮2৮","book_id":"1","label":"Sahih Bukhari"},{"id":"402","book_id":"2","label":"Sahih Muslim"},{"id":"৮31","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | তাশাহহুদের পর দোয়া করার শিক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. তাশাহহুদ ও দরূদের পর নিজের পছন্দমতো দোয়া বেছে নেওয়ার শিক্ষা।"},"heading":{"title":"তাশাহহুদের পর দোয়া: নামাজে নিজের প্রয়োজন চাওয়ার সুযোগ","description":"এই হাদিসে নামাজের শেষ অংশে দোয়া করার শিক্ষা এসেছে। বর্ণনাকারী বলেন, তারা যখন নবী করীম সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর পিছনে নামাজ পড়তেন, তখন শেষে বলা হয়েছে—তাশাহহুদ ও দরূদের পর প্রত্যেকে নিজের পছন্দমতো দোয়া বেছে নিয়ে দোয়া করবে। এখানে নামাজের ভেতরে দোয়ার একটি সুন্দর স্থান বোঝানো হয়েছে। তাশাহহুদ ও দরূদ পড়ার পর বান্দা নিজের প্রয়োজন, ক্ষমা, কল্যাণ ও আল্লাহর সাহায্য চাইতে পারে। হাদিসে নির্দিষ্ট কোনো দোয়ার তালিকা দেওয়া হয়নি; বরং নিজের পছন্দমতো দোয়া করার কথা এসেছে। তাই তাশাহহুদের পর দোয়া, নামাজের দোয়া এবং দরূদের পর চাওয়ার আদব—এই বিষয়গুলো এই হাদিসে সহজভাবে শেখানো হয়েছে।"},"teachings":["তাশাহহুদ ও দরূদের পর দোয়া করার শিক্ষা আছে।","নামাজের শেষ অংশে নিজের পছন্দমতো দোয়া বেছে নেওয়া যায়।","দরূদের পর আল্লাহর কাছে প্রয়োজন চাওয়া সুন্দর আমল।","নামাজ শুধু তিলাওয়াত নয়; এতে দোয়ার সুযোগও আছে।"],"related_hadiths":[{"id":"828","book_id":"1","label":"Sahih Bukhari"},{"id":"402","book_id":"2","label":"Sahih Muslim"},{"id":"831","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -768,7 +768,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সুন্নত নামাযের ফজিলত ও জান্নাতের ঘর","description":"$book_name$ $hadith_number$ - $chapter_name$. ফরয নামাযের বাইরে নিয়মিত বার রাকআত সুন্নত পড়ার বড় ফজিলত ও আল্লাহর সন্তুষ্টির পথ জানুন।"},"heading":{"title":"সুন্নত নামাযের ফজিলত: প্রতিদিন বার রাকআতের সুন্দর শিক্ষা","description":"এই হাদিসের মূল বিষয় হলো সুন্নত নামাযের ফজিলত। এখানে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, কোনো মুসলিম যদি আল্লাহর জন্য প্রতিদিন ফরয নামাযের বাইরে বার রাকআত সুন্নত নামায পড়ে, আল্লাহ তার জন্য জান্নাতে একটি ঘর তৈরি করেন। তাই এই হাদিস আমাদের শেখায়, ফরয নামাযের পাশাপাশি নফল ও সুন্নত আমলও মুমিনের জীবনে বড় মূল্য রাখে। এখানে আমলটি আল্লাহর জন্য করার কথা বলা হয়েছে, তাই নিয়তও গুরুত্বপূর্ণ। এই শিক্ষা সহজ হলেও গভীর। নিয়মিত সুন্নত নামায মানুষকে নামাযের সঙ্গে আরও বেশি যুক্ত করে এবং ইবাদতের ধারাবাহিকতা গড়ে তোলে।"},"teachings":["ফরয নামাযের বাইরে সুন্নত নামাযের বিশেষ ফজিলত আছে।","আমল আল্লাহর জন্য হলে তার মূল্য বেশি হয়।","নিয়মিত ছোট আমলও জান্নাতের ঘর লাভের কারণ হতে পারে।","নামাযের ধারাবাহিকতা মুমিনের ইবাদতকে সুন্দর করে।"],"related_hadiths":[{"id":"11৮0","book_id":"1","label":"Sahih Bukhari"},{"id":"11৮1","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সুন্নত নামাযের ফজিলত ও জান্নাতের ঘর","description":"$book_name$ $hadith_number$ - $chapter_name$. ফরয নামাযের বাইরে নিয়মিত বার রাকআত সুন্নত পড়ার বড় ফজিলত ও আল্লাহর সন্তুষ্টির পথ জানুন।"},"heading":{"title":"সুন্নত নামাযের ফজিলত: প্রতিদিন বার রাকআতের সুন্দর শিক্ষা","description":"এই হাদিসের মূল বিষয় হলো সুন্নত নামাযের ফজিলত। এখানে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, কোনো মুসলিম যদি আল্লাহর জন্য প্রতিদিন ফরয নামাযের বাইরে বার রাকআত সুন্নত নামায পড়ে, আল্লাহ তার জন্য জান্নাতে একটি ঘর তৈরি করেন। তাই এই হাদিস আমাদের শেখায়, ফরয নামাযের পাশাপাশি নফল ও সুন্নত আমলও মুমিনের জীবনে বড় মূল্য রাখে। এখানে আমলটি আল্লাহর জন্য করার কথা বলা হয়েছে, তাই নিয়তও গুরুত্বপূর্ণ। এই শিক্ষা সহজ হলেও গভীর। নিয়মিত সুন্নত নামায মানুষকে নামাযের সঙ্গে আরও বেশি যুক্ত করে এবং ইবাদতের ধারাবাহিকতা গড়ে তোলে।"},"teachings":["ফরয নামাযের বাইরে সুন্নত নামাযের বিশেষ ফজিলত আছে।","আমল আল্লাহর জন্য হলে তার মূল্য বেশি হয়।","নিয়মিত ছোট আমলও জান্নাতের ঘর লাভের কারণ হতে পারে।","নামাযের ধারাবাহিকতা মুমিনের ইবাদতকে সুন্দর করে।"],"related_hadiths":[{"id":"1180","book_id":"1","label":"Sahih Bukhari"},{"id":"1181","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -790,7 +790,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | চাশতের নামায ও দৈনিক সাদকাহ","description":"$book_name$ $hadith_number$ - $chapter_name$. তাসবিহ, তাকবির, ভালো কাজের আদেশ এবং চাশতের দু’রাকআত নামাযের সাদকাহর শিক্ষা জানুন।"},"heading":{"title":"চাশতের নামায: শরীরের জোড়ার পক্ষ থেকে সাদকাহ","description":"এই হাদিসের মূল বিষয় হলো চাশতের নামায ও সাদকাহ। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, মানুষের প্রতিটি জোড়ার জন্য সাদকাহ আছে। কিন্তু সাদকাহ শুধু টাকা দেওয়ার মধ্যে সীমাবদ্ধ নয়। লা-ইলাহা ইল্লাল্লাহ বলা, আল্লাহু আকবর বলা, সৎ কাজের আদেশ দেওয়া এবং অসৎ কাজ থেকে নিষেধ করাও সাদকাহ হিসেবে গণ্য হয়। এরপর বলা হয়েছে, এসবের মুকাবিলায় চাশতের দু’রাকআত নামায যথেষ্ট হয়। তাই হাদিসটি আমাদের শেখায়, জিকির, ভালো কথা, ভালো কাজে ডাক দেওয়া এবং চাশতের নামায—সবই আল্লাহর কাছে মূল্যবান আমল।"},"teachings":["সাদকাহ শুধু অর্থ দিয়ে নয়, জিকির ও ভালো কাজের মাধ্যমেও হয়।","লা-ইলাহা ইল্লাল্লাহ ও আল্লাহু আকবর বলা সাদকাহ হিসেবে গণ্য।","সৎ কাজের আদেশ ও অসৎ কাজের নিষেধ গুরুত্বপূর্ণ আমল।","চাশতের দু’রাকআত নামাযের বিশেষ মর্যাদা আছে।"],"related_hadiths":[{"id":"117৮","book_id":"1","label":"Sahih Bukhari"},{"id":"11৮0","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | চাশতের নামায ও দৈনিক সাদকাহ","description":"$book_name$ $hadith_number$ - $chapter_name$. তাসবিহ, তাকবির, ভালো কাজের আদেশ এবং চাশতের দু’রাকআত নামাযের সাদকাহর শিক্ষা জানুন।"},"heading":{"title":"চাশতের নামায: শরীরের জোড়ার পক্ষ থেকে সাদকাহ","description":"এই হাদিসের মূল বিষয় হলো চাশতের নামায ও সাদকাহ। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, মানুষের প্রতিটি জোড়ার জন্য সাদকাহ আছে। কিন্তু সাদকাহ শুধু টাকা দেওয়ার মধ্যে সীমাবদ্ধ নয়। লা-ইলাহা ইল্লাল্লাহ বলা, আল্লাহু আকবর বলা, সৎ কাজের আদেশ দেওয়া এবং অসৎ কাজ থেকে নিষেধ করাও সাদকাহ হিসেবে গণ্য হয়। এরপর বলা হয়েছে, এসবের মুকাবিলায় চাশতের দু’রাকআত নামায যথেষ্ট হয়। তাই হাদিসটি আমাদের শেখায়, জিকির, ভালো কথা, ভালো কাজে ডাক দেওয়া এবং চাশতের নামায—সবই আল্লাহর কাছে মূল্যবান আমল।"},"teachings":["সাদকাহ শুধু অর্থ দিয়ে নয়, জিকির ও ভালো কাজের মাধ্যমেও হয়।","লা-ইলাহা ইল্লাল্লাহ ও আল্লাহু আকবর বলা সাদকাহ হিসেবে গণ্য।","সৎ কাজের আদেশ ও অসৎ কাজের নিষেধ গুরুত্বপূর্ণ আমল।","চাশতের দু’রাকআত নামাযের বিশেষ মর্যাদা আছে।"],"related_hadiths":[{"id":"1178","book_id":"1","label":"Sahih Bukhari"},{"id":"1180","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -812,7 +812,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রাতের নামাযের মর্যাদা","description":"$book_name$ $hadith_number$ - $chapter_name$. ফরয নামাযের পর রাতের নামাযের মর্যাদা সম্পর্কে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লামের শিক্ষা পড়ুন।"},"heading":{"title":"রাতের নামায: ফরযের পর উত্তম নফল ইবাদত","description":"এই হাদিসের মূল বিষয় হলো রাতের নামায। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লামকে জিজ্ঞাসা করা হয়েছিল, ফরয নামাযের পর কোন নামায উত্তম। তিনি বলেছেন, রাতে উঠে নামায পড়া। এই কথার মাধ্যমে রাতের নফল নামাযের মর্যাদা বোঝা যায়। হাদিসটি আমাদের শেখায়, ফরয নামায আগে; তারপর নফল ইবাদতের মধ্যে রাতের নামাযের বিশেষ স্থান আছে। এখানে রাতের নামাযকে সহজভাবে তুলে ধরা হয়েছে—রাতে উঠে আল্লাহর সামনে দাঁড়ানো। তাই যে ব্যক্তি নিজের ইবাদত বাড়াতে চায়, সে ফরয নামায ঠিক রাখার পাশাপাশি রাতের নামাযের প্রতি আগ্রহী হতে পারে।"},"teachings":["ফরয নামাযের মর্যাদা সবার আগে।","ফরযের পর রাতের নামায বড় নফল ইবাদত।","রাতে উঠে নামায পড়া আল্লাহর ইবাদতে মনোযোগ বাড়ায়।","নফল আমলে ধীরে ধীরে অভ্যাস তৈরি করা ভালো।"],"related_hadiths":[{"id":"1147","book_id":"1","label":"Sahih Bukhari"},{"id":"117৮","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রাতের নামাযের মর্যাদা","description":"$book_name$ $hadith_number$ - $chapter_name$. ফরয নামাযের পর রাতের নামাযের মর্যাদা সম্পর্কে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লামের শিক্ষা পড়ুন।"},"heading":{"title":"রাতের নামায: ফরযের পর উত্তম নফল ইবাদত","description":"এই হাদিসের মূল বিষয় হলো রাতের নামায। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লামকে জিজ্ঞাসা করা হয়েছিল, ফরয নামাযের পর কোন নামায উত্তম। তিনি বলেছেন, রাতে উঠে নামায পড়া। এই কথার মাধ্যমে রাতের নফল নামাযের মর্যাদা বোঝা যায়। হাদিসটি আমাদের শেখায়, ফরয নামায আগে; তারপর নফল ইবাদতের মধ্যে রাতের নামাযের বিশেষ স্থান আছে। এখানে রাতের নামাযকে সহজভাবে তুলে ধরা হয়েছে—রাতে উঠে আল্লাহর সামনে দাঁড়ানো। তাই যে ব্যক্তি নিজের ইবাদত বাড়াতে চায়, সে ফরয নামায ঠিক রাখার পাশাপাশি রাতের নামাযের প্রতি আগ্রহী হতে পারে।"},"teachings":["ফরয নামাযের মর্যাদা সবার আগে।","ফরযের পর রাতের নামায বড় নফল ইবাদত।","রাতে উঠে নামায পড়া আল্লাহর ইবাদতে মনোযোগ বাড়ায়।","নফল আমলে ধীরে ধীরে অভ্যাস তৈরি করা ভালো।"],"related_hadiths":[{"id":"1147","book_id":"1","label":"Sahih Bukhari"},{"id":"1178","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -834,7 +834,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রাতের শেষ নামায বিতর","description":"$book_name$ $hadith_number$ - $chapter_name$. রাতের শেষ নামাযকে বিতর করার নববী নির্দেশনা ও বিতর নামাযের গুরুত্ব সহজ বাংলায় জানুন।"},"heading":{"title":"বিতর নামায: রাতের শেষ সালাত করার শিক্ষা","description":"এই হাদিসের মূল বিষয় হলো বিতর নামায। নবী করীম সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, তোমরা তোমাদের রাতের শেষ নামাযকে বিতর করে নাও। এখানে বিতর নামাযকে রাতের শেষ নামায হিসেবে রাখার শিক্ষা দেওয়া হয়েছে। হাদিসটি খুব সংক্ষিপ্ত, কিন্তু আমলের দিক থেকে স্পষ্ট। যারা রাতে নফল নামায পড়ে, তাদের জন্য শেষ নামায হিসেবে বিতর রাখা একটি সুন্দর নববী দিকনির্দেশনা। এর মাধ্যমে রাতের ইবাদত একটি পূর্ণতার অনুভব পায়। তবে হাদিসের কথার বাইরে গিয়ে অতিরিক্ত নিয়ম বলা হয়নি; মূল শিক্ষা হলো রাতের সালাত শেষ করা বিতর দিয়ে।"},"teachings":["রাতের শেষ নামায হিসেবে বিতর রাখার নির্দেশনা এসেছে।","বিতর নামায রাতের ইবাদতের গুরুত্বপূর্ণ অংশ।","নবীজির সংক্ষিপ্ত নির্দেশনাও আমলের জন্য যথেষ্ট শিক্ষা দেয়।","রাতের নফল নামাযে শৃঙ্খলা রাখা ভালো।"],"related_hadiths":[{"id":"৯৯7","book_id":"1","label":"Sahih Bukhari"},{"id":"117৮","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রাতের শেষ নামায বিতর","description":"$book_name$ $hadith_number$ - $chapter_name$. রাতের শেষ নামাযকে বিতর করার নববী নির্দেশনা ও বিতর নামাযের গুরুত্ব সহজ বাংলায় জানুন।"},"heading":{"title":"বিতর নামায: রাতের শেষ সালাত করার শিক্ষা","description":"এই হাদিসের মূল বিষয় হলো বিতর নামায। নবী করীম সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, তোমরা তোমাদের রাতের শেষ নামাযকে বিতর করে নাও। এখানে বিতর নামাযকে রাতের শেষ নামায হিসেবে রাখার শিক্ষা দেওয়া হয়েছে। হাদিসটি খুব সংক্ষিপ্ত, কিন্তু আমলের দিক থেকে স্পষ্ট। যারা রাতে নফল নামায পড়ে, তাদের জন্য শেষ নামায হিসেবে বিতর রাখা একটি সুন্দর নববী দিকনির্দেশনা। এর মাধ্যমে রাতের ইবাদত একটি পূর্ণতার অনুভব পায়। তবে হাদিসের কথার বাইরে গিয়ে অতিরিক্ত নিয়ম বলা হয়নি; মূল শিক্ষা হলো রাতের সালাত শেষ করা বিতর দিয়ে।"},"teachings":["রাতের শেষ নামায হিসেবে বিতর রাখার নির্দেশনা এসেছে।","বিতর নামায রাতের ইবাদতের গুরুত্বপূর্ণ অংশ।","নবীজির সংক্ষিপ্ত নির্দেশনাও আমলের জন্য যথেষ্ট শিক্ষা দেয়।","রাতের নফল নামাযে শৃঙ্খলা রাখা ভালো।"],"related_hadiths":[{"id":"997","book_id":"1","label":"Sahih Bukhari"},{"id":"1178","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জুতো পরে নামাযের বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. আনাস রাদিয়াল্লাহু আনহুর বর্ণনায় জুতো পরে নামায পড়া বিষয়ে রাসূলুল্লাহর আমলের সংক্ষিপ্ত শিক্ষা জানুন।"},"heading":{"title":"জুতো পরে নামায: আনাস রাদিয়াল্লাহু আনহুর সংক্ষিপ্ত উত্তর","description":"এই হাদিসের মূল বিষয় হলো জুতো পরে নামায পড়ার বর্ণনা। আনাস রাদিয়াল্লাহু আনহুকে জিজ্ঞাসা করা হয়েছিল, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম কি জুতো পরে নামায পড়েছেন? তিনি উত্তর দিয়েছেন, হ্যাঁ। হাদিসটি খুব ছোট, তাই এর ব্যাখ্যাতেও সীমা রাখা জরুরি। এখানে শুধু একটি আমলের ঘটনা জানা যায়। এর মাধ্যমে বোঝা যায়, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লামের নামাযের আমল সাহাবিরা দেখতেন, মনে রাখতেন এবং প্রশ্ন করা হলে সরাসরি উত্তর দিতেন। তাই নামাযের সুন্নাহ জানতে নির্ভরযোগ্য বর্ণনার গুরুত্ব অনেক।"},"teachings":["সাহাবিরা রাসূলুল্লাহর নামাযের আমল খেয়াল করে সংরক্ষণ করেছেন।","জুতো পরে নামায পড়ার বিষয়ে সংক্ষিপ্ত বর্ণনা এসেছে।","ধর্মীয় প্রশ্নের উত্তরে স্পষ্ট ও সংক্ষিপ্ত কথা বলা ভালো।","সুন্নাহ জানতে সহীহ বর্ণনার দিকে ফিরে যেতে হয়।"],"related_hadiths":[{"id":"5৮50","book_id":"1","label":"Sahih Bukhari"},{"id":"366","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জুতো পরে নামাযের বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. আনাস রাদিয়াল্লাহু আনহুর বর্ণনায় জুতো পরে নামায পড়া বিষয়ে রাসূলুল্লাহর আমলের সংক্ষিপ্ত শিক্ষা জানুন।"},"heading":{"title":"জুতো পরে নামায: আনাস রাদিয়াল্লাহু আনহুর সংক্ষিপ্ত উত্তর","description":"এই হাদিসের মূল বিষয় হলো জুতো পরে নামায পড়ার বর্ণনা। আনাস রাদিয়াল্লাহু আনহুকে জিজ্ঞাসা করা হয়েছিল, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম কি জুতো পরে নামায পড়েছেন? তিনি উত্তর দিয়েছেন, হ্যাঁ। হাদিসটি খুব ছোট, তাই এর ব্যাখ্যাতেও সীমা রাখা জরুরি। এখানে শুধু একটি আমলের ঘটনা জানা যায়। এর মাধ্যমে বোঝা যায়, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লামের নামাযের আমল সাহাবিরা দেখতেন, মনে রাখতেন এবং প্রশ্ন করা হলে সরাসরি উত্তর দিতেন। তাই নামাযের সুন্নাহ জানতে নির্ভরযোগ্য বর্ণনার গুরুত্ব অনেক।"},"teachings":["সাহাবিরা রাসূলুল্লাহর নামাযের আমল খেয়াল করে সংরক্ষণ করেছেন।","জুতো পরে নামায পড়ার বিষয়ে সংক্ষিপ্ত বর্ণনা এসেছে।","ধর্মীয় প্রশ্নের উত্তরে স্পষ্ট ও সংক্ষিপ্ত কথা বলা ভালো।","সুন্নাহ জানতে সহীহ বর্ণনার দিকে ফিরে যেতে হয়।"],"related_hadiths":[{"id":"5850","book_id":"1","label":"Sahih Bukhari"},{"id":"366","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -878,7 +878,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মসজিদে কুবায় দু’রাকআত নামায","description":"$book_name$ $hadith_number$ - $chapter_name$. রাসূলুল্লাহর মসজিদে কুবায় যাওয়া এবং সেখানে দু’রাকআত নামায পড়ার সুন্দর আমল সম্পর্কে জানুন।"},"heading":{"title":"মসজিদে কুবা: নবীজির আগমন ও দু’রাকআত নামায","description":"এই হাদিসের মূল বিষয় হলো মসজিদে কুবায় নামায। বর্ণনায় এসেছে, নবী করীম সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বাহনে চড়ে এবং পায়ে হেঁটে কুবার মসজিদে আসতেন এবং সেখানে দু’রাকআত নামায পড়তেন। হাদিসটি আমাদের সামনে একটি সুন্দর আমল তুলে ধরে। এখানে মূল কথা হলো, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম মসজিদে কুবায় যেতেন এবং সেখানে নামায আদায় করতেন। বাহনে বা পায়ে—দুইভাবেই যাওয়ার কথা এসেছে। তাই হাদিসের শিক্ষা হলো মসজিদে গিয়ে নামায পড়ার প্রতি নববী ভালোবাসা এবং আমলের ধারাবাহিকতা।"},"teachings":["মসজিদে কুবায় গিয়ে দু’রাকআত নামায পড়ার বর্ণনা এসেছে।","রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম কখনো বাহনে, কখনো পায়ে যেতেন।","মসজিদে গিয়ে নামায পড়া নববী আমলের অংশ।","সহজ আমলও নিয়মিত হলে তা সুন্দর অভ্যাস হয়।"],"related_hadiths":[{"id":"11৯3","book_id":"1","label":"Sahih Bukhari"},{"id":"1412","book_id":"6","label":"Sunan Ibn Majah"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মসজিদে কুবায় দু’রাকআত নামায","description":"$book_name$ $hadith_number$ - $chapter_name$. রাসূলুল্লাহর মসজিদে কুবায় যাওয়া এবং সেখানে দু’রাকআত নামায পড়ার সুন্দর আমল সম্পর্কে জানুন।"},"heading":{"title":"মসজিদে কুবা: নবীজির আগমন ও দু’রাকআত নামায","description":"এই হাদিসের মূল বিষয় হলো মসজিদে কুবায় নামায। বর্ণনায় এসেছে, নবী করীম সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বাহনে চড়ে এবং পায়ে হেঁটে কুবার মসজিদে আসতেন এবং সেখানে দু’রাকআত নামায পড়তেন। হাদিসটি আমাদের সামনে একটি সুন্দর আমল তুলে ধরে। এখানে মূল কথা হলো, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম মসজিদে কুবায় যেতেন এবং সেখানে নামায আদায় করতেন। বাহনে বা পায়ে—দুইভাবেই যাওয়ার কথা এসেছে। তাই হাদিসের শিক্ষা হলো মসজিদে গিয়ে নামায পড়ার প্রতি নববী ভালোবাসা এবং আমলের ধারাবাহিকতা।"},"teachings":["মসজিদে কুবায় গিয়ে দু’রাকআত নামায পড়ার বর্ণনা এসেছে।","রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম কখনো বাহনে, কখনো পায়ে যেতেন।","মসজিদে গিয়ে নামায পড়া নববী আমলের অংশ।","সহজ আমলও নিয়মিত হলে তা সুন্দর অভ্যাস হয়।"],"related_hadiths":[{"id":"1193","book_id":"1","label":"Sahih Bukhari"},{"id":"1412","book_id":"6","label":"Sunan Ibn Majah"}]}</t>
         </is>
       </c>
     </row>
@@ -900,7 +900,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঘরে নফল নামাযের কল্যাণ","description":"$book_name$ $hadith_number$ - $chapter_name$. মসজিদে নামায শেষে ঘরে কিছু নামায রাখার শিক্ষা ও বাড়িতে নামাযের কল্যাণ সম্পর্কে জানুন।"},"heading":{"title":"ঘরে নফল নামায: বাড়ির জন্য কল্যাণের দরজা","description":"এই হাদিসের মূল বিষয় হলো ঘরে নফল নামায পড়া। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, কেউ মসজিদে নামায শেষ করলে তার নামাযের কিছু অংশ যেন বাড়িতে পড়ার জন্য রাখে। কারণ আল্লাহ বাড়িতে নামায পড়ার মধ্যে অনেক কল্যাণ রেখেছেন। এখানে ফরয নামাযের কথা নয়, বরং নামাযের কিছু অংশ বাড়িতে রাখার শিক্ষা এসেছে। এতে ঘরও ইবাদতের সঙ্গে যুক্ত হয়। পরিবার ও ঘরের পরিবেশে নামাযের ভালো প্রভাব পড়ে—এ কথা হাদিসের মূল ভাবের সঙ্গে মানানসই। তাই নফল নামাযের একটি অংশ ঘরে পড়া সুন্দর আমল।"},"teachings":["মসজিদের পাশাপাশি ঘরেও কিছু নামায পড়ার শিক্ষা এসেছে।","বাড়িতে নামায পড়ার মধ্যে আল্লাহ কল্যাণ রেখেছেন।","নফল নামায ঘরের ইবাদতপূর্ণ পরিবেশ গড়তে সাহায্য করে।","ইবাদত শুধু মসজিদে সীমাবদ্ধ নয়, ঘরেও তার অংশ আছে।"],"related_hadiths":[{"id":"11৮7","book_id":"1","label":"Sahih Bukhari"},{"id":"731","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঘরে নফল নামাযের কল্যাণ","description":"$book_name$ $hadith_number$ - $chapter_name$. মসজিদে নামায শেষে ঘরে কিছু নামায রাখার শিক্ষা ও বাড়িতে নামাযের কল্যাণ সম্পর্কে জানুন।"},"heading":{"title":"ঘরে নফল নামায: বাড়ির জন্য কল্যাণের দরজা","description":"এই হাদিসের মূল বিষয় হলো ঘরে নফল নামায পড়া। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, কেউ মসজিদে নামায শেষ করলে তার নামাযের কিছু অংশ যেন বাড়িতে পড়ার জন্য রাখে। কারণ আল্লাহ বাড়িতে নামায পড়ার মধ্যে অনেক কল্যাণ রেখেছেন। এখানে ফরয নামাযের কথা নয়, বরং নামাযের কিছু অংশ বাড়িতে রাখার শিক্ষা এসেছে। এতে ঘরও ইবাদতের সঙ্গে যুক্ত হয়। পরিবার ও ঘরের পরিবেশে নামাযের ভালো প্রভাব পড়ে—এ কথা হাদিসের মূল ভাবের সঙ্গে মানানসই। তাই নফল নামাযের একটি অংশ ঘরে পড়া সুন্দর আমল।"},"teachings":["মসজিদের পাশাপাশি ঘরেও কিছু নামায পড়ার শিক্ষা এসেছে।","বাড়িতে নামায পড়ার মধ্যে আল্লাহ কল্যাণ রেখেছেন।","নফল নামায ঘরের ইবাদতপূর্ণ পরিবেশ গড়তে সাহায্য করে।","ইবাদত শুধু মসজিদে সীমাবদ্ধ নয়, ঘরেও তার অংশ আছে।"],"related_hadiths":[{"id":"1187","book_id":"1","label":"Sahih Bukhari"},{"id":"731","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইস্তিখারার নামায ও দুআ","description":"$book_name$ $hadith_number$ - $chapter_name$. গুরুত্বপূর্ণ কাজে আল্লাহর কাছে কল্যাণ চাওয়ার জন্য ইস্তিখারার নামায ও দুআর নববী শিক্ষা জানুন।"},"heading":{"title":"ইস্তিখারার নামায: সিদ্ধান্তে আল্লাহর কাছে কল্যাণ চাওয়া","description":"এই হাদিসের মূল বিষয় হলো ইস্তিখারার নামায। বর্ণনায় এসেছে, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম সাহাবিদের ইস্তিখারা এমনভাবে শেখাতেন, যেমন কুরআনের সূরা শেখাতেন। এরপর দু’রাকআত নামায পড়ে একটি দুআ পড়ার কথা এসেছে। দুআর কথাগুলোতে বান্দা আল্লাহর ইলম, কুদরত ও অনুগ্রহের মাধ্যমে কল্যাণ চায়। যদি কাজটি দ্বীন, জীবিকা ও পরিণতির দিক থেকে ভালো হয়, তবে তা সহজ ও বরকতময় করার প্রার্থনা করে। আর ক্ষতিকর হলে তা দূরে সরিয়ে কল্যাণ যেখানে আছে সেখানে নিয়ে যাওয়ার দুআ করে। এই হাদিস সিদ্ধান্তের সময় আল্লাহর ওপর ভরসা শেখায়।"},"teachings":["ইস্তিখারা গুরুত্বপূর্ণ কাজের আগে আল্লাহর কাছে কল্যাণ চাওয়ার আমল।","ইস্তিখারায় দু’রাকআত নামাযের পর দুআ পড়ার কথা এসেছে।","বান্দা নিজের অক্ষমতা মেনে আল্লাহর ইলম ও কুদরতের সাহায্য চায়।","যেখানে কল্যাণ আছে, সেটিতে সন্তুষ্ট থাকার দুআ করা হয়।"],"related_hadiths":[{"id":"63৮2","book_id":"1","label":"Sahih Bukhari"},{"id":"73৯0","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইস্তিখারার নামায ও দুআ","description":"$book_name$ $hadith_number$ - $chapter_name$. গুরুত্বপূর্ণ কাজে আল্লাহর কাছে কল্যাণ চাওয়ার জন্য ইস্তিখারার নামায ও দুআর নববী শিক্ষা জানুন।"},"heading":{"title":"ইস্তিখারার নামায: সিদ্ধান্তে আল্লাহর কাছে কল্যাণ চাওয়া","description":"এই হাদিসের মূল বিষয় হলো ইস্তিখারার নামায। বর্ণনায় এসেছে, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম সাহাবিদের ইস্তিখারা এমনভাবে শেখাতেন, যেমন কুরআনের সূরা শেখাতেন। এরপর দু’রাকআত নামায পড়ে একটি দুআ পড়ার কথা এসেছে। দুআর কথাগুলোতে বান্দা আল্লাহর ইলম, কুদরত ও অনুগ্রহের মাধ্যমে কল্যাণ চায়। যদি কাজটি দ্বীন, জীবিকা ও পরিণতির দিক থেকে ভালো হয়, তবে তা সহজ ও বরকতময় করার প্রার্থনা করে। আর ক্ষতিকর হলে তা দূরে সরিয়ে কল্যাণ যেখানে আছে সেখানে নিয়ে যাওয়ার দুআ করে। এই হাদিস সিদ্ধান্তের সময় আল্লাহর ওপর ভরসা শেখায়।"},"teachings":["ইস্তিখারা গুরুত্বপূর্ণ কাজের আগে আল্লাহর কাছে কল্যাণ চাওয়ার আমল।","ইস্তিখারায় দু’রাকআত নামাযের পর দুআ পড়ার কথা এসেছে।","বান্দা নিজের অক্ষমতা মেনে আল্লাহর ইলম ও কুদরতের সাহায্য চায়।","যেখানে কল্যাণ আছে, সেটিতে সন্তুষ্ট থাকার দুআ করা হয়।"],"related_hadiths":[{"id":"6382","book_id":"1","label":"Sahih Bukhari"},{"id":"7390","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ফজরের পর বসে থাকার আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. ফজর নামাযের পর সূর্য ভালোভাবে ওঠা পর্যন্ত জায়নামাযে বসে থাকার নববী আমল জানুন।"},"heading":{"title":"ফজরের পর বসে থাকা: সকাল শুরু করার সুন্দর আমল","description":"এই হাদিসের মূল বিষয় হলো ফজরের পর জায়নামাযে বসে থাকা। বর্ণনায় এসেছে, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম ফজর নামায পড়ার পর সূর্য ভালোভাবে ওঠা পর্যন্ত নিজের জায়নামাযেই বসে থাকতেন। হাদিসটি আমাদের সামনে সকালের একটি শান্ত আমল তুলে ধরে। এতে ফজরের নামাযের পর তাড়াহুড়া না করে কিছু সময় ইবাদতের জায়গায় থাকা বোঝা যায়। হাদিসে নির্দিষ্ট করে কী পড়তেন তা এই অংশে বলা হয়নি, তাই অতিরিক্ত দাবি করা ঠিক নয়। মূল শিক্ষা হলো, ফজরের পর সময়টিকে গুরুত্ব দেওয়া এবং আল্লাহর স্মরণে দিন শুরু করার মনোভাব রাখা।"},"teachings":["ফজরের পর কিছু সময় জায়নামাযে বসে থাকার বর্ণনা এসেছে।","সকালের শুরুতে ইবাদতের পরিবেশ ধরে রাখা সুন্দর আমল।","হাদিসে যা বলা হয়েছে, ব্যাখ্যায় তার সীমা রক্ষা করা জরুরি।","ফজর নামায দিনের ইবাদতপূর্ণ শুরু হতে পারে।"],"related_hadiths":[{"id":"647","book_id":"1","label":"Sahih Bukhari"},{"id":"64৯","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ফজরের পর বসে থাকার আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. ফজর নামাযের পর সূর্য ভালোভাবে ওঠা পর্যন্ত জায়নামাযে বসে থাকার নববী আমল জানুন।"},"heading":{"title":"ফজরের পর বসে থাকা: সকাল শুরু করার সুন্দর আমল","description":"এই হাদিসের মূল বিষয় হলো ফজরের পর জায়নামাযে বসে থাকা। বর্ণনায় এসেছে, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম ফজর নামায পড়ার পর সূর্য ভালোভাবে ওঠা পর্যন্ত নিজের জায়নামাযেই বসে থাকতেন। হাদিসটি আমাদের সামনে সকালের একটি শান্ত আমল তুলে ধরে। এতে ফজরের নামাযের পর তাড়াহুড়া না করে কিছু সময় ইবাদতের জায়গায় থাকা বোঝা যায়। হাদিসে নির্দিষ্ট করে কী পড়তেন তা এই অংশে বলা হয়নি, তাই অতিরিক্ত দাবি করা ঠিক নয়। মূল শিক্ষা হলো, ফজরের পর সময়টিকে গুরুত্ব দেওয়া এবং আল্লাহর স্মরণে দিন শুরু করার মনোভাব রাখা।"},"teachings":["ফজরের পর কিছু সময় জায়নামাযে বসে থাকার বর্ণনা এসেছে।","সকালের শুরুতে ইবাদতের পরিবেশ ধরে রাখা সুন্দর আমল।","হাদিসে যা বলা হয়েছে, ব্যাখ্যায় তার সীমা রক্ষা করা জরুরি।","ফজর নামায দিনের ইবাদতপূর্ণ শুরু হতে পারে।"],"related_hadiths":[{"id":"647","book_id":"1","label":"Sahih Bukhari"},{"id":"649","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জুমআর দিনে গোসলের শিক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. জুমআর জন্য মসজিদে আসার আগে গোসল করে আসার নববী নির্দেশনা ও পরিচ্ছন্নতার শিক্ষা জানুন।"},"heading":{"title":"জুমআর গোসল: মসজিদে আসার আগে পরিচ্ছন্নতার শিক্ষা","description":"এই হাদিসের মূল বিষয় হলো জুমআর দিনে গোসল। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, তোমাদের কেউ যখন জুমআর জন্য আসে, তখন সে যেন গোসল করে আসে। হাদিসটি সহজ ভাষায় জুমআর দিনের একটি গুরুত্বপূর্ণ আদব শেখায়। জুমআ মুসলিমদের সম্মিলিত নামাযের দিন, আর মসজিদে যাওয়ার আগে পরিচ্ছন্নতা রাখা ভদ্রতা ও ইবাদতের সৌন্দর্যের সঙ্গে যুক্ত। এখানে মূল নির্দেশনা হলো গোসল করে আসা। তাই জুমআর নামাযে যাওয়ার সময় শুধু উপস্থিত হওয়া নয়, নিজেকে পরিপাটি ও পরিষ্কার রাখাও একটি নববী শিক্ষা হিসেবে দেখা যায়।"},"teachings":["জুমআর জন্য আসার আগে গোসল করার নির্দেশনা এসেছে।","মসজিদে যাওয়ার সময় পরিচ্ছন্নতা রাখা গুরুত্বপূর্ণ।","জুমআর দিন মুসলিমদের সম্মিলিত ইবাদতের দিন।","ইবাদতের আগে শরীরের পরিষ্কার-পরিচ্ছন্নতার দিকেও খেয়াল রাখতে হয়।"],"related_hadiths":[{"id":"৮7৯","book_id":"1","label":"Sahih Bukhari"},{"id":"৮৮3","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জুমআর দিনে গোসলের শিক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. জুমআর জন্য মসজিদে আসার আগে গোসল করে আসার নববী নির্দেশনা ও পরিচ্ছন্নতার শিক্ষা জানুন।"},"heading":{"title":"জুমআর গোসল: মসজিদে আসার আগে পরিচ্ছন্নতার শিক্ষা","description":"এই হাদিসের মূল বিষয় হলো জুমআর দিনে গোসল। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, তোমাদের কেউ যখন জুমআর জন্য আসে, তখন সে যেন গোসল করে আসে। হাদিসটি সহজ ভাষায় জুমআর দিনের একটি গুরুত্বপূর্ণ আদব শেখায়। জুমআ মুসলিমদের সম্মিলিত নামাযের দিন, আর মসজিদে যাওয়ার আগে পরিচ্ছন্নতা রাখা ভদ্রতা ও ইবাদতের সৌন্দর্যের সঙ্গে যুক্ত। এখানে মূল নির্দেশনা হলো গোসল করে আসা। তাই জুমআর নামাযে যাওয়ার সময় শুধু উপস্থিত হওয়া নয়, নিজেকে পরিপাটি ও পরিষ্কার রাখাও একটি নববী শিক্ষা হিসেবে দেখা যায়।"},"teachings":["জুমআর জন্য আসার আগে গোসল করার নির্দেশনা এসেছে।","মসজিদে যাওয়ার সময় পরিচ্ছন্নতা রাখা গুরুত্বপূর্ণ।","জুমআর দিন মুসলিমদের সম্মিলিত ইবাদতের দিন।","ইবাদতের আগে শরীরের পরিষ্কার-পরিচ্ছন্নতার দিকেও খেয়াল রাখতে হয়।"],"related_hadiths":[{"id":"879","book_id":"1","label":"Sahih Bukhari"},{"id":"883","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জুমআয় আগে আসার ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. জুমআর দিনে আগে মসজিদে আসা, ফেরেশতাদের নাম লেখা এবং খুৎবা শোনার শিক্ষা জানুন।"},"heading":{"title":"জুমআয় আগে আসা: ফেরেশতাদের নাম লেখার বর্ণনা","description":"এই হাদিসের মূল বিষয় হলো জুমআয় আগে মসজিদে আসার ফজিলত। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, জুমআর দিনে মসজিদের দরজায় ফেরেশতারা অবস্থান করেন এবং আগে আসার ক্রম অনুযায়ী আগমনকারীদের নাম লেখেন। হাদিসে আগে আসা ব্যক্তির দানের উদাহরণ গাভী, দুম্বা, মুরগী ও ডিমের সঙ্গে দেওয়া হয়েছে। এরপর ইমাম উপস্থিত হলে ফেরেশতারা দফতর গুটিয়ে খুৎবা শুনতে থাকেন। এই হাদিস আমাদের শেখায়, জুমআর নামাযে দেরি না করে আগেভাগে আসা, খুৎবার গুরুত্ব বোঝা এবং মসজিদে উপস্থিতিকে মূল্যবান সময় হিসেবে দেখা।"},"teachings":["জুমআর দিনে আগে মসজিদে আসার বিশেষ ফজিলত আছে।","ফেরেশতারা আগমনকারীদের নাম ক্রমানুসারে লেখেন।","ইমাম আসার পর খুৎবা মনোযোগ দিয়ে শোনার সময়।","ইবাদতে আগে আসা আগ্রহ ও যত্নের পরিচয় দেয়।"],"related_hadiths":[{"id":"৮৮3","book_id":"1","label":"Sahih Bukhari"},{"id":"৯30","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জুমআয় আগে আসার ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. জুমআর দিনে আগে মসজিদে আসা, ফেরেশতাদের নাম লেখা এবং খুৎবা শোনার শিক্ষা জানুন।"},"heading":{"title":"জুমআয় আগে আসা: ফেরেশতাদের নাম লেখার বর্ণনা","description":"এই হাদিসের মূল বিষয় হলো জুমআয় আগে মসজিদে আসার ফজিলত। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, জুমআর দিনে মসজিদের দরজায় ফেরেশতারা অবস্থান করেন এবং আগে আসার ক্রম অনুযায়ী আগমনকারীদের নাম লেখেন। হাদিসে আগে আসা ব্যক্তির দানের উদাহরণ গাভী, দুম্বা, মুরগী ও ডিমের সঙ্গে দেওয়া হয়েছে। এরপর ইমাম উপস্থিত হলে ফেরেশতারা দফতর গুটিয়ে খুৎবা শুনতে থাকেন। এই হাদিস আমাদের শেখায়, জুমআর নামাযে দেরি না করে আগেভাগে আসা, খুৎবার গুরুত্ব বোঝা এবং মসজিদে উপস্থিতিকে মূল্যবান সময় হিসেবে দেখা।"},"teachings":["জুমআর দিনে আগে মসজিদে আসার বিশেষ ফজিলত আছে।","ফেরেশতারা আগমনকারীদের নাম ক্রমানুসারে লেখেন।","ইমাম আসার পর খুৎবা মনোযোগ দিয়ে শোনার সময়।","ইবাদতে আগে আসা আগ্রহ ও যত্নের পরিচয় দেয়।"],"related_hadiths":[{"id":"883","book_id":"1","label":"Sahih Bukhari"},{"id":"930","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জুমআর দিনের দুআ কবুলের মুহূর্ত","description":"$book_name$ $hadith_number$ - $chapter_name$. জুমআর দিনে সংক্ষিপ্ত এক মুহূর্তে দুআ কবুলের আশা ও নামাযরত অবস্থায় আল্লাহর কাছে চাওয়ার শিক্ষা জানুন।"},"heading":{"title":"জুমআর দিনের দুআ: সংক্ষিপ্ত এক কবুলের মুহূর্ত","description":"এই হাদিসের মূল বিষয় হলো জুমআর দিনের দুআ কবুলের মুহূর্ত। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, জুমআর দিনে এমন একটি মুহূর্ত আছে, কোনো মুসলিম বান্দা যদি সেই মুহূর্তে দাঁড়িয়ে নামায পড়া অবস্থায় আল্লাহর কাছে কিছু চায়, আল্লাহ তাকে তা দান করেন। তিনি হাত দিয়ে ইঙ্গিত করে বুঝিয়েছেন, সময়টি খুব সংক্ষিপ্ত। তাই হাদিসটি জুমআর দিনের মর্যাদা এবং দুআর গুরুত্ব শেখায়। তবে সময়টি ঠিক কোন মুহূর্ত—এই বর্ণনায় তা বলা হয়নি। তাই মূল শিক্ষা হলো জুমআর দিন দুআ ও নামাযে মন দেওয়া, বিশেষ করে সময়কে অবহেলা না করা।"},"teachings":["জুমআর দিনে দুআ কবুলের বিশেষ একটি মুহূর্তের কথা এসেছে।","মুমিনের উচিত নামায ও দুআর সময়কে গুরুত্ব দেওয়া।","সময়টি সংক্ষিপ্ত বলা হয়েছে, তাই জুমআর দিন অবহেলা করা ঠিক নয়।","আল্লাহর কাছে প্রয়োজন চাওয়া ইবাদতের অংশ।"],"related_hadiths":[{"id":"৯34","book_id":"1","label":"Sahih Bukhari"},{"id":"৮53","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জুমআর দিনের দুআ কবুলের মুহূর্ত","description":"$book_name$ $hadith_number$ - $chapter_name$. জুমআর দিনে সংক্ষিপ্ত এক মুহূর্তে দুআ কবুলের আশা ও নামাযরত অবস্থায় আল্লাহর কাছে চাওয়ার শিক্ষা জানুন।"},"heading":{"title":"জুমআর দিনের দুআ: সংক্ষিপ্ত এক কবুলের মুহূর্ত","description":"এই হাদিসের মূল বিষয় হলো জুমআর দিনের দুআ কবুলের মুহূর্ত। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, জুমআর দিনে এমন একটি মুহূর্ত আছে, কোনো মুসলিম বান্দা যদি সেই মুহূর্তে দাঁড়িয়ে নামায পড়া অবস্থায় আল্লাহর কাছে কিছু চায়, আল্লাহ তাকে তা দান করেন। তিনি হাত দিয়ে ইঙ্গিত করে বুঝিয়েছেন, সময়টি খুব সংক্ষিপ্ত। তাই হাদিসটি জুমআর দিনের মর্যাদা এবং দুআর গুরুত্ব শেখায়। তবে সময়টি ঠিক কোন মুহূর্ত—এই বর্ণনায় তা বলা হয়নি। তাই মূল শিক্ষা হলো জুমআর দিন দুআ ও নামাযে মন দেওয়া, বিশেষ করে সময়কে অবহেলা না করা।"},"teachings":["জুমআর দিনে দুআ কবুলের বিশেষ একটি মুহূর্তের কথা এসেছে।","মুমিনের উচিত নামায ও দুআর সময়কে গুরুত্ব দেওয়া।","সময়টি সংক্ষিপ্ত বলা হয়েছে, তাই জুমআর দিন অবহেলা করা ঠিক নয়।","আল্লাহর কাছে প্রয়োজন চাওয়া ইবাদতের অংশ।"],"related_hadiths":[{"id":"934","book_id":"1","label":"Sahih Bukhari"},{"id":"853","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঈদের দিন ভিন্ন পথে ফেরা","description":"$book_name$ $hadith_number$ - $chapter_name$. ঈদের দিন রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লামের ভিন্ন পথে ফেরার সংক্ষিপ্ত সুন্নাহ জানুন।"},"heading":{"title":"ঈদের দিন ভিন্ন পথে ফেরা: নবীজির সহজ আমল","description":"এই হাদিসের মূল বিষয় হলো ঈদের দিনের সুন্নাহ। বর্ণনায় এসেছে, নবী করীম সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম ঈদের দিন ফেরার সময় ভিন্ন পথে আসতেন। হাদিসটি সংক্ষিপ্ত, তাই এর শিক্ষা নিয়েও সীমা রাখা দরকার। এখানে শুধু এতটুকু জানা যায় যে, ঈদের দিন তিনি এক পথে গিয়ে ফেরার সময় অন্য পথ নিতেন। এটি ঈদের দিনের একটি আমল হিসেবে বর্ণিত হয়েছে। আমাদের জন্য শিক্ষা হলো, ঈদের নামায ও ঈদের দিনের ছোট ছোট নববী আদব জানার চেষ্টা করা। আমল ছোট হলেও সুন্নাহ অনুসরণের নিয়ত থাকলে তা সুন্দর হয়ে ওঠে।"},"teachings":["ঈদের দিন ফেরার সময় ভিন্ন পথ নেওয়ার বর্ণনা এসেছে।","নবীজির ছোট আমলও সাহাবিরা সংরক্ষণ করেছেন।","ঈদের দিন শুধু আনন্দ নয়, সুন্নাহ মানার দিনও।","হাদিস সংক্ষিপ্ত হলে অতিরিক্ত ব্যাখ্যায় সতর্ক থাকা উচিত।"],"related_hadiths":[{"id":"৯56","book_id":"1","label":"Sahih Bukhari"},{"id":"৯63","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঈদের দিন ভিন্ন পথে ফেরা","description":"$book_name$ $hadith_number$ - $chapter_name$. ঈদের দিন রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লামের ভিন্ন পথে ফেরার সংক্ষিপ্ত সুন্নাহ জানুন।"},"heading":{"title":"ঈদের দিন ভিন্ন পথে ফেরা: নবীজির সহজ আমল","description":"এই হাদিসের মূল বিষয় হলো ঈদের দিনের সুন্নাহ। বর্ণনায় এসেছে, নবী করীম সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম ঈদের দিন ফেরার সময় ভিন্ন পথে আসতেন। হাদিসটি সংক্ষিপ্ত, তাই এর শিক্ষা নিয়েও সীমা রাখা দরকার। এখানে শুধু এতটুকু জানা যায় যে, ঈদের দিন তিনি এক পথে গিয়ে ফেরার সময় অন্য পথ নিতেন। এটি ঈদের দিনের একটি আমল হিসেবে বর্ণিত হয়েছে। আমাদের জন্য শিক্ষা হলো, ঈদের নামায ও ঈদের দিনের ছোট ছোট নববী আদব জানার চেষ্টা করা। আমল ছোট হলেও সুন্নাহ অনুসরণের নিয়ত থাকলে তা সুন্দর হয়ে ওঠে।"},"teachings":["ঈদের দিন ফেরার সময় ভিন্ন পথ নেওয়ার বর্ণনা এসেছে।","নবীজির ছোট আমলও সাহাবিরা সংরক্ষণ করেছেন।","ঈদের দিন শুধু আনন্দ নয়, সুন্নাহ মানার দিনও।","হাদিস সংক্ষিপ্ত হলে অতিরিক্ত ব্যাখ্যায় সতর্ক থাকা উচিত।"],"related_hadiths":[{"id":"956","book_id":"1","label":"Sahih Bukhari"},{"id":"963","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1098,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কবর যিয়ারতের অনুমতি","description":"$book_name$ $hadith_number$ - $chapter_name$. আগে নিষেধের পর কবর যিয়ারতের অনুমতি সম্পর্কে রাসূলুল্লাহর সংক্ষিপ্ত নির্দেশনা জানুন।"},"heading":{"title":"কবর যিয়ারত: নিষেধের পর অনুমতির নববী নির্দেশনা","description":"এই হাদিসের মূল বিষয় হলো কবর যিয়ারত। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, আমি তোমাদের কবর যিয়ারত করতে নিষেধ করেছিলাম; এখন তোমরা তা যিয়ারত করো। হাদিসটি একটি পরিবর্তিত নির্দেশনা জানায়—আগে নিষেধ ছিল, পরে অনুমতি দেওয়া হয়েছে। এখানে কবর যিয়ারতের নির্দিষ্ট পদ্ধতি বা বিস্তারিত দুআ বলা হয়নি, তাই ব্যাখ্যায় অতিরিক্ত কথা যোগ করা ঠিক নয়। মূল শিক্ষা হলো, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লামের নির্দেশ মানা এবং তিনি যখন অনুমতি দিয়েছেন, তখন তা বৈধ আমল হিসেবে গ্রহণ করা।"},"teachings":["আগে কবর যিয়ারত নিষেধ ছিল, পরে অনুমতি দেওয়া হয়েছে।","রাসূলুল্লাহর নির্দেশ পরিবর্তন হলে সেটিও মানতে হয়।","কবর যিয়ারতের বিষয়ে সহীহ বর্ণনা অনুসরণ জরুরি।","হাদিসে যতটুকু আছে, ব্যাখ্যায় ততটুকুর সীমা রাখা উচিত।"],"related_hadiths":[{"id":"৯75","book_id":"2","label":"Sahih Muslim"},{"id":"156৯","book_id":"6","label":"Sunan Ibn Majah"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কবর যিয়ারতের অনুমতি","description":"$book_name$ $hadith_number$ - $chapter_name$. আগে নিষেধের পর কবর যিয়ারতের অনুমতি সম্পর্কে রাসূলুল্লাহর সংক্ষিপ্ত নির্দেশনা জানুন।"},"heading":{"title":"কবর যিয়ারত: নিষেধের পর অনুমতির নববী নির্দেশনা","description":"এই হাদিসের মূল বিষয় হলো কবর যিয়ারত। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, আমি তোমাদের কবর যিয়ারত করতে নিষেধ করেছিলাম; এখন তোমরা তা যিয়ারত করো। হাদিসটি একটি পরিবর্তিত নির্দেশনা জানায়—আগে নিষেধ ছিল, পরে অনুমতি দেওয়া হয়েছে। এখানে কবর যিয়ারতের নির্দিষ্ট পদ্ধতি বা বিস্তারিত দুআ বলা হয়নি, তাই ব্যাখ্যায় অতিরিক্ত কথা যোগ করা ঠিক নয়। মূল শিক্ষা হলো, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লামের নির্দেশ মানা এবং তিনি যখন অনুমতি দিয়েছেন, তখন তা বৈধ আমল হিসেবে গ্রহণ করা।"},"teachings":["আগে কবর যিয়ারত নিষেধ ছিল, পরে অনুমতি দেওয়া হয়েছে।","রাসূলুল্লাহর নির্দেশ পরিবর্তন হলে সেটিও মানতে হয়।","কবর যিয়ারতের বিষয়ে সহীহ বর্ণনা অনুসরণ জরুরি।","হাদিসে যতটুকু আছে, ব্যাখ্যায় ততটুকুর সীমা রাখা উচিত।"],"related_hadiths":[{"id":"975","book_id":"2","label":"Sahih Muslim"},{"id":"1569","book_id":"6","label":"Sunan Ibn Majah"}]}</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সাহরীর বরকত","description":"$book_name$ $hadith_number$ - $chapter_name$. রোযার আগে সাহরী খাওয়ার নির্দেশনা এবং সাহরীর মধ্যে বরকত থাকার নববী শিক্ষা জানুন।"},"heading":{"title":"সাহরীর বরকত: রোযার আগে নববী নির্দেশনা","description":"এই হাদিসের মূল বিষয় হলো সাহরী। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, তোমরা সাহরী খাও; কারণ সাহরীর মধ্যে বরকত রয়েছে। হাদিসটি খুব সহজ ভাষায় রোযার একটি সুন্দর আমল শেখায়। সাহরী শুধু খাবার নয়; এটি রোযার প্রস্তুতির অংশ এবং নবীজির নির্দেশিত একটি আমল। এখানে সাহরীর পরিমাণ, খাবারের ধরন বা নির্দিষ্ট সময়ের বিস্তারিত বলা হয়নি। তাই মূল শিক্ষা হলো, রোযার আগে সাহরীকে গুরুত্ব দেওয়া এবং বরকতের আশায় তা গ্রহণ করা। এই আমল রোযার সঙ্গে ইবাদতের অনুভবও বাড়ায়।"},"teachings":["রোযার আগে সাহরী খাওয়ার নির্দেশনা এসেছে।","সাহরীর মধ্যে বরকত রয়েছে বলে হাদিসে বলা হয়েছে।","রোযার প্রস্তুতিতে সাহরী একটি গুরুত্বপূর্ণ আমল।","ছোট খাবার হলেও সাহরীকে অবহেলা করা ঠিক নয়।"],"related_hadiths":[{"id":"1৯21","book_id":"1","label":"Sahih Bukhari"},{"id":"10৯6","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সাহরীর বরকত","description":"$book_name$ $hadith_number$ - $chapter_name$. রোযার আগে সাহরী খাওয়ার নির্দেশনা এবং সাহরীর মধ্যে বরকত থাকার নববী শিক্ষা জানুন।"},"heading":{"title":"সাহরীর বরকত: রোযার আগে নববী নির্দেশনা","description":"এই হাদিসের মূল বিষয় হলো সাহরী। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, তোমরা সাহরী খাও; কারণ সাহরীর মধ্যে বরকত রয়েছে। হাদিসটি খুব সহজ ভাষায় রোযার একটি সুন্দর আমল শেখায়। সাহরী শুধু খাবার নয়; এটি রোযার প্রস্তুতির অংশ এবং নবীজির নির্দেশিত একটি আমল। এখানে সাহরীর পরিমাণ, খাবারের ধরন বা নির্দিষ্ট সময়ের বিস্তারিত বলা হয়নি। তাই মূল শিক্ষা হলো, রোযার আগে সাহরীকে গুরুত্ব দেওয়া এবং বরকতের আশায় তা গ্রহণ করা। এই আমল রোযার সঙ্গে ইবাদতের অনুভবও বাড়ায়।"},"teachings":["রোযার আগে সাহরী খাওয়ার নির্দেশনা এসেছে।","সাহরীর মধ্যে বরকত রয়েছে বলে হাদিসে বলা হয়েছে।","রোযার প্রস্তুতিতে সাহরী একটি গুরুত্বপূর্ণ আমল।","ছোট খাবার হলেও সাহরীকে অবহেলা করা ঠিক নয়।"],"related_hadiths":[{"id":"1921","book_id":"1","label":"Sahih Bukhari"},{"id":"1096","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | দ্রুত ইফতারের কল্যাণ","description":"$book_name$ $hadith_number$ - $chapter_name$. সময় হলে দ্রুত ইফতার করার নববী শিক্ষা এবং কল্যাণের মধ্যে থাকার কারণ সম্পর্কে জানুন।"},"heading":{"title":"দ্রুত ইফতার: সময় হলে দেরি না করার নববী শিক্ষা","description":"এই হাদিসের মূল বিষয় হলো দ্রুত ইফতার। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, লোকেরা যতদিন দ্রুত ইফতার করবে, ততদিন কল্যাণের মধ্যে থাকবে। এখানে দ্রুত ইফতার বলতে সময় হওয়ার পর অযথা দেরি না করা বোঝায়। হাদিসটি রোযার আদবের একটি সহজ শিক্ষা দেয়। রোযা আল্লাহর জন্য রাখা হয়, আর ইফতারও নবীজির নির্দেশনা মেনে করা উচিত। এই বর্ণনায় ইফতারের নির্দিষ্ট খাবার বা বাড়তি নিয়ম বলা হয়নি। মূল কথা হলো, সময় হলে ইফতার করা এবং এতে কল্যাণের আশা রাখা।"},"teachings":["ইফতারের সময় হলে অযথা দেরি না করার শিক্ষা এসেছে।","দ্রুত ইফতারকে কল্যাণের সঙ্গে যুক্ত করা হয়েছে।","রোযার শেষ মুহূর্তেও নবীজির নির্দেশনা মানা জরুরি।","ইবাদতে সহজতা ও সুন্নাহর অনুসরণ রাখা ভালো।"],"related_hadiths":[{"id":"1৯54","book_id":"1","label":"Sahih Bukhari"},{"id":"1৯55","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | দ্রুত ইফতারের কল্যাণ","description":"$book_name$ $hadith_number$ - $chapter_name$. সময় হলে দ্রুত ইফতার করার নববী শিক্ষা এবং কল্যাণের মধ্যে থাকার কারণ সম্পর্কে জানুন।"},"heading":{"title":"দ্রুত ইফতার: সময় হলে দেরি না করার নববী শিক্ষা","description":"এই হাদিসের মূল বিষয় হলো দ্রুত ইফতার। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, লোকেরা যতদিন দ্রুত ইফতার করবে, ততদিন কল্যাণের মধ্যে থাকবে। এখানে দ্রুত ইফতার বলতে সময় হওয়ার পর অযথা দেরি না করা বোঝায়। হাদিসটি রোযার আদবের একটি সহজ শিক্ষা দেয়। রোযা আল্লাহর জন্য রাখা হয়, আর ইফতারও নবীজির নির্দেশনা মেনে করা উচিত। এই বর্ণনায় ইফতারের নির্দিষ্ট খাবার বা বাড়তি নিয়ম বলা হয়নি। মূল কথা হলো, সময় হলে ইফতার করা এবং এতে কল্যাণের আশা রাখা।"},"teachings":["ইফতারের সময় হলে অযথা দেরি না করার শিক্ষা এসেছে।","দ্রুত ইফতারকে কল্যাণের সঙ্গে যুক্ত করা হয়েছে।","রোযার শেষ মুহূর্তেও নবীজির নির্দেশনা মানা জরুরি।","ইবাদতে সহজতা ও সুন্নাহর অনুসরণ রাখা ভালো।"],"related_hadiths":[{"id":"1954","book_id":"1","label":"Sahih Bukhari"},{"id":"1955","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রমযানের কিয়াম ও ক্ষমা","description":"$book_name$ $hadith_number$ - $chapter_name$. ঈমান ও নেকীর আশায় রমযানের কিয়াম করার ফজিলত এবং গোনাহ মাফের হাদিস জানুন।"},"heading":{"title":"রমযানের কিয়াম: ঈমান ও সওয়াবের আশায় তারাবীহ","description":"এই হাদিসের মূল বিষয় হলো রমযানের কিয়াম বা তারাবীহ নামায। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, যে ব্যক্তি ঈমানের সাথে এবং নেকীর আশায় রমযানের কিয়াম করে, তার পূর্বেকার গোনাহ মাফ করে দেওয়া হবে। এখানে দুটি বিষয় স্পষ্ট—ঈমান এবং নেকীর আশা। অর্থাৎ আমল শুধু বাহ্যিকভাবে নয়, অন্তরের নিয়তসহ হওয়া দরকার। রমযানের রাতের নামাযকে এই হাদিসে বড় ফজিলতের সঙ্গে উল্লেখ করা হয়েছে। তবে হাদিসের ভাষা অনুযায়ী কথা বলা জরুরি; এখানে রমযানের কিয়ামের ফজিলত বলা হয়েছে, অন্য কোনো অতিরিক্ত শর্ত যোগ করা হয়নি।"},"teachings":["রমযানের কিয়াম ঈমানের সঙ্গে করা দরকার।","নেকীর আশায় আমল করলে তার বিশেষ ফজিলত আছে।","রমযানের রাতের নামায গোনাহ মাফের কারণ হতে পারে।","আমলের মূল্য নিয়ত ও ঈমানের সঙ্গে জড়িত।"],"related_hadiths":[{"id":"1৯01","book_id":"1","label":"Sahih Bukhari"},{"id":"200৯","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রমযানের কিয়াম ও ক্ষমা","description":"$book_name$ $hadith_number$ - $chapter_name$. ঈমান ও নেকীর আশায় রমযানের কিয়াম করার ফজিলত এবং গোনাহ মাফের হাদিস জানুন।"},"heading":{"title":"রমযানের কিয়াম: ঈমান ও সওয়াবের আশায় তারাবীহ","description":"এই হাদিসের মূল বিষয় হলো রমযানের কিয়াম বা তারাবীহ নামায। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, যে ব্যক্তি ঈমানের সাথে এবং নেকীর আশায় রমযানের কিয়াম করে, তার পূর্বেকার গোনাহ মাফ করে দেওয়া হবে। এখানে দুটি বিষয় স্পষ্ট—ঈমান এবং নেকীর আশা। অর্থাৎ আমল শুধু বাহ্যিকভাবে নয়, অন্তরের নিয়তসহ হওয়া দরকার। রমযানের রাতের নামাযকে এই হাদিসে বড় ফজিলতের সঙ্গে উল্লেখ করা হয়েছে। তবে হাদিসের ভাষা অনুযায়ী কথা বলা জরুরি; এখানে রমযানের কিয়ামের ফজিলত বলা হয়েছে, অন্য কোনো অতিরিক্ত শর্ত যোগ করা হয়নি।"},"teachings":["রমযানের কিয়াম ঈমানের সঙ্গে করা দরকার।","নেকীর আশায় আমল করলে তার বিশেষ ফজিলত আছে।","রমযানের রাতের নামায গোনাহ মাফের কারণ হতে পারে।","আমলের মূল্য নিয়ত ও ঈমানের সঙ্গে জড়িত।"],"related_hadiths":[{"id":"1901","book_id":"1","label":"Sahih Bukhari"},{"id":"2009","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রাতে জাগলে দোয়া ও ইস্তিগফার","description":"$book_name$ $hadith_number$ - $chapter_name$. রাতের ঘুম ভাঙলে তাওহীদের জিকির, ইস্তিগফার ও দোয়ার মাধ্যমে আল্লাহর কাছে ফেরার শিক্ষা।"},"heading":{"title":"রাতে ঘুম ভাঙলে দোয়া: তাওহীদের জিকির ও ইস্তিগফার","description":"এই হাদিসে রাতে ঘুম ভেঙে গেলে পড়ার দোয়া এবং আল্লাহর কাছে চাওয়ার আদব এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, যে ব্যক্তি রাতে নিদ্রা ভঙ্গ হলে আল্লাহর একত্ব, তাঁর রাজত্ব, প্রশংসা, ক্ষমতা এবং নিজের অক্ষমতার কথা স্মরণ করে এই জিকির পড়ে, তারপর ক্ষমা চায় বা অন্য কোনো দোয়া করে, তার দোয়া কবুল হয়। হাদিসের দোয়ায় তাওহীদ, তাহমিদ, তাসবিহ, তাকবির এবং “লা হাওলা ওয়ালা কুওয়াতা ইল্লা বিল্লাহ”—সবই আছে। অর্থাৎ, রাতের নিরিবিলি সময়ে ঘুম ভাঙলে তা শুধু বিরক্তির বিষয় নয়; বরং আল্লাহকে স্মরণ করার সুযোগ। রাতে জাগলে দোয়া, ইস্তিগফার এবং তাওহীদের জিকির—এই তিনটি বিষয় এই হাদিসে খুব পরিষ্কারভাবে এসেছে।"},"teachings":["রাতে ঘুম ভাঙলে আল্লাহর তাওহীদ ও প্রশংসার জিকির করা উচিত।","জিকিরের পর ইস্তিগফার করা হাদিসে উৎসাহিত হয়েছে।","ঘুম ভাঙার সময় দোয়া করার একটি বিশেষ সুযোগ আছে।","ভালো কাজ ও মন্দ থেকে বাঁচার শক্তি আল্লাহর সাহায্যেই আসে।"],"related_hadiths":[{"id":"6311","book_id":"1","label":"Sahih Bukhari"},{"id":"631৮","book_id":"1","label":"Sahih Bukhari"},{"id":"6307","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রাতে জাগলে দোয়া ও ইস্তিগফার","description":"$book_name$ $hadith_number$ - $chapter_name$. রাতের ঘুম ভাঙলে তাওহীদের জিকির, ইস্তিগফার ও দোয়ার মাধ্যমে আল্লাহর কাছে ফেরার শিক্ষা।"},"heading":{"title":"রাতে ঘুম ভাঙলে দোয়া: তাওহীদের জিকির ও ইস্তিগফার","description":"এই হাদিসে রাতে ঘুম ভেঙে গেলে পড়ার দোয়া এবং আল্লাহর কাছে চাওয়ার আদব এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, যে ব্যক্তি রাতে নিদ্রা ভঙ্গ হলে আল্লাহর একত্ব, তাঁর রাজত্ব, প্রশংসা, ক্ষমতা এবং নিজের অক্ষমতার কথা স্মরণ করে এই জিকির পড়ে, তারপর ক্ষমা চায় বা অন্য কোনো দোয়া করে, তার দোয়া কবুল হয়। হাদিসের দোয়ায় তাওহীদ, তাহমিদ, তাসবিহ, তাকবির এবং “লা হাওলা ওয়ালা কুওয়াতা ইল্লা বিল্লাহ”—সবই আছে। অর্থাৎ, রাতের নিরিবিলি সময়ে ঘুম ভাঙলে তা শুধু বিরক্তির বিষয় নয়; বরং আল্লাহকে স্মরণ করার সুযোগ। রাতে জাগলে দোয়া, ইস্তিগফার এবং তাওহীদের জিকির—এই তিনটি বিষয় এই হাদিসে খুব পরিষ্কারভাবে এসেছে।"},"teachings":["রাতে ঘুম ভাঙলে আল্লাহর তাওহীদ ও প্রশংসার জিকির করা উচিত।","জিকিরের পর ইস্তিগফার করা হাদিসে উৎসাহিত হয়েছে।","ঘুম ভাঙার সময় দোয়া করার একটি বিশেষ সুযোগ আছে।","ভালো কাজ ও মন্দ থেকে বাঁচার শক্তি আল্লাহর সাহায্যেই আসে।"],"related_hadiths":[{"id":"6311","book_id":"1","label":"Sahih Bukhari"},{"id":"6318","book_id":"1","label":"Sahih Bukhari"},{"id":"6307","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1230,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শাওয়ালের ছয় রোযার ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. রমযানের রোযার পর শাওয়ালের ছয় রোযা রাখার ফজিলত ও এক বছরের রোযার তুলনা জানুন।"},"heading":{"title":"শাওয়ালের ছয় রোযা: রমযানের পর ধারাবাহিক আমল","description":"এই হাদিসের মূল বিষয় হলো শাওয়ালের ছয় রোযা। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, যে ব্যক্তি রমযানের রোযা রাখল, তারপর এর পরপরই শাওয়ালের ছয়টি রোযা রাখল, সে যেন পূর্ণ এক বছরের রোযা রাখল। হাদিসটি রমযানের পর ইবাদতের ধারাবাহিকতা শেখায়। রমযান শেষ হলেই আমল থেমে যায় না; শাওয়ালের ছয় রোযা সেই ভালো অভ্যাস ধরে রাখার একটি পথ। এখানে শাওয়ালের ছয় রোযার ফজিলত স্পষ্টভাবে এসেছে। তবে হাদিসে যেভাবে বলা হয়েছে, সেভাবেই কথা বলা উচিত—এটি এক বছরের রোযার মতো ফজিলতের বর্ণনা।"},"teachings":["রমযানের রোযার পর শাওয়ালের ছয় রোযার ফজিলত আছে।","শাওয়ালের ছয় রোযাকে পূর্ণ এক বছরের রোযার মতো বলা হয়েছে।","রমযানের পরও ভালো আমল চালিয়ে যাওয়া সুন্দর অভ্যাস।","রোযা শুধু রমযানে সীমিত নয়, নফল রোযারও মূল্য আছে।"],"related_hadiths":[{"id":"1৯01","book_id":"1","label":"Sahih Bukhari"},{"id":"1162","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শাওয়ালের ছয় রোযার ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. রমযানের রোযার পর শাওয়ালের ছয় রোযা রাখার ফজিলত ও এক বছরের রোযার তুলনা জানুন।"},"heading":{"title":"শাওয়ালের ছয় রোযা: রমযানের পর ধারাবাহিক আমল","description":"এই হাদিসের মূল বিষয় হলো শাওয়ালের ছয় রোযা। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, যে ব্যক্তি রমযানের রোযা রাখল, তারপর এর পরপরই শাওয়ালের ছয়টি রোযা রাখল, সে যেন পূর্ণ এক বছরের রোযা রাখল। হাদিসটি রমযানের পর ইবাদতের ধারাবাহিকতা শেখায়। রমযান শেষ হলেই আমল থেমে যায় না; শাওয়ালের ছয় রোযা সেই ভালো অভ্যাস ধরে রাখার একটি পথ। এখানে শাওয়ালের ছয় রোযার ফজিলত স্পষ্টভাবে এসেছে। তবে হাদিসে যেভাবে বলা হয়েছে, সেভাবেই কথা বলা উচিত—এটি এক বছরের রোযার মতো ফজিলতের বর্ণনা।"},"teachings":["রমযানের রোযার পর শাওয়ালের ছয় রোযার ফজিলত আছে।","শাওয়ালের ছয় রোযাকে পূর্ণ এক বছরের রোযার মতো বলা হয়েছে।","রমযানের পরও ভালো আমল চালিয়ে যাওয়া সুন্দর অভ্যাস।","রোযা শুধু রমযানে সীমিত নয়, নফল রোযারও মূল্য আছে।"],"related_hadiths":[{"id":"1901","book_id":"1","label":"Sahih Bukhari"},{"id":"1162","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মাসিক তিন রোজা, চাশতের নামাজ ও বিতর","description":"$book_name$ $hadith_number$ - $chapter_name$. মাসিক তিন রোজা, চাশতের নামাজ ও বিতর আদায়—নবীজির অসিয়তে নিয়মিত নেক আমলের সুন্দর শিক্ষা।"},"heading":{"title":"মাসিক তিন রোজা, চাশতের নামাজ ও বিতরের আমল","description":"এই হাদিসে সাহাবি তাঁর প্রিয় বন্ধু রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম)-এর তিনটি অসিয়ত তুলে ধরেছেন। প্রথমটি হলো প্রতি মাসে তিন দিন রোজা রাখা। দ্বিতীয়টি হলো চাশতের নামাজ পড়া। তৃতীয়টি হলো ঘুমানোর আগে বিতর নামাজ পড়ে নেওয়া। হাদিসের ভাষা থেকে বোঝা যায়, তিনি এই আমলগুলোকে খুব গুরুত্ব দিয়ে গ্রহণ করেছিলেন এবং জীবিত থাকা পর্যন্ত এগুলো না ছাড়ার সংকল্প করেছিলেন। এখানে সুন্নত নামাজ, নফল রোজা এবং বিতর নামাজের প্রতি ভালোবাসা দেখা যায়। এটি আমাদের শেখায়, ছোট কিন্তু নিয়মিত আমলও একজন মুমিনের জীবনে বড় প্রভাব রাখতে পারে। তবে হাদিসে যতটুকু বলা হয়েছে, আমাদের ব্যাখ্যাও সেই সীমার মধ্যেই রাখা উচিত।"},"teachings":["নিয়মিত নফল আমল জীবনে ভালো অভ্যাস গড়ে তুলতে সাহায্য করে।","প্রতি মাসে তিন দিন রোজা রাখা একটি গুরুত্বপূর্ণ নেক আমল।","চাশতের নামাজ ও বিতর নামাজের প্রতি যত্ন নেওয়া সুন্নাহর অনুসরণের অংশ।","ঘুমানোর আগে বিতর পড়ে নেওয়া আমলের ধারাবাহিকতা রক্ষায় সহায়ক।"],"related_hadiths":[{"id":"1৯৮1","book_id":"1","label":"Sahih Bukhari"},{"id":"722","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মাসিক তিন রোজা, চাশতের নামাজ ও বিতর","description":"$book_name$ $hadith_number$ - $chapter_name$. মাসিক তিন রোজা, চাশতের নামাজ ও বিতর আদায়—নবীজির অসিয়তে নিয়মিত নেক আমলের সুন্দর শিক্ষা।"},"heading":{"title":"মাসিক তিন রোজা, চাশতের নামাজ ও বিতরের আমল","description":"এই হাদিসে সাহাবি তাঁর প্রিয় বন্ধু রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম)-এর তিনটি অসিয়ত তুলে ধরেছেন। প্রথমটি হলো প্রতি মাসে তিন দিন রোজা রাখা। দ্বিতীয়টি হলো চাশতের নামাজ পড়া। তৃতীয়টি হলো ঘুমানোর আগে বিতর নামাজ পড়ে নেওয়া। হাদিসের ভাষা থেকে বোঝা যায়, তিনি এই আমলগুলোকে খুব গুরুত্ব দিয়ে গ্রহণ করেছিলেন এবং জীবিত থাকা পর্যন্ত এগুলো না ছাড়ার সংকল্প করেছিলেন। এখানে সুন্নত নামাজ, নফল রোজা এবং বিতর নামাজের প্রতি ভালোবাসা দেখা যায়। এটি আমাদের শেখায়, ছোট কিন্তু নিয়মিত আমলও একজন মুমিনের জীবনে বড় প্রভাব রাখতে পারে। তবে হাদিসে যতটুকু বলা হয়েছে, আমাদের ব্যাখ্যাও সেই সীমার মধ্যেই রাখা উচিত।"},"teachings":["নিয়মিত নফল আমল জীবনে ভালো অভ্যাস গড়ে তুলতে সাহায্য করে।","প্রতি মাসে তিন দিন রোজা রাখা একটি গুরুত্বপূর্ণ নেক আমল।","চাশতের নামাজ ও বিতর নামাজের প্রতি যত্ন নেওয়া সুন্নাহর অনুসরণের অংশ।","ঘুমানোর আগে বিতর পড়ে নেওয়া আমলের ধারাবাহিকতা রক্ষায় সহায়ক।"],"related_hadiths":[{"id":"1981","book_id":"1","label":"Sahih Bukhari"},{"id":"722","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -1274,7 +1274,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আরাফার দিনের রোজার ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. আরাফার দিনের রোজা বিগত ও আগামী বছরের গোনাহ মাফের আশার কথা জানায়—এটি বড় নফল আমল।"},"heading":{"title":"আরাফার দিনের রোজার ফজিলত ও গোনাহ মাফের আশা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম) আরাফার দিনের রোজার বিশেষ ফজিলত বলেছেন। তিনি বলেছেন, এই রোজার ব্যাপারে আল্লাহর কাছে আশা করা যায় যে, তিনি বিগত এক বছর ও আগামী এক বছরের গোনাহ মাফ করে দেবেন। এখানে লক্ষ করার বিষয় হলো, নবীজি ‘আশা রাখি’ বলেছেন। তাই এ আমলকে বড় ফজিলতের আমল হিসেবে ভালোবাসা উচিত, কিন্তু নিজের পক্ষ থেকে অতিরিক্ত দাবি করা ঠিক নয়। আরাফার দিনের রোজা নফল রোজার মধ্যে খুব পরিচিত একটি আমল। এটি বান্দাকে আল্লাহর ক্ষমার দিকে আগ্রহী করে। হাদিসটি আমাদের শেখায়, বিশেষ দিনের নেক আমলকে গুরুত্ব দেওয়া মুমিনের জন্য কল্যাণকর।"},"teachings":["আরাফার দিনের রোজা বিশেষ ফজিলতপূর্ণ নফল রোজা।","এই রোজার মাধ্যমে গোনাহ মাফের আশা করা যায়।","নেক আমল করার সময় আল্লাহর রহমতের প্রতি আশা রাখা উচিত।","হাদিসে যেমন বলা হয়েছে, তেমন ভারসাম্যপূর্ণ ভাষা ব্যবহার করা উচিত।"],"related_hadiths":[{"id":"1163","book_id":"2","label":"Sahih Muslim"},{"id":"1৯৮৮","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আরাফার দিনের রোজার ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. আরাফার দিনের রোজা বিগত ও আগামী বছরের গোনাহ মাফের আশার কথা জানায়—এটি বড় নফল আমল।"},"heading":{"title":"আরাফার দিনের রোজার ফজিলত ও গোনাহ মাফের আশা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম) আরাফার দিনের রোজার বিশেষ ফজিলত বলেছেন। তিনি বলেছেন, এই রোজার ব্যাপারে আল্লাহর কাছে আশা করা যায় যে, তিনি বিগত এক বছর ও আগামী এক বছরের গোনাহ মাফ করে দেবেন। এখানে লক্ষ করার বিষয় হলো, নবীজি ‘আশা রাখি’ বলেছেন। তাই এ আমলকে বড় ফজিলতের আমল হিসেবে ভালোবাসা উচিত, কিন্তু নিজের পক্ষ থেকে অতিরিক্ত দাবি করা ঠিক নয়। আরাফার দিনের রোজা নফল রোজার মধ্যে খুব পরিচিত একটি আমল। এটি বান্দাকে আল্লাহর ক্ষমার দিকে আগ্রহী করে। হাদিসটি আমাদের শেখায়, বিশেষ দিনের নেক আমলকে গুরুত্ব দেওয়া মুমিনের জন্য কল্যাণকর।"},"teachings":["আরাফার দিনের রোজা বিশেষ ফজিলতপূর্ণ নফল রোজা।","এই রোজার মাধ্যমে গোনাহ মাফের আশা করা যায়।","নেক আমল করার সময় আল্লাহর রহমতের প্রতি আশা রাখা উচিত।","হাদিসে যেমন বলা হয়েছে, তেমন ভারসাম্যপূর্ণ ভাষা ব্যবহার করা উচিত।"],"related_hadiths":[{"id":"1163","book_id":"2","label":"Sahih Muslim"},{"id":"1988","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সফরে আমীর বানানোর সুন্নত","description":"$book_name$ $hadith_number$ - $chapter_name$. তিনজন সফরে বের হলে একজনকে আমীর বানানোর নির্দেশ দেওয়া হয়েছে—এতে শৃঙ্খলা ও পরামর্শের শিক্ষা আছে।"},"heading":{"title":"সফরে আমীর বানানোর হাদিস ও দলগত শৃঙ্খলা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম) সফরের একটি সহজ কিন্তু গুরুত্বপূর্ণ আদব শিখিয়েছেন। তিনি বলেছেন, যখন তিনজন কোনো সফরে বের হয়, তখন তারা যেন একজনকে আমীর বানিয়ে নেয়। এখানে আমীর বানানোর উদ্দেশ্য হলো সফরে কাজ সহজ হওয়া, সিদ্ধান্তে শৃঙ্খলা থাকা এবং মতভেদ কমে আসা। হাদিসে সফরের কথা বলা হয়েছে, তাই এটিকে সরাসরি সফরের আদব হিসেবেই বোঝা উচিত। একজন আমীর থাকলে পথ, বিরতি, প্রয়োজনীয় কাজ ও দলীয় সিদ্ধান্তে সুবিধা হয়। এই শিক্ষা আমাদের জানায়, ইসলামে ছোট দলেও বিশৃঙ্খলা পছন্দ নয়। পরামর্শ, দায়িত্ব ও শৃঙ্খলা—সবই ভালো সফরের অংশ।"},"teachings":["তিনজন সফরে গেলে একজনকে দায়িত্বশীল করা উচিত।","দলগত কাজে শৃঙ্খলা রাখা ইসলামের সুন্দর শিক্ষা।","সফরে সিদ্ধান্ত নেওয়ার জন্য দায়িত্ব ভাগ করা উপকারী।","আমীর বানানো মানে ঝগড়া নয়, বরং কাজ সহজ করা।"],"related_hadiths":[{"id":"2৯৯3","book_id":"1","label":"Sahih Bukhari"},{"id":"30৮৮","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সফরে আমীর বানানোর সুন্নত","description":"$book_name$ $hadith_number$ - $chapter_name$. তিনজন সফরে বের হলে একজনকে আমীর বানানোর নির্দেশ দেওয়া হয়েছে—এতে শৃঙ্খলা ও পরামর্শের শিক্ষা আছে।"},"heading":{"title":"সফরে আমীর বানানোর হাদিস ও দলগত শৃঙ্খলা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম) সফরের একটি সহজ কিন্তু গুরুত্বপূর্ণ আদব শিখিয়েছেন। তিনি বলেছেন, যখন তিনজন কোনো সফরে বের হয়, তখন তারা যেন একজনকে আমীর বানিয়ে নেয়। এখানে আমীর বানানোর উদ্দেশ্য হলো সফরে কাজ সহজ হওয়া, সিদ্ধান্তে শৃঙ্খলা থাকা এবং মতভেদ কমে আসা। হাদিসে সফরের কথা বলা হয়েছে, তাই এটিকে সরাসরি সফরের আদব হিসেবেই বোঝা উচিত। একজন আমীর থাকলে পথ, বিরতি, প্রয়োজনীয় কাজ ও দলীয় সিদ্ধান্তে সুবিধা হয়। এই শিক্ষা আমাদের জানায়, ইসলামে ছোট দলেও বিশৃঙ্খলা পছন্দ নয়। পরামর্শ, দায়িত্ব ও শৃঙ্খলা—সবই ভালো সফরের অংশ।"},"teachings":["তিনজন সফরে গেলে একজনকে দায়িত্বশীল করা উচিত।","দলগত কাজে শৃঙ্খলা রাখা ইসলামের সুন্দর শিক্ষা।","সফরে সিদ্ধান্ত নেওয়ার জন্য দায়িত্ব ভাগ করা উপকারী।","আমীর বানানো মানে ঝগড়া নয়, বরং কাজ সহজ করা।"],"related_hadiths":[{"id":"2993","book_id":"1","label":"Sahih Bukhari"},{"id":"3088","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সফরে তাকবীর ও তাসবীহ পাঠের আদব","description":"$book_name$ $hadith_number$ - $chapter_name$. সফরে উঁচু পথে তাকবীর ও নিচু পথে তাসবীহ পাঠের আমল শেখানো হয়েছে—এটি যিক্রের সুন্দর আদব।"},"heading":{"title":"সফরে তাকবীর ও তাসবীহ পাঠের সুন্নত আদব","description":"এই হাদিসে সফরের সময় যিক্রের একটি সুন্দর আমল এসেছে। সাহাবি বলেন, তাঁরা যখন উঁচু রাস্তায় উঠতেন, তখন তাকবীর পাঠ করতেন। আর যখন নিচু রাস্তায় নামতেন, তখন তাসবীহ পাঠ করতেন। তাকবীর মানে আল্লাহর বড়ত্ব ঘোষণা করা, আর তাসবীহ মানে আল্লাহকে পবিত্র বলা। হাদিসটি দেখায়, সফর শুধু চলাফেরা নয়; সফরের মধ্যেও আল্লাহর স্মরণ রাখা যায়। পাহাড়ি পথ, উঁচু-নিচু রাস্তা বা যাত্রার পরিবর্তন—এসব সময় যিক্র করা একজন মুমিনকে আল্লাহমুখী রাখে। এখানে কোনো জটিল নিয়ম নয়, বরং সহজ আমলের শিক্ষা দেওয়া হয়েছে। সফরে তাকবীর ও তাসবীহ তাই হৃদয়কে আল্লাহর স্মরণে রাখার উপায়।"},"teachings":["সফরের মাঝেও আল্লাহর যিক্র করা উচিত।","উঁচু পথে ওঠার সময় তাকবীর পাঠের আমল এসেছে।","নিচু পথে নামার সময় তাসবীহ পাঠের আমল এসেছে।","যাত্রার পরিবর্তনেও আল্লাহকে স্মরণ করা মুমিনের সুন্দর অভ্যাস।"],"related_hadiths":[{"id":"373","book_id":"2","label":"Sahih Muslim"},{"id":"270৮","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সফরে তাকবীর ও তাসবীহ পাঠের আদব","description":"$book_name$ $hadith_number$ - $chapter_name$. সফরে উঁচু পথে তাকবীর ও নিচু পথে তাসবীহ পাঠের আমল শেখানো হয়েছে—এটি যিক্রের সুন্দর আদব।"},"heading":{"title":"সফরে তাকবীর ও তাসবীহ পাঠের সুন্নত আদব","description":"এই হাদিসে সফরের সময় যিক্রের একটি সুন্দর আমল এসেছে। সাহাবি বলেন, তাঁরা যখন উঁচু রাস্তায় উঠতেন, তখন তাকবীর পাঠ করতেন। আর যখন নিচু রাস্তায় নামতেন, তখন তাসবীহ পাঠ করতেন। তাকবীর মানে আল্লাহর বড়ত্ব ঘোষণা করা, আর তাসবীহ মানে আল্লাহকে পবিত্র বলা। হাদিসটি দেখায়, সফর শুধু চলাফেরা নয়; সফরের মধ্যেও আল্লাহর স্মরণ রাখা যায়। পাহাড়ি পথ, উঁচু-নিচু রাস্তা বা যাত্রার পরিবর্তন—এসব সময় যিক্র করা একজন মুমিনকে আল্লাহমুখী রাখে। এখানে কোনো জটিল নিয়ম নয়, বরং সহজ আমলের শিক্ষা দেওয়া হয়েছে। সফরে তাকবীর ও তাসবীহ তাই হৃদয়কে আল্লাহর স্মরণে রাখার উপায়।"},"teachings":["সফরের মাঝেও আল্লাহর যিক্র করা উচিত।","উঁচু পথে ওঠার সময় তাকবীর পাঠের আমল এসেছে।","নিচু পথে নামার সময় তাসবীহ পাঠের আমল এসেছে।","যাত্রার পরিবর্তনেও আল্লাহকে স্মরণ করা মুমিনের সুন্দর অভ্যাস।"],"related_hadiths":[{"id":"373","book_id":"2","label":"Sahih Muslim"},{"id":"2708","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নতুন স্থানে অবতরণের দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. কোনো স্থানে অবতরণ করলে আল্লাহর পরিপূর্ণ বাক্যের আশ্রয় চাওয়ার দোয়া শেখানো হয়েছে।"},"heading":{"title":"নতুন স্থানে অবতরণের দোয়া ও আল্লাহর আশ্রয়","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম) নতুন কোনো স্থানে অবতরণ করার সময় একটি দোয়া শিখিয়েছেন। দোয়াটির অর্থ হলো, আল্লাহর পরিপূর্ণ বাক্যের মাধ্যমে তাঁর সৃষ্টির অনিষ্ট থেকে আশ্রয় চাওয়া। হাদিসে বলা হয়েছে, যে ব্যক্তি কোনো স্থানে অবতরণ করে এই দোয়া পড়ে, সে ওই স্থান ত্যাগ না করা পর্যন্ত কোনো কিছু তার ক্ষতি করতে পারবে না। এই বর্ণনায় আল্লাহর কাছে আশ্রয় চাওয়ার শিক্ষা খুব স্পষ্ট। সফর, যাত্রা, নতুন ঘর, পথের বিরতি—এমন অবস্থায় মানুষ অজানা জায়গায় থাকে। তখন নিজের শক্তির ওপর ভরসা না করে আল্লাহর আশ্রয় চাইতে শেখানো হয়েছে। এটি সফরের দোয়া ও নিরাপত্তার গুরুত্বপূর্ণ আমল।"},"teachings":["নতুন স্থানে অবতরণ করলে আল্লাহর আশ্রয় চাওয়া উচিত।","দোয়ার মাধ্যমে বান্দা নিজের দুর্বলতা ও আল্লাহর ক্ষমতা স্বীকার করে।","সফরে অজানা জায়গায় যিক্র ও দোয়া গুরুত্বপূর্ণ।","হাদিসে শেখানো দোয়া অর্থ বুঝে পড়া বেশি উপকারী।"],"related_hadiths":[{"id":"2৯৯3","book_id":"1","label":"Sahih Bukhari"},{"id":"373","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নতুন স্থানে অবতরণের দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. কোনো স্থানে অবতরণ করলে আল্লাহর পরিপূর্ণ বাক্যের আশ্রয় চাওয়ার দোয়া শেখানো হয়েছে।"},"heading":{"title":"নতুন স্থানে অবতরণের দোয়া ও আল্লাহর আশ্রয়","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম) নতুন কোনো স্থানে অবতরণ করার সময় একটি দোয়া শিখিয়েছেন। দোয়াটির অর্থ হলো, আল্লাহর পরিপূর্ণ বাক্যের মাধ্যমে তাঁর সৃষ্টির অনিষ্ট থেকে আশ্রয় চাওয়া। হাদিসে বলা হয়েছে, যে ব্যক্তি কোনো স্থানে অবতরণ করে এই দোয়া পড়ে, সে ওই স্থান ত্যাগ না করা পর্যন্ত কোনো কিছু তার ক্ষতি করতে পারবে না। এই বর্ণনায় আল্লাহর কাছে আশ্রয় চাওয়ার শিক্ষা খুব স্পষ্ট। সফর, যাত্রা, নতুন ঘর, পথের বিরতি—এমন অবস্থায় মানুষ অজানা জায়গায় থাকে। তখন নিজের শক্তির ওপর ভরসা না করে আল্লাহর আশ্রয় চাইতে শেখানো হয়েছে। এটি সফরের দোয়া ও নিরাপত্তার গুরুত্বপূর্ণ আমল।"},"teachings":["নতুন স্থানে অবতরণ করলে আল্লাহর আশ্রয় চাওয়া উচিত।","দোয়ার মাধ্যমে বান্দা নিজের দুর্বলতা ও আল্লাহর ক্ষমতা স্বীকার করে।","সফরে অজানা জায়গায় যিক্র ও দোয়া গুরুত্বপূর্ণ।","হাদিসে শেখানো দোয়া অর্থ বুঝে পড়া বেশি উপকারী।"],"related_hadiths":[{"id":"2993","book_id":"1","label":"Sahih Bukhari"},{"id":"373","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সফর থেকে ফিরে মসজিদে নামাজ","description":"$book_name$ $hadith_number$ - $chapter_name$. সফর থেকে ফিরে রাসূলুল্লাহ প্রথমে মসজিদে গিয়ে নামাজ পড়তেন—এতে মসজিদমুখী জীবনের শিক্ষা আছে।"},"heading":{"title":"সফর থেকে ফিরে মসজিদে নামাজ পড়ার সুন্নত","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম)-এর একটি সুন্দর আমল বর্ণনা করা হয়েছে। তিনি যখন সফর থেকে ফিরতেন, তখন আগে মসজিদে গিয়ে নামাজ পড়তেন। হাদিসটি সফর শেষে ঘরে ফেরার আগে মসজিদে নামাজের আমলকে সামনে আনে। এতে বোঝা যায়, একজন মুমিনের জীবনে মসজিদ শুধু জামাতে নামাজের স্থান নয়, বরং আল্লাহর কাছে ফিরে আসার একটি প্রিয় জায়গা। সফর শেষে ক্লান্তি থাকলেও নবীজি মসজিদে গিয়ে নামাজ পড়তেন। তবে হাদিসে যতটুকু আছে, ব্যাখ্যাও ততটুকুতেই সীমিত থাকা উচিত। এই আমল আমাদের শেখায়, যাত্রার শুরু ও শেষ—সব অবস্থাতেই আল্লাহর স্মরণ রাখা সুন্দর আচরণ।"},"teachings":["সফর থেকে ফিরে মসজিদে গিয়ে নামাজ পড়ার আমল এসেছে।","মসজিদের সঙ্গে সম্পর্ক রাখা মুমিনের ভালো অভ্যাস।","সফর শেষে আল্লাহর স্মরণে নামাজ পড়া সুন্দর কাজ।","নবীজির আমল অনুসরণে দৈনন্দিন জীবন সাজানো উচিত।"],"related_hadiths":[{"id":"2৯৯3","book_id":"1","label":"Sahih Bukhari"},{"id":"270৮","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সফর থেকে ফিরে মসজিদে নামাজ","description":"$book_name$ $hadith_number$ - $chapter_name$. সফর থেকে ফিরে রাসূলুল্লাহ প্রথমে মসজিদে গিয়ে নামাজ পড়তেন—এতে মসজিদমুখী জীবনের শিক্ষা আছে।"},"heading":{"title":"সফর থেকে ফিরে মসজিদে নামাজ পড়ার সুন্নত","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম)-এর একটি সুন্দর আমল বর্ণনা করা হয়েছে। তিনি যখন সফর থেকে ফিরতেন, তখন আগে মসজিদে গিয়ে নামাজ পড়তেন। হাদিসটি সফর শেষে ঘরে ফেরার আগে মসজিদে নামাজের আমলকে সামনে আনে। এতে বোঝা যায়, একজন মুমিনের জীবনে মসজিদ শুধু জামাতে নামাজের স্থান নয়, বরং আল্লাহর কাছে ফিরে আসার একটি প্রিয় জায়গা। সফর শেষে ক্লান্তি থাকলেও নবীজি মসজিদে গিয়ে নামাজ পড়তেন। তবে হাদিসে যতটুকু আছে, ব্যাখ্যাও ততটুকুতেই সীমিত থাকা উচিত। এই আমল আমাদের শেখায়, যাত্রার শুরু ও শেষ—সব অবস্থাতেই আল্লাহর স্মরণ রাখা সুন্দর আচরণ।"},"teachings":["সফর থেকে ফিরে মসজিদে গিয়ে নামাজ পড়ার আমল এসেছে।","মসজিদের সঙ্গে সম্পর্ক রাখা মুমিনের ভালো অভ্যাস।","সফর শেষে আল্লাহর স্মরণে নামাজ পড়া সুন্দর কাজ।","নবীজির আমল অনুসরণে দৈনন্দিন জীবন সাজানো উচিত।"],"related_hadiths":[{"id":"2993","book_id":"1","label":"Sahih Bukhari"},{"id":"2708","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -1428,7 +1428,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জুতো পরা ও খোলার সুন্নত আদব","description":"$book_name$ $hadith_number$ - $chapter_name$. জুতো পরতে ডান পা আগে এবং খুলতে বাঁ পা আগে—এটি দৈনন্দিন জীবনের সহজ সুন্নত আদব।"},"heading":{"title":"জুতো পরা ও খোলার সুন্নত আদব","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম) জুতো পরা ও খোলার সহজ আদব শিখিয়েছেন। তিনি বলেছেন, কেউ জুতো পরলে ডান পা দিয়ে শুরু করবে। আর জুতো খুললে বাঁ পা থেকে শুরু করবে। এরপর তিনি আরেকটি বিষয় বলেছেন—জুতো পরলে দুটোই পরবে, আর খুলে রাখলে দুটোই খুলে রাখবে। হাদিসটি আমাদের দৈনন্দিন জীবনের ছোট কাজেও সুন্নাহর শিক্ষা দেখায়। জুতো পরা সাধারণ কাজ মনে হলেও নবীজি এরও সুন্দর নিয়ম শিখিয়েছেন। এতে বোঝা যায়, ইসলামে পরিচ্ছন্ন, পরিপাটি ও ভারসাম্যপূর্ণ আচরণ গুরুত্ব পায়। মুমিন ছোট আমলকেও হালকা করে না, কারণ এগুলো নবীজির আদবের অংশ।"},"teachings":["জুতো পরার সময় ডান পা আগে দেওয়া সুন্নত আদব।","জুতো খোলার সময় বাঁ পা আগে দেওয়া শেখানো হয়েছে।","এক পায়ে জুতো পরে চলার বদলে দুটোই পরা বা দুটোই খোলা উচিত।","দৈনন্দিন ছোট কাজেও নবীজির আদব অনুসরণ করা যায়।"],"related_hadiths":[{"id":"5৮56","book_id":"1","label":"Sahih Bukhari"},{"id":"20৯৮","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জুতো পরা ও খোলার সুন্নত আদব","description":"$book_name$ $hadith_number$ - $chapter_name$. জুতো পরতে ডান পা আগে এবং খুলতে বাঁ পা আগে—এটি দৈনন্দিন জীবনের সহজ সুন্নত আদব।"},"heading":{"title":"জুতো পরা ও খোলার সুন্নত আদব","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম) জুতো পরা ও খোলার সহজ আদব শিখিয়েছেন। তিনি বলেছেন, কেউ জুতো পরলে ডান পা দিয়ে শুরু করবে। আর জুতো খুললে বাঁ পা থেকে শুরু করবে। এরপর তিনি আরেকটি বিষয় বলেছেন—জুতো পরলে দুটোই পরবে, আর খুলে রাখলে দুটোই খুলে রাখবে। হাদিসটি আমাদের দৈনন্দিন জীবনের ছোট কাজেও সুন্নাহর শিক্ষা দেখায়। জুতো পরা সাধারণ কাজ মনে হলেও নবীজি এরও সুন্দর নিয়ম শিখিয়েছেন। এতে বোঝা যায়, ইসলামে পরিচ্ছন্ন, পরিপাটি ও ভারসাম্যপূর্ণ আচরণ গুরুত্ব পায়। মুমিন ছোট আমলকেও হালকা করে না, কারণ এগুলো নবীজির আদবের অংশ।"},"teachings":["জুতো পরার সময় ডান পা আগে দেওয়া সুন্নত আদব।","জুতো খোলার সময় বাঁ পা আগে দেওয়া শেখানো হয়েছে।","এক পায়ে জুতো পরে চলার বদলে দুটোই পরা বা দুটোই খোলা উচিত।","দৈনন্দিন ছোট কাজেও নবীজির আদব অনুসরণ করা যায়।"],"related_hadiths":[{"id":"5856","book_id":"1","label":"Sahih Bukhari"},{"id":"2098","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -1631,7 +1631,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঈদুল ফিতরে বের হওয়ার আগে খেজুর খাওয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. ঈদুল ফিতরের দিন বের হওয়ার আগে কয়েকটি খেজুর খাওয়ার আমল এসেছে, অন্য বর্ণনায় বিজোড় সংখ্যার কথা আছে।"},"heading":{"title":"ঈদুল ফিতরে বের হওয়ার আগে খেজুর খাওয়ার সুন্নত","description":"এই হাদিসে ঈদুল ফিতরের দিনের একটি সুন্দর আমল এসেছে। বর্ণনাকারী বলেন, রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম) ঈদুল ফিতরের দিন কয়েকটি খেজুর না খেয়ে বের হতেন না। অপর বর্ণনায় এসেছে, তিনি বিজোড় সংখ্যক খেজুর খেতেন। হাদিসটি ঈদের দিনের খাবারের একটি বিশেষ আদব শেখায়। রমজানের রোজা শেষ হওয়ার পর ঈদুল ফিতরের সকালে খেজুর খেয়ে বের হওয়া নবীজির আমল হিসেবে এসেছে। এখানে খেজুরের কথা নির্দিষ্টভাবে বলা হয়েছে, তাই ব্যাখ্যায় অন্য খাবার বা অতিরিক্ত বিধান যোগ করা ঠিক নয়। মূল শিক্ষা হলো, ঈদের আনন্দও সুন্নাহ মেনে শুরু করা যায়। ছোট একটি আমল দিনটিকে আল্লাহর স্মরণ ও নবীজির অনুসরণে সাজায়।"},"teachings":["ঈদুল ফিতরের দিন বের হওয়ার আগে খেজুর খাওয়ার আমল এসেছে।","অপর বর্ণনায় বিজোড় সংখ্যক খেজুর খাওয়ার কথা আছে।","ঈদের আনন্দও নবীজির সুন্নাহ মেনে শুরু করা যায়।","সাধারণ খাবারের মধ্যেও ইবাদতের আদব থাকতে পারে।"],"related_hadiths":[{"id":"৯53","book_id":"1","label":"Sahih Bukhari"},{"id":"৯56","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঈদুল ফিতরে বের হওয়ার আগে খেজুর খাওয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. ঈদুল ফিতরের দিন বের হওয়ার আগে কয়েকটি খেজুর খাওয়ার আমল এসেছে, অন্য বর্ণনায় বিজোড় সংখ্যার কথা আছে।"},"heading":{"title":"ঈদুল ফিতরে বের হওয়ার আগে খেজুর খাওয়ার সুন্নত","description":"এই হাদিসে ঈদুল ফিতরের দিনের একটি সুন্দর আমল এসেছে। বর্ণনাকারী বলেন, রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম) ঈদুল ফিতরের দিন কয়েকটি খেজুর না খেয়ে বের হতেন না। অপর বর্ণনায় এসেছে, তিনি বিজোড় সংখ্যক খেজুর খেতেন। হাদিসটি ঈদের দিনের খাবারের একটি বিশেষ আদব শেখায়। রমজানের রোজা শেষ হওয়ার পর ঈদুল ফিতরের সকালে খেজুর খেয়ে বের হওয়া নবীজির আমল হিসেবে এসেছে। এখানে খেজুরের কথা নির্দিষ্টভাবে বলা হয়েছে, তাই ব্যাখ্যায় অন্য খাবার বা অতিরিক্ত বিধান যোগ করা ঠিক নয়। মূল শিক্ষা হলো, ঈদের আনন্দও সুন্নাহ মেনে শুরু করা যায়। ছোট একটি আমল দিনটিকে আল্লাহর স্মরণ ও নবীজির অনুসরণে সাজায়।"},"teachings":["ঈদুল ফিতরের দিন বের হওয়ার আগে খেজুর খাওয়ার আমল এসেছে।","অপর বর্ণনায় বিজোড় সংখ্যক খেজুর খাওয়ার কথা আছে।","ঈদের আনন্দও নবীজির সুন্নাহ মেনে শুরু করা যায়।","সাধারণ খাবারের মধ্যেও ইবাদতের আদব থাকতে পারে।"],"related_hadiths":[{"id":"953","book_id":"1","label":"Sahih Bukhari"},{"id":"956","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুরআন পাঠকারীর জন্য সুপারিশকারী","description":"$book_name$ $hadith_number$ - $chapter_name$. কুরআন পড়ার নির্দেশ এসেছে, কারণ কিয়ামতের দিন তা পাঠকের জন্য সুপারিশকারী হয়ে আসবে।"},"heading":{"title":"কুরআন পড়ার ফজিলত: কিয়ামতের দিন সুপারিশকারী","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম) কুরআন পড়ার নির্দেশ দিয়েছেন। তিনি বলেছেন, তোমরা কুরআন পড়ো, কারণ তা কিয়ামতের দিন তার পাঠকের জন্য সুপারিশকারী হয়ে আগমন করবে। এখানে কুরআন তেলাওয়াতের বড় ফজিলত খুব স্পষ্টভাবে বলা হয়েছে। কুরআন শুধু পড়ার বই নয়; এটি মুমিনের জীবনের দিশা। তবে এই হাদিসের মূল বক্তব্য হলো কুরআন পাঠ এবং কিয়ামতের দিনে পাঠকের জন্য সুপারিশ। তাই ব্যাখ্যায় এই সীমার মধ্যেই থাকা উচিত। কুরআন নিয়মিত পড়া বান্দার হৃদয়কে আল্লাহর কথার সঙ্গে যুক্ত রাখে। যে ব্যক্তি কুরআন পাঠে অভ্যস্ত হয়, তার জীবনে আল্লাহর বাণীর প্রতি ভালোবাসা বাড়ার সুযোগ তৈরি হয়।"},"teachings":["কুরআন নিয়মিত পড়ার নির্দেশ এসেছে।","কিয়ামতের দিন কুরআন পাঠকের জন্য সুপারিশকারী হবে।","কুরআন তেলাওয়াত মুমিনের গুরুত্বপূর্ণ আমল।","আল্লাহর বাণীর সঙ্গে সম্পর্ক রাখা ঈমানি জীবনের অংশ।"],"related_hadiths":[{"id":"5027","book_id":"1","label":"Sahih Bukhari"},{"id":"7৯2","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুরআন পাঠকারীর জন্য সুপারিশকারী","description":"$book_name$ $hadith_number$ - $chapter_name$. কুরআন পড়ার নির্দেশ এসেছে, কারণ কিয়ামতের দিন তা পাঠকের জন্য সুপারিশকারী হয়ে আসবে।"},"heading":{"title":"কুরআন পড়ার ফজিলত: কিয়ামতের দিন সুপারিশকারী","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম) কুরআন পড়ার নির্দেশ দিয়েছেন। তিনি বলেছেন, তোমরা কুরআন পড়ো, কারণ তা কিয়ামতের দিন তার পাঠকের জন্য সুপারিশকারী হয়ে আগমন করবে। এখানে কুরআন তেলাওয়াতের বড় ফজিলত খুব স্পষ্টভাবে বলা হয়েছে। কুরআন শুধু পড়ার বই নয়; এটি মুমিনের জীবনের দিশা। তবে এই হাদিসের মূল বক্তব্য হলো কুরআন পাঠ এবং কিয়ামতের দিনে পাঠকের জন্য সুপারিশ। তাই ব্যাখ্যায় এই সীমার মধ্যেই থাকা উচিত। কুরআন নিয়মিত পড়া বান্দার হৃদয়কে আল্লাহর কথার সঙ্গে যুক্ত রাখে। যে ব্যক্তি কুরআন পাঠে অভ্যস্ত হয়, তার জীবনে আল্লাহর বাণীর প্রতি ভালোবাসা বাড়ার সুযোগ তৈরি হয়।"},"teachings":["কুরআন নিয়মিত পড়ার নির্দেশ এসেছে।","কিয়ামতের দিন কুরআন পাঠকের জন্য সুপারিশকারী হবে।","কুরআন তেলাওয়াত মুমিনের গুরুত্বপূর্ণ আমল।","আল্লাহর বাণীর সঙ্গে সম্পর্ক রাখা ঈমানি জীবনের অংশ।"],"related_hadiths":[{"id":"5027","book_id":"1","label":"Sahih Bukhari"},{"id":"792","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সুন্দর সুরে কুরআন তেলাওয়াত","description":"$book_name$ $hadith_number$ - $chapter_name$. সুন্দর ও মধুর সুরে কুরআন তেলাওয়াতের কথা এসেছে—আল্লাহর বাণী পাঠে সৌন্দর্যের শিক্ষা।"},"heading":{"title":"সুন্দর সুরে কুরআন তেলাওয়াতের ফজিলত","description":"এই হাদিসে কুরআন তেলাওয়াতের সৌন্দর্য নিয়ে গুরুত্বপূর্ণ শিক্ষা এসেছে। রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম) বলেছেন, আল্লাহ নবী করীমকে যেরূপ মধুর সুরে কুরআন তেলাওয়াত করার অনুমতি দিয়েছেন, অন্য কোনো জিনিসকে ঐরূপ পড়ার অনুমতি দেননি। বর্ণনায় আরও এসেছে, তিনি উচ্চস্বরে সুন্দর সুরে তেলাওয়াত করতেন। এখানে মূল বিষয় হলো কুরআন তেলাওয়াতে সুন্দর সুর, মনোযোগ এবং আল্লাহর বাণীর মর্যাদা। তবে সুন্দর সুর মানে শুধু কণ্ঠের সৌন্দর্য নয়; কুরআনের প্রতি সম্মানও জরুরি। হাদিসে যেমন বলা হয়েছে, নবীজির তেলাওয়াত ছিল মধুর ও উচ্চস্বরে। তাই কুরআন পড়ার সময় পরিষ্কার, সুন্দর ও শ্রদ্ধাপূর্ণ তেলাওয়াতের চেষ্টা করা উচিত।"},"teachings":["কুরআন সুন্দর সুরে তেলাওয়াত করা প্রশংসনীয় আমল।","নবীজি উচ্চস্বরে সুন্দর সুরে কুরআন তেলাওয়াত করতেন।","কুরআন পাঠে শ্রদ্ধা, মনোযোগ ও সুন্দর উচ্চারণ থাকা উচিত।","আল্লাহর বাণী পড়ার সময় তা সাধারণ কথার মতো নেওয়া উচিত নয়।"],"related_hadiths":[{"id":"৮04","book_id":"2","label":"Sahih Muslim"},{"id":"5027","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সুন্দর সুরে কুরআন তেলাওয়াত","description":"$book_name$ $hadith_number$ - $chapter_name$. সুন্দর ও মধুর সুরে কুরআন তেলাওয়াতের কথা এসেছে—আল্লাহর বাণী পাঠে সৌন্দর্যের শিক্ষা।"},"heading":{"title":"সুন্দর সুরে কুরআন তেলাওয়াতের ফজিলত","description":"এই হাদিসে কুরআন তেলাওয়াতের সৌন্দর্য নিয়ে গুরুত্বপূর্ণ শিক্ষা এসেছে। রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম) বলেছেন, আল্লাহ নবী করীমকে যেরূপ মধুর সুরে কুরআন তেলাওয়াত করার অনুমতি দিয়েছেন, অন্য কোনো জিনিসকে ঐরূপ পড়ার অনুমতি দেননি। বর্ণনায় আরও এসেছে, তিনি উচ্চস্বরে সুন্দর সুরে তেলাওয়াত করতেন। এখানে মূল বিষয় হলো কুরআন তেলাওয়াতে সুন্দর সুর, মনোযোগ এবং আল্লাহর বাণীর মর্যাদা। তবে সুন্দর সুর মানে শুধু কণ্ঠের সৌন্দর্য নয়; কুরআনের প্রতি সম্মানও জরুরি। হাদিসে যেমন বলা হয়েছে, নবীজির তেলাওয়াত ছিল মধুর ও উচ্চস্বরে। তাই কুরআন পড়ার সময় পরিষ্কার, সুন্দর ও শ্রদ্ধাপূর্ণ তেলাওয়াতের চেষ্টা করা উচিত।"},"teachings":["কুরআন সুন্দর সুরে তেলাওয়াত করা প্রশংসনীয় আমল।","নবীজি উচ্চস্বরে সুন্দর সুরে কুরআন তেলাওয়াত করতেন।","কুরআন পাঠে শ্রদ্ধা, মনোযোগ ও সুন্দর উচ্চারণ থাকা উচিত।","আল্লাহর বাণী পড়ার সময় তা সাধারণ কথার মতো নেওয়া উচিত নয়।"],"related_hadiths":[{"id":"804","book_id":"2","label":"Sahih Muslim"},{"id":"5027","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | এক অঞ্জলি পানিতে কুলি ও নাকে পানি","description":"$book_name$ $hadith_number$ - $chapter_name$. রাসূল صلى الله عليه وسلم এক অঞ্জলি পানি দিয়ে কুলি ও নাকে পানি দেওয়ার সহজ ওজুর আমল দেখিয়েছেন।"},"heading":{"title":"ওজুতে কুলি ও নাকে পানি: এক অঞ্জলি পানির নববী পদ্ধতি","description":"এই হাদিসে ওজুর সময় কুলি করা এবং নাকে পানি দেওয়ার একটি সহজ পদ্ধতি এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম এক অঞ্জলি পানি দিয়ে কুলি করেছেন এবং নাকে পানি দিয়েছেন। হাদিসটি খুব ছোট, কিন্তু ওজুর বাস্তব পদ্ধতি বোঝার জন্য গুরুত্বপূর্ণ। এখানে পানির অপচয় বা বাড়তি কষ্টের কথা নেই; বরং অল্প পানিতেও ওজুর কাজ সুন্দরভাবে করা যায়, তা দেখা যায়। কুলি ও নাকে পানি দেওয়া ওজুর পরিচ্ছন্নতার অংশ। এই হাদিস থেকে আমরা শিখি, নবীজির ওজু ছিল সহজ, পরিমিত এবং বাস্তব জীবনের জন্য উপযোগী। ওজুর নিয়ম, কুলি করার পদ্ধতি এবং নাকে পানি দেওয়ার সুন্নাহ জানতে চাইলে এই বর্ণনা সরাসরি সাহায্য করে।"},"teachings":["ওজুর সময় কুলি ও নাকে পানি দেওয়া নবী صلى الله عليه وسلم-এর আমল।","এক অঞ্জলি পানি দিয়েও কুলি ও নাকে পানি দেওয়া যায়।","ওজুতে সরলতা ও পরিমিত পানির ব্যবহার বোঝা যায়।","পরিচ্ছন্নতার ছোট ধাপও সুন্নাহর অংশ হতে পারে।"],"related_hadiths":[{"id":"15৯","book_id":"1","label":"Sahih Bukhari"},{"id":"234","book_id":"2","label":"Sahih Muslim"},{"id":"201","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | এক অঞ্জলি পানিতে কুলি ও নাকে পানি","description":"$book_name$ $hadith_number$ - $chapter_name$. রাসূল صلى الله عليه وسلم এক অঞ্জলি পানি দিয়ে কুলি ও নাকে পানি দেওয়ার সহজ ওজুর আমল দেখিয়েছেন।"},"heading":{"title":"ওজুতে কুলি ও নাকে পানি: এক অঞ্জলি পানির নববী পদ্ধতি","description":"এই হাদিসে ওজুর সময় কুলি করা এবং নাকে পানি দেওয়ার একটি সহজ পদ্ধতি এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম এক অঞ্জলি পানি দিয়ে কুলি করেছেন এবং নাকে পানি দিয়েছেন। হাদিসটি খুব ছোট, কিন্তু ওজুর বাস্তব পদ্ধতি বোঝার জন্য গুরুত্বপূর্ণ। এখানে পানির অপচয় বা বাড়তি কষ্টের কথা নেই; বরং অল্প পানিতেও ওজুর কাজ সুন্দরভাবে করা যায়, তা দেখা যায়। কুলি ও নাকে পানি দেওয়া ওজুর পরিচ্ছন্নতার অংশ। এই হাদিস থেকে আমরা শিখি, নবীজির ওজু ছিল সহজ, পরিমিত এবং বাস্তব জীবনের জন্য উপযোগী। ওজুর নিয়ম, কুলি করার পদ্ধতি এবং নাকে পানি দেওয়ার সুন্নাহ জানতে চাইলে এই বর্ণনা সরাসরি সাহায্য করে।"},"teachings":["ওজুর সময় কুলি ও নাকে পানি দেওয়া নবী صلى الله عليه وسلم-এর আমল।","এক অঞ্জলি পানি দিয়েও কুলি ও নাকে পানি দেওয়া যায়।","ওজুতে সরলতা ও পরিমিত পানির ব্যবহার বোঝা যায়।","পরিচ্ছন্নতার ছোট ধাপও সুন্নাহর অংশ হতে পারে।"],"related_hadiths":[{"id":"159","book_id":"1","label":"Sahih Bukhari"},{"id":"234","book_id":"2","label":"Sahih Muslim"},{"id":"201","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -1719,7 +1719,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সর্বাবস্থায় আল্লাহর যিক্র","description":"$book_name$ $hadith_number$ - $chapter_name$. রাসূলুল্লাহ সর্বাবস্থায় আল্লাহর যিক্র করতেন—জীবনের প্রতিটি অবস্থায় আল্লাহকে স্মরণের শিক্ষা।"},"heading":{"title":"সর্বাবস্থায় আল্লাহর যিক্র করার শিক্ষা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম)-এর একটি বড় গুণ খুব সংক্ষেপে বলা হয়েছে। তিনি সর্বাবস্থায় আল্লাহর যিক্র করতেন। অর্থাৎ তাঁর জীবন আল্লাহর স্মরণে ভরা ছিল। হাদিসটি আমাদের শেখায়, যিক্র শুধু নির্দিষ্ট সময়ের আমল নয়; মুমিনের জীবনের নানা অবস্থায় আল্লাহকে স্মরণ করা যায়। হাঁটা, বসা, সফর, ঘর, খাবার, পোশাক—জীবনের অনেক কাজে দোয়া ও যিক্রের শিক্ষা আছে। তবে এই হাদিসে মূল বক্তব্য হলো নবীজির সর্বাবস্থায় আল্লাহর যিক্র করা। তাই আমাদেরও নিজের সামর্থ্য অনুযায়ী বেশি বেশি আল্লাহকে স্মরণ করার চেষ্টা করা উচিত। যিক্র হৃদয়কে আল্লাহমুখী রাখে এবং আমলকে জীবন্ত করে।"},"teachings":["রাসূলুল্লাহ সর্বাবস্থায় আল্লাহর যিক্র করতেন।","যিক্র জীবনের নানা অবস্থায় করা যায়।","দৈনন্দিন কাজে আল্লাহকে স্মরণ করা ভালো অভ্যাস।","নবীজির অনুসরণে যিক্রকে জীবনের অংশ করা উচিত।"],"related_hadiths":[{"id":"6407","book_id":"1","label":"Sahih Bukhari"},{"id":"26৯৯","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সর্বাবস্থায় আল্লাহর যিক্র","description":"$book_name$ $hadith_number$ - $chapter_name$. রাসূলুল্লাহ সর্বাবস্থায় আল্লাহর যিক্র করতেন—জীবনের প্রতিটি অবস্থায় আল্লাহকে স্মরণের শিক্ষা।"},"heading":{"title":"সর্বাবস্থায় আল্লাহর যিক্র করার শিক্ষা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম)-এর একটি বড় গুণ খুব সংক্ষেপে বলা হয়েছে। তিনি সর্বাবস্থায় আল্লাহর যিক্র করতেন। অর্থাৎ তাঁর জীবন আল্লাহর স্মরণে ভরা ছিল। হাদিসটি আমাদের শেখায়, যিক্র শুধু নির্দিষ্ট সময়ের আমল নয়; মুমিনের জীবনের নানা অবস্থায় আল্লাহকে স্মরণ করা যায়। হাঁটা, বসা, সফর, ঘর, খাবার, পোশাক—জীবনের অনেক কাজে দোয়া ও যিক্রের শিক্ষা আছে। তবে এই হাদিসে মূল বক্তব্য হলো নবীজির সর্বাবস্থায় আল্লাহর যিক্র করা। তাই আমাদেরও নিজের সামর্থ্য অনুযায়ী বেশি বেশি আল্লাহকে স্মরণ করার চেষ্টা করা উচিত। যিক্র হৃদয়কে আল্লাহমুখী রাখে এবং আমলকে জীবন্ত করে।"},"teachings":["রাসূলুল্লাহ সর্বাবস্থায় আল্লাহর যিক্র করতেন।","যিক্র জীবনের নানা অবস্থায় করা যায়।","দৈনন্দিন কাজে আল্লাহকে স্মরণ করা ভালো অভ্যাস।","নবীজির অনুসরণে যিক্রকে জীবনের অংশ করা উচিত।"],"related_hadiths":[{"id":"6407","book_id":"1","label":"Sahih Bukhari"},{"id":"2699","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সুবহানাল্লাহি ওয়া বিহামদিহির ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. অল্প কথার গভীর যিকর কীভাবে বড় সাওয়াবের কারণ হতে পারে, এ হাদিসে সেই সুন্দর শিক্ষা আছে।"},"heading":{"title":"সুবহানাল্লাহি ওয়া বিহামদিহি যিকরের ফজিলত ও শিক্ষা","description":"মূল বিষয়: যিকর। এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম একটি সংক্ষিপ্ত কিন্তু ভারী যিকর শিক্ষা দিয়েছেন। জুয়াইরিয়া রাঃ সকাল থেকে চাশতের সময় পর্যন্ত তাঁর নামাযের স্থানে বসে ছিলেন। তখন নবী সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম বললেন, তিনি যাওয়ার পর চারটি কালেমা তিনবার বলেছেন, যা সেদিন তাঁর দীর্ঘ সময়ের পাঠের সঙ্গে ওজন করলে বেশি ভারী হবে। এই হাদিস থেকে বোঝা যায়, যিকরের মূল্য শুধু সময়ের দৈর্ঘ্যে নয়; বরং শব্দের অর্থ, আল্লাহর প্রশংসা ও আন্তরিকতার দিক থেকেও বড় হতে পারে। এখানে মূল দুআ হলো: সুবহানাল্লাহি ওয়া বিহামদিহি, আদাদা খালকিহি, ওয়া রিযা নাফসিহি, ওয়া যিনাতা আরশিহি, ওয়া মিদাদা কালিমাতিহি। বাংলা অর্থে এতে আল্লাহর পবিত্রতা ও প্রশংসা তাঁর সৃষ্টি, সন্তুষ্টি, আরশের ওজন এবং তাঁর কালেমার বিস্তারের সঙ্গে যুক্ত করে বলা হয়েছে।"},"teachings":["অল্প সময়েও অর্থবহ যিকর করা যায়।","আল্লাহর প্রশংসা ও পবিত্রতা বর্ণনা করা মুমিনের সুন্দর আমল।","রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম সহজ শব্দে বড় শিক্ষা দিয়েছেন।","যিকরের শব্দ ও অর্থ বুঝে পড়া বেশি মনোযোগ আনতে পারে।"],"related_hadiths":[{"id":"201৮","book_id":"2","label":"Sahih Muslim"},{"id":"33৮0","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"2732","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সুবহানাল্লাহি ওয়া বিহামদিহির ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. অল্প কথার গভীর যিকর কীভাবে বড় সাওয়াবের কারণ হতে পারে, এ হাদিসে সেই সুন্দর শিক্ষা আছে।"},"heading":{"title":"সুবহানাল্লাহি ওয়া বিহামদিহি যিকরের ফজিলত ও শিক্ষা","description":"মূল বিষয়: যিকর। এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম একটি সংক্ষিপ্ত কিন্তু ভারী যিকর শিক্ষা দিয়েছেন। জুয়াইরিয়া রাঃ সকাল থেকে চাশতের সময় পর্যন্ত তাঁর নামাযের স্থানে বসে ছিলেন। তখন নবী সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম বললেন, তিনি যাওয়ার পর চারটি কালেমা তিনবার বলেছেন, যা সেদিন তাঁর দীর্ঘ সময়ের পাঠের সঙ্গে ওজন করলে বেশি ভারী হবে। এই হাদিস থেকে বোঝা যায়, যিকরের মূল্য শুধু সময়ের দৈর্ঘ্যে নয়; বরং শব্দের অর্থ, আল্লাহর প্রশংসা ও আন্তরিকতার দিক থেকেও বড় হতে পারে। এখানে মূল দুআ হলো: সুবহানাল্লাহি ওয়া বিহামদিহি, আদাদা খালকিহি, ওয়া রিযা নাফসিহি, ওয়া যিনাতা আরশিহি, ওয়া মিদাদা কালিমাতিহি। বাংলা অর্থে এতে আল্লাহর পবিত্রতা ও প্রশংসা তাঁর সৃষ্টি, সন্তুষ্টি, আরশের ওজন এবং তাঁর কালেমার বিস্তারের সঙ্গে যুক্ত করে বলা হয়েছে।"},"teachings":["অল্প সময়েও অর্থবহ যিকর করা যায়।","আল্লাহর প্রশংসা ও পবিত্রতা বর্ণনা করা মুমিনের সুন্দর আমল।","রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম সহজ শব্দে বড় শিক্ষা দিয়েছেন।","যিকরের শব্দ ও অর্থ বুঝে পড়া বেশি মনোযোগ আনতে পারে।"],"related_hadiths":[{"id":"2018","book_id":"2","label":"Sahih Muslim"},{"id":"3380","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"2732","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | হাঁচির দোয়া ও ইসলামী আদব","description":"$book_name$ $hadith_number$ - $chapter_name$. হাঁচির পর আলহামদুলিল্লাহ বলা ও উত্তরে রহমতের দোয়া করার সুন্দর ইসলামী আদব এ হাদিসে শেখানো হয়েছে।"},"heading":{"title":"হাঁচির দোয়া: আলহামদুলিল্লাহ ও ইয়ারহামুকাল্লাহর আদব","description":"মূল বিষয়: আদব। এই হাদিসে হাঁচি দেওয়ার পর কী বলা উচিত এবং পাশে থাকা মুসলিম ভাই বা সাথী কীভাবে উত্তর দেবে, তা সহজভাবে শেখানো হয়েছে। নবী করীম সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম বলেছেন, কেউ হাঁচি দিলে সে যেন বলে, আলহামদুলিল্লাহ। অর্থাৎ সে আল্লাহর প্রশংসা করবে। তার ভাই বা সাথী উত্তরে বলবে, ইয়ারহামুকাল্লাহ, অর্থাৎ আল্লাহ তোমার প্রতি রহম করুন। এরপর হাঁচি দেওয়া ব্যক্তি বলবে, ইয়াহদীকুমুল্লাহু ওয়া ইউসলিহ বালাকুম, অর্থাৎ আল্লাহ তোমাদের হিদায়াত দিন এবং তোমাদের অবস্থা ঠিক করে দিন। এই ছোট্ট আদবের মধ্যে আল্লাহর প্রশংসা, একে অন্যের জন্য দোয়া, ভালো সম্পর্ক এবং সুন্দর কথা—সবই আছে। তাই হাঁচির দোয়া শুধু মুখের কথা নয়; এটি মুসলিমদের পারস্পরিক দোয়া ও সৌজন্যের একটি সহজ শিক্ষা।"},"teachings":["হাঁচির পর আল্লাহর প্রশংসা করা সুন্নত আদব।","অন্য মুসলিমের জন্য রহমতের দোয়া করা ভালো আচরণের অংশ।","দোয়ার জবাবে হিদায়াত ও অবস্থা ভালো হওয়ার দোয়া করা শেখানো হয়েছে।","ছোট ঘটনাতেও ইসলামে সুন্দর কথা বলার শিক্ষা আছে।"],"related_hadiths":[{"id":"201৮","book_id":"2","label":"Sahih Muslim"},{"id":"6245","book_id":"1","label":"Sahih Bukhari"},{"id":"2066","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | হাঁচির দোয়া ও ইসলামী আদব","description":"$book_name$ $hadith_number$ - $chapter_name$. হাঁচির পর আলহামদুলিল্লাহ বলা ও উত্তরে রহমতের দোয়া করার সুন্দর ইসলামী আদব এ হাদিসে শেখানো হয়েছে।"},"heading":{"title":"হাঁচির দোয়া: আলহামদুলিল্লাহ ও ইয়ারহামুকাল্লাহর আদব","description":"মূল বিষয়: আদব। এই হাদিসে হাঁচি দেওয়ার পর কী বলা উচিত এবং পাশে থাকা মুসলিম ভাই বা সাথী কীভাবে উত্তর দেবে, তা সহজভাবে শেখানো হয়েছে। নবী করীম সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম বলেছেন, কেউ হাঁচি দিলে সে যেন বলে, আলহামদুলিল্লাহ। অর্থাৎ সে আল্লাহর প্রশংসা করবে। তার ভাই বা সাথী উত্তরে বলবে, ইয়ারহামুকাল্লাহ, অর্থাৎ আল্লাহ তোমার প্রতি রহম করুন। এরপর হাঁচি দেওয়া ব্যক্তি বলবে, ইয়াহদীকুমুল্লাহু ওয়া ইউসলিহ বালাকুম, অর্থাৎ আল্লাহ তোমাদের হিদায়াত দিন এবং তোমাদের অবস্থা ঠিক করে দিন। এই ছোট্ট আদবের মধ্যে আল্লাহর প্রশংসা, একে অন্যের জন্য দোয়া, ভালো সম্পর্ক এবং সুন্দর কথা—সবই আছে। তাই হাঁচির দোয়া শুধু মুখের কথা নয়; এটি মুসলিমদের পারস্পরিক দোয়া ও সৌজন্যের একটি সহজ শিক্ষা।"},"teachings":["হাঁচির পর আল্লাহর প্রশংসা করা সুন্নত আদব।","অন্য মুসলিমের জন্য রহমতের দোয়া করা ভালো আচরণের অংশ।","দোয়ার জবাবে হিদায়াত ও অবস্থা ভালো হওয়ার দোয়া করা শেখানো হয়েছে।","ছোট ঘটনাতেও ইসলামে সুন্দর কথা বলার শিক্ষা আছে।"],"related_hadiths":[{"id":"2018","book_id":"2","label":"Sahih Muslim"},{"id":"6245","book_id":"1","label":"Sahih Bukhari"},{"id":"2066","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -1785,7 +1785,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রোগী দেখার দোয়া ও সান্ত্বনা","description":"$book_name$ $hadith_number$ - $chapter_name$. অসুস্থ মানুষকে দেখতে গিয়ে সান্ত্বনা দেওয়া ও পাপ মোচনের আশা জাগানো—এ হাদিসের কোমল শিক্ষা।"},"heading":{"title":"রোগী দেখার দোয়া: লা বাসা ত্বহুর ইনশাআল্লাহ","description":"মূল বিষয়: রোগী দেখা। এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম অসুস্থ ব্যক্তিকে দেখতে গেলে কী বলতেন, তা বলা হয়েছে। তিনি বলতেন, লা বাসা ত্বহুর ইনশাআল্লাহ। অর্থ হলো, চিন্তার কোনো কারণ নেই, আল্লাহ চাইলে এটি পাপ মোচনের কারণ হবে। এখানে রোগীর প্রতি কোমল ব্যবহার, ভালো কথা বলা এবং আশা জাগানোর শিক্ষা আছে। অসুস্থ মানুষ সাধারণত দুর্বল ও চিন্তিত থাকে। তখন তাকে ভয় না দেখিয়ে সুন্দর কথা বলা, আল্লাহর দিকে মন ফেরানো এবং সান্ত্বনা দেওয়া খুব দরকার। এই হাদিসে রোগী দেখার দোয়া শুধু একটি বাক্য নয়; এটি রোগীর মনকে শান্ত করার একটি সুন্নতি পদ্ধতি। তবে এখানে সবকিছু আল্লাহর ইচ্ছার সঙ্গে যুক্ত করা হয়েছে—ইনশাআল্লাহ। তাই কথা বলার সময় আশা রাখা হবে, কিন্তু অতিরঞ্জন করা হবে না।"},"teachings":["অসুস্থ মানুষকে দেখতে গেলে সান্ত্বনামূলক কথা বলা উচিত।","রোগের সময় আল্লাহর দিকে আশা নিয়ে মন ফেরানো শেখানো হয়েছে।","ইনশাআল্লাহ বলে বিষয়টি আল্লাহর ইচ্ছার সঙ্গে যুক্ত করা হয়েছে।","রোগী দেখার সময় সংক্ষিপ্ত দোয়া ও কোমল ভাষা সুন্দর আদব।"],"related_hadiths":[{"id":"2202","book_id":"2","label":"Sahih Muslim"},{"id":"256৮","book_id":"2","label":"Sahih Muslim"},{"id":"2066","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রোগী দেখার দোয়া ও সান্ত্বনা","description":"$book_name$ $hadith_number$ - $chapter_name$. অসুস্থ মানুষকে দেখতে গিয়ে সান্ত্বনা দেওয়া ও পাপ মোচনের আশা জাগানো—এ হাদিসের কোমল শিক্ষা।"},"heading":{"title":"রোগী দেখার দোয়া: লা বাসা ত্বহুর ইনশাআল্লাহ","description":"মূল বিষয়: রোগী দেখা। এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম অসুস্থ ব্যক্তিকে দেখতে গেলে কী বলতেন, তা বলা হয়েছে। তিনি বলতেন, লা বাসা ত্বহুর ইনশাআল্লাহ। অর্থ হলো, চিন্তার কোনো কারণ নেই, আল্লাহ চাইলে এটি পাপ মোচনের কারণ হবে। এখানে রোগীর প্রতি কোমল ব্যবহার, ভালো কথা বলা এবং আশা জাগানোর শিক্ষা আছে। অসুস্থ মানুষ সাধারণত দুর্বল ও চিন্তিত থাকে। তখন তাকে ভয় না দেখিয়ে সুন্দর কথা বলা, আল্লাহর দিকে মন ফেরানো এবং সান্ত্বনা দেওয়া খুব দরকার। এই হাদিসে রোগী দেখার দোয়া শুধু একটি বাক্য নয়; এটি রোগীর মনকে শান্ত করার একটি সুন্নতি পদ্ধতি। তবে এখানে সবকিছু আল্লাহর ইচ্ছার সঙ্গে যুক্ত করা হয়েছে—ইনশাআল্লাহ। তাই কথা বলার সময় আশা রাখা হবে, কিন্তু অতিরঞ্জন করা হবে না।"},"teachings":["অসুস্থ মানুষকে দেখতে গেলে সান্ত্বনামূলক কথা বলা উচিত।","রোগের সময় আল্লাহর দিকে আশা নিয়ে মন ফেরানো শেখানো হয়েছে।","ইনশাআল্লাহ বলে বিষয়টি আল্লাহর ইচ্ছার সঙ্গে যুক্ত করা হয়েছে।","রোগী দেখার সময় সংক্ষিপ্ত দোয়া ও কোমল ভাষা সুন্দর আদব।"],"related_hadiths":[{"id":"2202","book_id":"2","label":"Sahih Muslim"},{"id":"2568","book_id":"2","label":"Sahih Muslim"},{"id":"2066","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1807,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শরীরের ব্যথার দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. শরীরের ব্যথার স্থানে হাত রেখে বিসমিল্লাহ ও আশ্রয়ের দোয়া পড়ার সুন্নতি পদ্ধতি এ হাদিসে আছে।"},"heading":{"title":"শরীরের ব্যথার দোয়া: বিসমিল্লাহ ও আল্লাহর আশ্রয়","description":"মূল বিষয়: দোয়া। এই হাদিসে শরীরের ব্যথা হলে কীভাবে দোয়া করতে হবে, তা রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম শিখিয়েছেন। একজন সাহাবী তাঁর শরীরের ব্যথার কথা জানালে নবী সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম বললেন, যেখানে ব্যথা অনুভব করছো সেখানে হাত রাখো। তারপর তিনবার বিসমিল্লাহ বলো এবং সাতবার পড়ো: আউযু বিল্লাহি ওয়া কুদরতিহি মিন শাররি মা আজিদু ওয়া উহাযির। অর্থ হলো, আমি আল্লাহর মর্যাদা ও তাঁর ক্ষমতার মাধ্যমে সেই ব্যথা থেকে আশ্রয় চাই, যা আমি অনুভব করছি এবং যার আশঙ্কা করছি। এই হাদিসে চিকিৎসা বাদ দেওয়ার কথা বলা হয়নি; বরং ব্যথার সময় আল্লাহর সাহায্য চাওয়ার একটি সুন্নতি দোয়া শেখানো হয়েছে। এতে বান্দা নিজের দুর্বলতা বুঝে আল্লাহর শক্তি ও আশ্রয়ের দিকে ফিরে যায়।"},"teachings":["ব্যথার সময় আল্লাহর নামে দোয়া করা শেখানো হয়েছে।","ব্যথার স্থানে হাত রেখে নির্দিষ্ট দোয়া পড়ার নির্দেশ আছে।","ভয় ও কষ্টের সময় আল্লাহর আশ্রয় চাওয়া মুমিনের আদব।","দোয়ার ভাষায় নিজের অনুভূত কষ্ট ও আশঙ্কার কথা বলা যায়।"],"related_hadiths":[{"id":"5662","book_id":"1","label":"Sahih Bukhari"},{"id":"৯1৮","book_id":"2","label":"Sahih Muslim"},{"id":"256৮","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শরীরের ব্যথার দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. শরীরের ব্যথার স্থানে হাত রেখে বিসমিল্লাহ ও আশ্রয়ের দোয়া পড়ার সুন্নতি পদ্ধতি এ হাদিসে আছে।"},"heading":{"title":"শরীরের ব্যথার দোয়া: বিসমিল্লাহ ও আল্লাহর আশ্রয়","description":"মূল বিষয়: দোয়া। এই হাদিসে শরীরের ব্যথা হলে কীভাবে দোয়া করতে হবে, তা রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম শিখিয়েছেন। একজন সাহাবী তাঁর শরীরের ব্যথার কথা জানালে নবী সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম বললেন, যেখানে ব্যথা অনুভব করছো সেখানে হাত রাখো। তারপর তিনবার বিসমিল্লাহ বলো এবং সাতবার পড়ো: আউযু বিল্লাহি ওয়া কুদরতিহি মিন শাররি মা আজিদু ওয়া উহাযির। অর্থ হলো, আমি আল্লাহর মর্যাদা ও তাঁর ক্ষমতার মাধ্যমে সেই ব্যথা থেকে আশ্রয় চাই, যা আমি অনুভব করছি এবং যার আশঙ্কা করছি। এই হাদিসে চিকিৎসা বাদ দেওয়ার কথা বলা হয়নি; বরং ব্যথার সময় আল্লাহর সাহায্য চাওয়ার একটি সুন্নতি দোয়া শেখানো হয়েছে। এতে বান্দা নিজের দুর্বলতা বুঝে আল্লাহর শক্তি ও আশ্রয়ের দিকে ফিরে যায়।"},"teachings":["ব্যথার সময় আল্লাহর নামে দোয়া করা শেখানো হয়েছে।","ব্যথার স্থানে হাত রেখে নির্দিষ্ট দোয়া পড়ার নির্দেশ আছে।","ভয় ও কষ্টের সময় আল্লাহর আশ্রয় চাওয়া মুমিনের আদব।","দোয়ার ভাষায় নিজের অনুভূত কষ্ট ও আশঙ্কার কথা বলা যায়।"],"related_hadiths":[{"id":"5662","book_id":"1","label":"Sahih Bukhari"},{"id":"918","book_id":"2","label":"Sahih Muslim"},{"id":"2568","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মোরগের ডাক ও গাধার আওয়াজের দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. মোরগের ডাক শুনে আল্লাহর অনুগ্রহ চাওয়া ও গাধার আওয়াজে শয়তান থেকে আশ্রয় চাওয়ার শিক্ষা আছে।"},"heading":{"title":"মোরগের ডাক শুনলে দোয়া ও গাধার আওয়াজ শুনলে আশ্রয়","description":"মূল বিষয়: দোয়া। এই হাদিসে নবী করীম সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম দুটি শব্দ শোনার সময় দুটি ভিন্ন আমল শিখিয়েছেন। তিনি বলেছেন, মোরগের ডাক শুনলে আল্লাহর অনুগ্রহ চাইতে হবে। কারণ, সে ফেরেশতা দেখেছে। আর গাধার আওয়াজ শুনলে আল্লাহর কাছে শয়তান থেকে আশ্রয় চাইতে হবে। কারণ, সে শয়তান দেখেছে। এই হাদিসে আমাদের শেখানো হয়েছে, দৈনন্দিন জীবনের সাধারণ শব্দও একজন মুমিনকে আল্লাহর দিকে ফিরিয়ে নিতে পারে। মোরগের ডাক শুনে আল্লাহর রহমত ও অনুগ্রহ চাওয়া হবে। আবার গাধার আওয়াজ শুনে অশুভ কিছু নিয়ে ভয় ছড়ানো নয়; বরং শয়তান থেকে আল্লাহর আশ্রয় চাওয়া হবে। এভাবে ছোট ছোট মুহূর্তে দোয়া ও যিকরের অভ্যাস তৈরি হয়।"},"teachings":["মোরগের ডাক শুনে আল্লাহর অনুগ্রহ চাওয়ার শিক্ষা আছে।","গাধার আওয়াজ শুনে শয়তান থেকে আল্লাহর আশ্রয় চাইতে বলা হয়েছে।","সাধারণ শব্দও মুমিনকে দোয়ার দিকে ফিরিয়ে নিতে পারে।","ভয় না ছড়িয়ে আল্লাহর কাছে আশ্রয় চাওয়া উচিত।"],"related_hadiths":[{"id":"201৮","book_id":"2","label":"Sahih Muslim"},{"id":"৮৯৯","book_id":"2","label":"Sahih Muslim"},{"id":"6322","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মোরগের ডাক ও গাধার আওয়াজের দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. মোরগের ডাক শুনে আল্লাহর অনুগ্রহ চাওয়া ও গাধার আওয়াজে শয়তান থেকে আশ্রয় চাওয়ার শিক্ষা আছে।"},"heading":{"title":"মোরগের ডাক শুনলে দোয়া ও গাধার আওয়াজ শুনলে আশ্রয়","description":"মূল বিষয়: দোয়া। এই হাদিসে নবী করীম সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম দুটি শব্দ শোনার সময় দুটি ভিন্ন আমল শিখিয়েছেন। তিনি বলেছেন, মোরগের ডাক শুনলে আল্লাহর অনুগ্রহ চাইতে হবে। কারণ, সে ফেরেশতা দেখেছে। আর গাধার আওয়াজ শুনলে আল্লাহর কাছে শয়তান থেকে আশ্রয় চাইতে হবে। কারণ, সে শয়তান দেখেছে। এই হাদিসে আমাদের শেখানো হয়েছে, দৈনন্দিন জীবনের সাধারণ শব্দও একজন মুমিনকে আল্লাহর দিকে ফিরিয়ে নিতে পারে। মোরগের ডাক শুনে আল্লাহর রহমত ও অনুগ্রহ চাওয়া হবে। আবার গাধার আওয়াজ শুনে অশুভ কিছু নিয়ে ভয় ছড়ানো নয়; বরং শয়তান থেকে আল্লাহর আশ্রয় চাওয়া হবে। এভাবে ছোট ছোট মুহূর্তে দোয়া ও যিকরের অভ্যাস তৈরি হয়।"},"teachings":["মোরগের ডাক শুনে আল্লাহর অনুগ্রহ চাওয়ার শিক্ষা আছে।","গাধার আওয়াজ শুনে শয়তান থেকে আল্লাহর আশ্রয় চাইতে বলা হয়েছে।","সাধারণ শব্দও মুমিনকে দোয়ার দিকে ফিরিয়ে নিতে পারে।","ভয় না ছড়িয়ে আল্লাহর কাছে আশ্রয় চাওয়া উচিত।"],"related_hadiths":[{"id":"2018","book_id":"2","label":"Sahih Muslim"},{"id":"899","book_id":"2","label":"Sahih Muslim"},{"id":"6322","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | বৃষ্টির দোয়া ও উপকারী বৃষ্টি","description":"$book_name$ $hadith_number$ - $chapter_name$. বৃষ্টি দেখলে উপকারী বৃষ্টির জন্য আল্লাহর কাছে দোয়া করার সুন্নতি শিক্ষা এ হাদিসে পাওয়া যায়।"},"heading":{"title":"বৃষ্টির দোয়া: আল্লাহুম্মা সাইয়েবান নাফিআ","description":"মূল বিষয়: বৃষ্টির দোয়া। এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম বৃষ্টি দেখলে যে দোয়া পড়তেন, তা শেখানো হয়েছে। তিনি বলতেন, আল্লাহুম্মা সাইয়েবান নাফিআ। এর অর্থ: হে আল্লাহ, মুষলধারে উপকারী বৃষ্টি বর্ষাও। এখানে বৃষ্টিকে শুধু প্রাকৃতিক ঘটনা হিসেবে দেখা হয়নি; বরং আল্লাহর দান হিসেবে দেখা হয়েছে। তাই বৃষ্টি শুরু হলে অভিযোগ বা অস্থিরতার বদলে আল্লাহর কাছে উপকার চাওয়া শেখানো হয়েছে। দোয়াটিতে গুরুত্বপূর্ণ কথা হলো ‘নাফিআ’—উপকারী। অর্থাৎ বৃষ্টি যেন কল্যাণ নিয়ে আসে, ক্ষতি নয়। এই হাদিস আমাদের শেখায়, প্রকৃতির পরিবর্তন দেখলেও মুমিনের জিহ্বা দোয়ার সঙ্গে যুক্ত থাকে। বৃষ্টির দোয়া ছোট হলেও এর অর্থ গভীর এবং দৈনন্দিন জীবনে সহজে আমল করা যায়।"},"teachings":["বৃষ্টি দেখলে আল্লাহর কাছে উপকারী বৃষ্টি চাওয়া উচিত।","প্রকৃতির ঘটনায় আল্লাহর দানের কথা স্মরণ করা শেখানো হয়েছে।","দোয়া সংক্ষিপ্ত হলেও অর্থপূর্ণ হতে পারে।","বৃষ্টির সময় অভিযোগের বদলে কল্যাণের দোয়া করা সুন্দর আদব।"],"related_hadiths":[{"id":"৮৯৮","book_id":"2","label":"Sahih Muslim"},{"id":"৮৯৯","book_id":"2","label":"Sahih Muslim"},{"id":"272৯","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | বৃষ্টির দোয়া ও উপকারী বৃষ্টি","description":"$book_name$ $hadith_number$ - $chapter_name$. বৃষ্টি দেখলে উপকারী বৃষ্টির জন্য আল্লাহর কাছে দোয়া করার সুন্নতি শিক্ষা এ হাদিসে পাওয়া যায়।"},"heading":{"title":"বৃষ্টির দোয়া: আল্লাহুম্মা সাইয়েবান নাফিআ","description":"মূল বিষয়: বৃষ্টির দোয়া। এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম বৃষ্টি দেখলে যে দোয়া পড়তেন, তা শেখানো হয়েছে। তিনি বলতেন, আল্লাহুম্মা সাইয়েবান নাফিআ। এর অর্থ: হে আল্লাহ, মুষলধারে উপকারী বৃষ্টি বর্ষাও। এখানে বৃষ্টিকে শুধু প্রাকৃতিক ঘটনা হিসেবে দেখা হয়নি; বরং আল্লাহর দান হিসেবে দেখা হয়েছে। তাই বৃষ্টি শুরু হলে অভিযোগ বা অস্থিরতার বদলে আল্লাহর কাছে উপকার চাওয়া শেখানো হয়েছে। দোয়াটিতে গুরুত্বপূর্ণ কথা হলো ‘নাফিআ’—উপকারী। অর্থাৎ বৃষ্টি যেন কল্যাণ নিয়ে আসে, ক্ষতি নয়। এই হাদিস আমাদের শেখায়, প্রকৃতির পরিবর্তন দেখলেও মুমিনের জিহ্বা দোয়ার সঙ্গে যুক্ত থাকে। বৃষ্টির দোয়া ছোট হলেও এর অর্থ গভীর এবং দৈনন্দিন জীবনে সহজে আমল করা যায়।"},"teachings":["বৃষ্টি দেখলে আল্লাহর কাছে উপকারী বৃষ্টি চাওয়া উচিত।","প্রকৃতির ঘটনায় আল্লাহর দানের কথা স্মরণ করা শেখানো হয়েছে।","দোয়া সংক্ষিপ্ত হলেও অর্থপূর্ণ হতে পারে।","বৃষ্টির সময় অভিযোগের বদলে কল্যাণের দোয়া করা সুন্দর আদব।"],"related_hadiths":[{"id":"898","book_id":"2","label":"Sahih Muslim"},{"id":"899","book_id":"2","label":"Sahih Muslim"},{"id":"2729","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঘরে প্রবেশের সময় যিকর","description":"$book_name$ $hadith_number$ - $chapter_name$. ঘরে ঢোকার সময় আল্লাহর যিকর করলে শয়তান থেকে ঘর ও খাবারকে বাঁচানোর শিক্ষা এ হাদিসে আছে।"},"heading":{"title":"ঘরে প্রবেশের সময় যিকর ও শয়তান থেকে বাঁচার শিক্ষা","description":"মূল বিষয়: ঘরের আদব। এই হাদিসে ঘরে প্রবেশের সময় আল্লাহর যিকরের গুরুত্ব বলা হয়েছে। রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম বলেছেন, মানুষ যখন নিজের বাড়িতে প্রবেশ করার সময় মহান আল্লাহর যিকর করে, তখন শয়তান তার সাথীদের বলে, তোমরা এখানে রাত কাটাতে পারবে না, রাতের খাবারও পাবে না। কিন্তু প্রবেশের সময় যদি আল্লাহর যিকর না করা হয়, তখন সে বলে, তোমরা রাত কাটাতেও পারবে এবং খাবারও পাবে। এই বর্ণনা ঘরে ঢোকার সময় আল্লাহকে স্মরণ করার গুরুত্ব বুঝিয়ে দেয়। ঘর শুধু থাকার জায়গা নয়; সেখানে শান্তি, খাবার ও পরিবার থাকে। তাই ঘরে ঢোকার সময় যিকর করা একটি সহজ কিন্তু গুরুত্বপূর্ণ আদব। এতে বান্দা বুঝে নেয়, ঘরের নিরাপত্তা ও বরকত আল্লাহর কাছেই চাওয়া উচিত।"},"teachings":["ঘরে প্রবেশের সময় আল্লাহর যিকর করা উচিত।","যিকর না করলে শয়তানের অংশ নেওয়ার কথা হাদিসে এসেছে।","বাড়ির খাবার ও রাতযাপনেও আল্লাহকে স্মরণ করার শিক্ষা আছে।","দৈনন্দিন ঘরোয়া জীবনেও সুন্নতি আদব মানা যায়।"],"related_hadiths":[{"id":"6322","book_id":"1","label":"Sahih Bukhari"},{"id":"33৮0","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"2726","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঘরে প্রবেশের সময় যিকর","description":"$book_name$ $hadith_number$ - $chapter_name$. ঘরে ঢোকার সময় আল্লাহর যিকর করলে শয়তান থেকে ঘর ও খাবারকে বাঁচানোর শিক্ষা এ হাদিসে আছে।"},"heading":{"title":"ঘরে প্রবেশের সময় যিকর ও শয়তান থেকে বাঁচার শিক্ষা","description":"মূল বিষয়: ঘরের আদব। এই হাদিসে ঘরে প্রবেশের সময় আল্লাহর যিকরের গুরুত্ব বলা হয়েছে। রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম বলেছেন, মানুষ যখন নিজের বাড়িতে প্রবেশ করার সময় মহান আল্লাহর যিকর করে, তখন শয়তান তার সাথীদের বলে, তোমরা এখানে রাত কাটাতে পারবে না, রাতের খাবারও পাবে না। কিন্তু প্রবেশের সময় যদি আল্লাহর যিকর না করা হয়, তখন সে বলে, তোমরা রাত কাটাতেও পারবে এবং খাবারও পাবে। এই বর্ণনা ঘরে ঢোকার সময় আল্লাহকে স্মরণ করার গুরুত্ব বুঝিয়ে দেয়। ঘর শুধু থাকার জায়গা নয়; সেখানে শান্তি, খাবার ও পরিবার থাকে। তাই ঘরে ঢোকার সময় যিকর করা একটি সহজ কিন্তু গুরুত্বপূর্ণ আদব। এতে বান্দা বুঝে নেয়, ঘরের নিরাপত্তা ও বরকত আল্লাহর কাছেই চাওয়া উচিত।"},"teachings":["ঘরে প্রবেশের সময় আল্লাহর যিকর করা উচিত।","যিকর না করলে শয়তানের অংশ নেওয়ার কথা হাদিসে এসেছে।","বাড়ির খাবার ও রাতযাপনেও আল্লাহকে স্মরণ করার শিক্ষা আছে।","দৈনন্দিন ঘরোয়া জীবনেও সুন্নতি আদব মানা যায়।"],"related_hadiths":[{"id":"6322","book_id":"1","label":"Sahih Bukhari"},{"id":"3380","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"2726","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -1895,7 +1895,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মজলিসে যিকর ও দরূদের গুরুত্ব","description":"$book_name$ $hadith_number$ - $chapter_name$. যে মজলিসে আল্লাহর যিকর ও নবীর প্রতি দরূদ নেই, তা অনুতাপের কারণ হতে পারে—এ হাদিসের শিক্ষা।"},"heading":{"title":"মজলিসে যিকর ও দরূদ: অনুতাপ থেকে বাঁচার শিক্ষা","description":"মূল বিষয়: মজলিসের আদব। এই হাদিসে নবী করীম সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম এমন মজলিসের কথা বলেছেন, যেখানে মানুষ বসে কিন্তু আল্লাহর যিকর করে না এবং নবীর প্রতি দরূদও পাঠ করে না। তিনি বলেছেন, এমন মজলিস তাদের অনুতাপের কারণ হয়। এরপর বলা হয়েছে, আল্লাহ চাইলে তাদের শাস্তি দিতে পারেন, আবার ক্ষমাও করতে পারেন। এই হাদিস আমাদের কথাবার্তা ও বসার জায়গাকে আল্লাহর স্মরণ থেকে একেবারে খালি না রাখার শিক্ষা দেয়। মজলিস মানে শুধু বড় সভা নয়; মানুষ যেখানে বসে কথা বলে, সেটিও হতে পারে। তাই আলাপের মাঝে আল্লাহর যিকর, ভালো কথা এবং নবী সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লামের প্রতি দরূদ পাঠ করা মুমিনের সুন্দর অভ্যাস। এতে সময়ের ব্যবহার ভালো হয় এবং অনুতাপের কারণ কমে।"},"teachings":["মজলিসে আল্লাহর যিকর থাকা উচিত।","নবী সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লামের প্রতি দরূদ পাঠের গুরুত্ব আছে।","যিকরহীন মজলিস অনুতাপের কারণ হতে পারে।","মানুষের বসা ও আলাপও আমলের অংশ হতে পারে।"],"related_hadiths":[{"id":"201৮","book_id":"2","label":"Sahih Muslim"},{"id":"2726","book_id":"2","label":"Sahih Muslim"},{"id":"2732","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মজলিসে যিকর ও দরূদের গুরুত্ব","description":"$book_name$ $hadith_number$ - $chapter_name$. যে মজলিসে আল্লাহর যিকর ও নবীর প্রতি দরূদ নেই, তা অনুতাপের কারণ হতে পারে—এ হাদিসের শিক্ষা।"},"heading":{"title":"মজলিসে যিকর ও দরূদ: অনুতাপ থেকে বাঁচার শিক্ষা","description":"মূল বিষয়: মজলিসের আদব। এই হাদিসে নবী করীম সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম এমন মজলিসের কথা বলেছেন, যেখানে মানুষ বসে কিন্তু আল্লাহর যিকর করে না এবং নবীর প্রতি দরূদও পাঠ করে না। তিনি বলেছেন, এমন মজলিস তাদের অনুতাপের কারণ হয়। এরপর বলা হয়েছে, আল্লাহ চাইলে তাদের শাস্তি দিতে পারেন, আবার ক্ষমাও করতে পারেন। এই হাদিস আমাদের কথাবার্তা ও বসার জায়গাকে আল্লাহর স্মরণ থেকে একেবারে খালি না রাখার শিক্ষা দেয়। মজলিস মানে শুধু বড় সভা নয়; মানুষ যেখানে বসে কথা বলে, সেটিও হতে পারে। তাই আলাপের মাঝে আল্লাহর যিকর, ভালো কথা এবং নবী সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লামের প্রতি দরূদ পাঠ করা মুমিনের সুন্দর অভ্যাস। এতে সময়ের ব্যবহার ভালো হয় এবং অনুতাপের কারণ কমে।"},"teachings":["মজলিসে আল্লাহর যিকর থাকা উচিত।","নবী সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লামের প্রতি দরূদ পাঠের গুরুত্ব আছে।","যিকরহীন মজলিস অনুতাপের কারণ হতে পারে।","মানুষের বসা ও আলাপও আমলের অংশ হতে পারে।"],"related_hadiths":[{"id":"2018","book_id":"2","label":"Sahih Muslim"},{"id":"2726","book_id":"2","label":"Sahih Muslim"},{"id":"2732","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -1917,7 +1917,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পায়খানায় প্রবেশের দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. পায়খানায় প্রবেশের আগে খবিস জিন নরনারীর অনিষ্ট থেকে আল্লাহর আশ্রয় চাওয়ার দোয়া শেখানো হয়েছে।"},"heading":{"title":"পায়খানায় প্রবেশের দোয়া ও আল্লাহর আশ্রয়","description":"মূল বিষয়: পবিত্রতার আদব। এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম পায়খানায় প্রবেশের আগে যে দোয়া পড়তেন, তা এসেছে। তিনি বলতেন: আল্লাহুম্মা ইন্নী আউযু বিকা মিনাল খুবুসী ওয়াল খাবাইস। অর্থ হলো, হে আল্লাহ, আমি তোমার কাছে খবিস জিন নরনারীর অনিষ্ট থেকে আশ্রয় চাই। এখানে শিক্ষা হলো, মানুষের এমন জায়গায় যাওয়ার সময়ও আল্লাহর আশ্রয় দরকার, যেখানে সে একা থাকে এবং সাধারণত অন্যের নজর থেকে দূরে থাকে। ইসলামে দৈনন্দিন কাজেও আদব আছে। পায়খানায় প্রবেশের দোয়া ছোট হলেও এতে আল্লাহর কাছে নিরাপত্তা চাওয়ার বিষয়টি স্পষ্ট। এই দোয়া মানুষকে মনে করিয়ে দেয়, নিজের শক্তি যথেষ্ট নয়; প্রতিটি অবস্থায় আল্লাহর সাহায্য দরকার।"},"teachings":["পায়খানায় প্রবেশের আগে আল্লাহর আশ্রয় চাওয়ার শিক্ষা আছে।","একান্ত অবস্থাতেও আল্লাহকে স্মরণ করা উচিত।","খারাপ জিনের অনিষ্ট থেকে আশ্রয় চাওয়ার দোয়া শেখানো হয়েছে।","দৈনন্দিন কাজের মধ্যেও সুন্নতি আদব আছে।"],"related_hadiths":[{"id":"2202","book_id":"2","label":"Sahih Muslim"},{"id":"201৮","book_id":"2","label":"Sahih Muslim"},{"id":"272৯","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পায়খানায় প্রবেশের দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. পায়খানায় প্রবেশের আগে খবিস জিন নরনারীর অনিষ্ট থেকে আল্লাহর আশ্রয় চাওয়ার দোয়া শেখানো হয়েছে।"},"heading":{"title":"পায়খানায় প্রবেশের দোয়া ও আল্লাহর আশ্রয়","description":"মূল বিষয়: পবিত্রতার আদব। এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম পায়খানায় প্রবেশের আগে যে দোয়া পড়তেন, তা এসেছে। তিনি বলতেন: আল্লাহুম্মা ইন্নী আউযু বিকা মিনাল খুবুসী ওয়াল খাবাইস। অর্থ হলো, হে আল্লাহ, আমি তোমার কাছে খবিস জিন নরনারীর অনিষ্ট থেকে আশ্রয় চাই। এখানে শিক্ষা হলো, মানুষের এমন জায়গায় যাওয়ার সময়ও আল্লাহর আশ্রয় দরকার, যেখানে সে একা থাকে এবং সাধারণত অন্যের নজর থেকে দূরে থাকে। ইসলামে দৈনন্দিন কাজেও আদব আছে। পায়খানায় প্রবেশের দোয়া ছোট হলেও এতে আল্লাহর কাছে নিরাপত্তা চাওয়ার বিষয়টি স্পষ্ট। এই দোয়া মানুষকে মনে করিয়ে দেয়, নিজের শক্তি যথেষ্ট নয়; প্রতিটি অবস্থায় আল্লাহর সাহায্য দরকার।"},"teachings":["পায়খানায় প্রবেশের আগে আল্লাহর আশ্রয় চাওয়ার শিক্ষা আছে।","একান্ত অবস্থাতেও আল্লাহকে স্মরণ করা উচিত।","খারাপ জিনের অনিষ্ট থেকে আশ্রয় চাওয়ার দোয়া শেখানো হয়েছে।","দৈনন্দিন কাজের মধ্যেও সুন্নতি আদব আছে।"],"related_hadiths":[{"id":"2202","book_id":"2","label":"Sahih Muslim"},{"id":"2018","book_id":"2","label":"Sahih Muslim"},{"id":"2729","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -1939,7 +1939,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ফরজ গোসলের সুন্নতি পদ্ধতি","description":"$book_name$ $hadith_number$ - $chapter_name$. ফরজ গোসলে হাত ধোয়া, ওজু করা, মাথায় পানি দেওয়া ও পুরো শরীর ধোয়ার পদ্ধতি।"},"heading":{"title":"ফরজ গোসলের নিয়ম: রাসূল صلى الله عليه وسلم-এর শেখানো ধাপে ধাপে পদ্ধতি","description":"এই হাদিসে ফরজ গোসলের নিয়ম পরিষ্কারভাবে বর্ণিত হয়েছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম যখন ফরজ গোসল করতেন, তখন প্রথমে নিজের দুই হাত ধৌত করতেন। এরপর নামাজের ওজুর মতো ওজু করতেন। তারপর দুই হাত দিয়ে তিন অঞ্জলি পানি মাথায় ঢালতেন। শেষে পুরো শরীরে পানি ঢেলে দিতেন। এই বর্ণনা থেকে বোঝা যায়, ফরজ গোসল শুধু শরীরে পানি ঢেলে শেষ করার বিষয় নয়; বরং এর একটি সুন্দর ধাপ আছে। হাত ধোয়া, ওজু করা, মাথায় পানি দেওয়া এবং পুরো শরীর ধোয়া—এই ধারাটি খুব সহজ ও পরিষ্কার। ফরজ গোসলের পদ্ধতি, গোসলের সুন্নাহ এবং পবিত্রতার নিয়ম জানতে চাইলে এই হাদিস সরাসরি একটি ব্যবহারযোগ্য নির্দেশনা দেয়।"},"teachings":["ফরজ গোসলের শুরুতে দুই হাত ধোয়ার আমল আছে।","গোসলের আগে নামাজের ওজুর মতো ওজু করা হাদিসে এসেছে।","মাথায় তিন অঞ্জলি পানি ঢালার বর্ণনা রয়েছে।","শেষে পুরো শরীরে পানি পৌঁছানো ফরজ গোসলের মূল অংশ।"],"related_hadiths":[{"id":"201","book_id":"1","label":"Sahih Bukhari"},{"id":"325","book_id":"2","label":"Sahih Muslim"},{"id":"24৮","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ফরজ গোসলের সুন্নতি পদ্ধতি","description":"$book_name$ $hadith_number$ - $chapter_name$. ফরজ গোসলে হাত ধোয়া, ওজু করা, মাথায় পানি দেওয়া ও পুরো শরীর ধোয়ার পদ্ধতি।"},"heading":{"title":"ফরজ গোসলের নিয়ম: রাসূল صلى الله عليه وسلم-এর শেখানো ধাপে ধাপে পদ্ধতি","description":"এই হাদিসে ফরজ গোসলের নিয়ম পরিষ্কারভাবে বর্ণিত হয়েছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম যখন ফরজ গোসল করতেন, তখন প্রথমে নিজের দুই হাত ধৌত করতেন। এরপর নামাজের ওজুর মতো ওজু করতেন। তারপর দুই হাত দিয়ে তিন অঞ্জলি পানি মাথায় ঢালতেন। শেষে পুরো শরীরে পানি ঢেলে দিতেন। এই বর্ণনা থেকে বোঝা যায়, ফরজ গোসল শুধু শরীরে পানি ঢেলে শেষ করার বিষয় নয়; বরং এর একটি সুন্দর ধাপ আছে। হাত ধোয়া, ওজু করা, মাথায় পানি দেওয়া এবং পুরো শরীর ধোয়া—এই ধারাটি খুব সহজ ও পরিষ্কার। ফরজ গোসলের পদ্ধতি, গোসলের সুন্নাহ এবং পবিত্রতার নিয়ম জানতে চাইলে এই হাদিস সরাসরি একটি ব্যবহারযোগ্য নির্দেশনা দেয়।"},"teachings":["ফরজ গোসলের শুরুতে দুই হাত ধোয়ার আমল আছে।","গোসলের আগে নামাজের ওজুর মতো ওজু করা হাদিসে এসেছে।","মাথায় তিন অঞ্জলি পানি ঢালার বর্ণনা রয়েছে।","শেষে পুরো শরীরে পানি পৌঁছানো ফরজ গোসলের মূল অংশ।"],"related_hadiths":[{"id":"201","book_id":"1","label":"Sahih Bukhari"},{"id":"325","book_id":"2","label":"Sahih Muslim"},{"id":"248","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঝড়-তুফানের দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. ঝড়-তুফানের কল্যাণ চাওয়া এবং তার অনিষ্ট থেকে আল্লাহর আশ্রয় নেওয়ার দোয়া এ হাদিসে আছে।"},"heading":{"title":"ঝড়-তুফানের দোয়া: কল্যাণ চাওয়া ও অনিষ্ট থেকে আশ্রয়","description":"মূল বিষয়: বিপদের দোয়া। এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম ঝড়-তুফানের সময় যে দোয়া পড়তেন, তা বলা হয়েছে। দোয়ায় তিনি ঝড়ের কল্যাণ, তার ভেতরে থাকা কল্যাণ এবং যার জন্য তা পাঠানো হয়েছে সেই কল্যাণ আল্লাহর কাছে চাইতেন। একই সঙ্গে তিনি ঝড়ের অনিষ্ট, তার ভেতরের অনিষ্ট এবং তার সঙ্গে পাঠানো ক্ষতির অনিষ্ট থেকে আল্লাহর আশ্রয় চাইতেন। এই দোয়া খুব ভারসাম্যপূর্ণ। এতে শুধু ভয় নেই, আবার শুধু নিশ্চিন্ততাও নেই। বরং কল্যাণ চাইতে বলা হয়েছে এবং ক্ষতি থেকে বাঁচার জন্য আল্লাহর আশ্রয় নিতে শেখানো হয়েছে। ঝড়-তুফানের দোয়া আমাদের মনে করায়, প্রকৃতির বড় ঘটনার সামনে মানুষ দুর্বল। তাই মুমিন আতঙ্ক ছড়ায় না; আল্লাহর কাছে ভালো চায় এবং অনিষ্ট থেকে আশ্রয় নেয়।"},"teachings":["ঝড়-তুফানের সময় আল্লাহর কাছে কল্যাণ চাওয়া উচিত।","প্রাকৃতিক বিপদের অনিষ্ট থেকে আল্লাহর আশ্রয় নিতে শেখানো হয়েছে।","ভয়ের সময় দোয়া মুমিনের মনকে আল্লাহর দিকে ফেরায়।","দোয়ায় কল্যাণ ও নিরাপত্তা—দুটিই চাওয়া যায়।"],"related_hadiths":[{"id":"1032","book_id":"1","label":"Sahih Bukhari"},{"id":"৮৯৮","book_id":"2","label":"Sahih Muslim"},{"id":"272৯","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঝড়-তুফানের দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. ঝড়-তুফানের কল্যাণ চাওয়া এবং তার অনিষ্ট থেকে আল্লাহর আশ্রয় নেওয়ার দোয়া এ হাদিসে আছে।"},"heading":{"title":"ঝড়-তুফানের দোয়া: কল্যাণ চাওয়া ও অনিষ্ট থেকে আশ্রয়","description":"মূল বিষয়: বিপদের দোয়া। এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম ঝড়-তুফানের সময় যে দোয়া পড়তেন, তা বলা হয়েছে। দোয়ায় তিনি ঝড়ের কল্যাণ, তার ভেতরে থাকা কল্যাণ এবং যার জন্য তা পাঠানো হয়েছে সেই কল্যাণ আল্লাহর কাছে চাইতেন। একই সঙ্গে তিনি ঝড়ের অনিষ্ট, তার ভেতরের অনিষ্ট এবং তার সঙ্গে পাঠানো ক্ষতির অনিষ্ট থেকে আল্লাহর আশ্রয় চাইতেন। এই দোয়া খুব ভারসাম্যপূর্ণ। এতে শুধু ভয় নেই, আবার শুধু নিশ্চিন্ততাও নেই। বরং কল্যাণ চাইতে বলা হয়েছে এবং ক্ষতি থেকে বাঁচার জন্য আল্লাহর আশ্রয় নিতে শেখানো হয়েছে। ঝড়-তুফানের দোয়া আমাদের মনে করায়, প্রকৃতির বড় ঘটনার সামনে মানুষ দুর্বল। তাই মুমিন আতঙ্ক ছড়ায় না; আল্লাহর কাছে ভালো চায় এবং অনিষ্ট থেকে আশ্রয় নেয়।"},"teachings":["ঝড়-তুফানের সময় আল্লাহর কাছে কল্যাণ চাওয়া উচিত।","প্রাকৃতিক বিপদের অনিষ্ট থেকে আল্লাহর আশ্রয় নিতে শেখানো হয়েছে।","ভয়ের সময় দোয়া মুমিনের মনকে আল্লাহর দিকে ফেরায়।","দোয়ায় কল্যাণ ও নিরাপত্তা—দুটিই চাওয়া যায়।"],"related_hadiths":[{"id":"1032","book_id":"1","label":"Sahih Bukhari"},{"id":"898","book_id":"2","label":"Sahih Muslim"},{"id":"2729","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | অনুপস্থিত ভাইয়ের জন্য দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. অনুপস্থিত মুসলিম ভাইয়ের জন্য দোয়া করলে ফেরেশতা আমীন বলেন এবং দোয়ার মতো কল্যাণ কামনা করেন।"},"heading":{"title":"অনুপস্থিত ভাইয়ের জন্য দোয়া ও ফেরেশতার আমীন","description":"মূল বিষয়: দোয়া। এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম বলেছেন, যে ব্যক্তি তার অনুপস্থিত ভাইয়ের জন্য দোয়া করে, তার সঙ্গে নিযুক্ত ফেরেশতা বলেন, আমীন, তোমার জন্যও অনুরূপ। এখানে দোয়ার একটি সুন্দর দিক শেখানো হয়েছে। কেউ সামনে নেই, সে জানেও না—তবু তার জন্য ভালো চাওয়া মুমিনের আন্তরিকতার পরিচয়। এই দোয়া দেখানোর জন্য নয়; বরং আল্লাহর সন্তুষ্টির আশায়। হাদিসে বলা হয়েছে, এমন দোয়ার সময় ফেরেশতা আমীন বলেন এবং দোয়া করা ব্যক্তির জন্যও অনুরূপ কল্যাণ কামনা করেন। তাই মুসলিম ভাইয়ের জন্য দোয়া করা নিজের মনকে হিংসা ও সংকীর্ণতা থেকে দূরে রাখতে সাহায্য করে। তবে হাদিসের ভাষা অনুযায়ী আমরা বলব, আল্লাহর কাছে ভাইয়ের জন্য ভালো চাইলে ফেরেশতার আমীনের কথা এসেছে।"},"teachings":["অনুপস্থিত মুসলিম ভাইয়ের জন্য দোয়া করা সুন্দর আমল।","দোয়া গোপনে হলেও আল্লাহর কাছে মূল্যবান হতে পারে।","ফেরেশতা আমীন বলেন এবং দোয়া করা ব্যক্তির জন্যও অনুরূপ বলেন।","অন্যের জন্য ভালো চাওয়া মুমিনের হৃদয়কে নরম রাখে।"],"related_hadiths":[{"id":"৯1৮","book_id":"2","label":"Sahih Muslim"},{"id":"33৮0","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"26৯৯","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | অনুপস্থিত ভাইয়ের জন্য দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. অনুপস্থিত মুসলিম ভাইয়ের জন্য দোয়া করলে ফেরেশতা আমীন বলেন এবং দোয়ার মতো কল্যাণ কামনা করেন।"},"heading":{"title":"অনুপস্থিত ভাইয়ের জন্য দোয়া ও ফেরেশতার আমীন","description":"মূল বিষয়: দোয়া। এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম বলেছেন, যে ব্যক্তি তার অনুপস্থিত ভাইয়ের জন্য দোয়া করে, তার সঙ্গে নিযুক্ত ফেরেশতা বলেন, আমীন, তোমার জন্যও অনুরূপ। এখানে দোয়ার একটি সুন্দর দিক শেখানো হয়েছে। কেউ সামনে নেই, সে জানেও না—তবু তার জন্য ভালো চাওয়া মুমিনের আন্তরিকতার পরিচয়। এই দোয়া দেখানোর জন্য নয়; বরং আল্লাহর সন্তুষ্টির আশায়। হাদিসে বলা হয়েছে, এমন দোয়ার সময় ফেরেশতা আমীন বলেন এবং দোয়া করা ব্যক্তির জন্যও অনুরূপ কল্যাণ কামনা করেন। তাই মুসলিম ভাইয়ের জন্য দোয়া করা নিজের মনকে হিংসা ও সংকীর্ণতা থেকে দূরে রাখতে সাহায্য করে। তবে হাদিসের ভাষা অনুযায়ী আমরা বলব, আল্লাহর কাছে ভাইয়ের জন্য ভালো চাইলে ফেরেশতার আমীনের কথা এসেছে।"},"teachings":["অনুপস্থিত মুসলিম ভাইয়ের জন্য দোয়া করা সুন্দর আমল।","দোয়া গোপনে হলেও আল্লাহর কাছে মূল্যবান হতে পারে।","ফেরেশতা আমীন বলেন এবং দোয়া করা ব্যক্তির জন্যও অনুরূপ বলেন।","অন্যের জন্য ভালো চাওয়া মুমিনের হৃদয়কে নরম রাখে।"],"related_hadiths":[{"id":"918","book_id":"2","label":"Sahih Muslim"},{"id":"3380","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"2699","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -2049,7 +2049,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | অনুমতি চাওয়ার সুন্নত আদব","description":"$book_name$ $hadith_number$ - $chapter_name$. ঘরে বা স্থানে প্রবেশের আগে তিনবার অনুমতি চাওয়া, অনুমতি না পেলে ফিরে যাওয়ার আদব শেখানো হয়েছে।"},"heading":{"title":"তিনবার অনুমতি চাওয়ার আদব ও ইসলামী শিষ্টাচার","description":"মূল বিষয়: অনুমতির আদব। এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম খুব পরিষ্কারভাবে প্রবেশের আগে অনুমতি চাওয়ার নিয়ম বলেছেন। তিনি বলেন, তিনবার অনুমতি চাইবে। অনুমতি দিলে প্রবেশ করবে, অন্যথায় ফিরে যাবে। এতে অন্যের ব্যক্তিগত সময়, ঘর ও অবস্থার প্রতি সম্মান শেখানো হয়েছে। কেউ দরজা খুলল না বা সাড়া দিল না মানেই বিরক্ত করা যাবে—এমন নয়। বরং তিনবারের পর ফিরে যাওয়া আদব। এই হাদিসে অনুমতি নেওয়ার নিয়মকে সহজ করে দেওয়া হয়েছে: জোর করা নয়, চাপ দেওয়া নয়, অনুমতি পেলে ঢোকা, না পেলে ফিরে যাওয়া। মুসলিমের আচরণে ভদ্রতা, ধৈর্য ও অন্যের অধিকার রক্ষা থাকা উচিত। তাই অনুমতি চাওয়ার হাদিস পরিবার, প্রতিবেশী, বন্ধু—সব ক্ষেত্রেই ব্যবহারযোগ্য একটি সুন্দর শিক্ষা।"},"teachings":["প্রবেশের আগে অনুমতি চাওয়া উচিত।","তিনবার অনুমতি চাওয়ার পর অনুমতি না পেলে ফিরে যেতে বলা হয়েছে।","অন্যের ব্যক্তিগত সময় ও জায়গার প্রতি সম্মান রাখা দরকার।","ইসলামী আদব জোরাজুরির বদলে ভদ্রতা শেখায়।"],"related_hadiths":[{"id":"201৮","book_id":"2","label":"Sahih Muslim"},{"id":"6224","book_id":"1","label":"Sahih Bukhari"},{"id":"2066","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | অনুমতি চাওয়ার সুন্নত আদব","description":"$book_name$ $hadith_number$ - $chapter_name$. ঘরে বা স্থানে প্রবেশের আগে তিনবার অনুমতি চাওয়া, অনুমতি না পেলে ফিরে যাওয়ার আদব শেখানো হয়েছে।"},"heading":{"title":"তিনবার অনুমতি চাওয়ার আদব ও ইসলামী শিষ্টাচার","description":"মূল বিষয়: অনুমতির আদব। এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম খুব পরিষ্কারভাবে প্রবেশের আগে অনুমতি চাওয়ার নিয়ম বলেছেন। তিনি বলেন, তিনবার অনুমতি চাইবে। অনুমতি দিলে প্রবেশ করবে, অন্যথায় ফিরে যাবে। এতে অন্যের ব্যক্তিগত সময়, ঘর ও অবস্থার প্রতি সম্মান শেখানো হয়েছে। কেউ দরজা খুলল না বা সাড়া দিল না মানেই বিরক্ত করা যাবে—এমন নয়। বরং তিনবারের পর ফিরে যাওয়া আদব। এই হাদিসে অনুমতি নেওয়ার নিয়মকে সহজ করে দেওয়া হয়েছে: জোর করা নয়, চাপ দেওয়া নয়, অনুমতি পেলে ঢোকা, না পেলে ফিরে যাওয়া। মুসলিমের আচরণে ভদ্রতা, ধৈর্য ও অন্যের অধিকার রক্ষা থাকা উচিত। তাই অনুমতি চাওয়ার হাদিস পরিবার, প্রতিবেশী, বন্ধু—সব ক্ষেত্রেই ব্যবহারযোগ্য একটি সুন্দর শিক্ষা।"},"teachings":["প্রবেশের আগে অনুমতি চাওয়া উচিত।","তিনবার অনুমতি চাওয়ার পর অনুমতি না পেলে ফিরে যেতে বলা হয়েছে।","অন্যের ব্যক্তিগত সময় ও জায়গার প্রতি সম্মান রাখা দরকার।","ইসলামী আদব জোরাজুরির বদলে ভদ্রতা শেখায়।"],"related_hadiths":[{"id":"2018","book_id":"2","label":"Sahih Muslim"},{"id":"6224","book_id":"1","label":"Sahih Bukhari"},{"id":"2066","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2071,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নবজাতকের নাম ও বরকতের দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. নবজাতকের নাম রাখা, খেজুর চিবিয়ে মুখে দেওয়া এবং বরকতের দোয়া করার শিক্ষা এ হাদিসে এসেছে।"},"heading":{"title":"নবজাতকের নাম রাখা ও বরকতের দোয়ার সুন্নতি শিক্ষা","description":"মূল বিষয়: নবজাতক। এই হাদিসে একজন সাহাবী তাঁর নবজাতক পুত্রকে নবী করীম সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লামের কাছে নিয়ে গেলেন। নবী সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম শিশুটির নাম রাখলেন ইবরাহীম। এরপর খেজুর চিবিয়ে তার মুখে দিলেন এবং তার জন্য বরকতের দোয়া করলেন। এই বর্ণনা থেকে নবজাতকের জন্য ভালো নাম রাখা, তার জন্য বরকতের দোয়া করা এবং শিশুকে ভালোবাসার সঙ্গে গ্রহণ করার শিক্ষা পাওয়া যায়। এখানে যে কাজগুলো উল্লেখ আছে, ব্যাখ্যাও সেগুলোর মধ্যেই সীমিত। শিশুর জন্ম পরিবারে আনন্দের বিষয়। সেই আনন্দকে আল্লাহর বরকতের দোয়ার সঙ্গে যুক্ত করা মুমিনের সুন্দর আদব। নবজাতকের জন্য দোয়া করা মানে তার জীবনের শুরুতেই আল্লাহর কল্যাণ কামনা করা।"},"teachings":["নবজাতকের জন্য সুন্দর নাম রাখা গুরুত্বপূর্ণ।","শিশুর জন্য বরকতের দোয়া করা সুন্নতি আদব।","নবজাতককে স্নেহ ও দোয়ার সঙ্গে গ্রহণ করার শিক্ষা আছে।","পরিবারের আনন্দকে আল্লাহর বরকতের সঙ্গে যুক্ত করা উচিত।"],"related_hadiths":[{"id":"256৮","book_id":"2","label":"Sahih Muslim"},{"id":"2732","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নবজাতকের নাম ও বরকতের দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. নবজাতকের নাম রাখা, খেজুর চিবিয়ে মুখে দেওয়া এবং বরকতের দোয়া করার শিক্ষা এ হাদিসে এসেছে।"},"heading":{"title":"নবজাতকের নাম রাখা ও বরকতের দোয়ার সুন্নতি শিক্ষা","description":"মূল বিষয়: নবজাতক। এই হাদিসে একজন সাহাবী তাঁর নবজাতক পুত্রকে নবী করীম সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লামের কাছে নিয়ে গেলেন। নবী সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম শিশুটির নাম রাখলেন ইবরাহীম। এরপর খেজুর চিবিয়ে তার মুখে দিলেন এবং তার জন্য বরকতের দোয়া করলেন। এই বর্ণনা থেকে নবজাতকের জন্য ভালো নাম রাখা, তার জন্য বরকতের দোয়া করা এবং শিশুকে ভালোবাসার সঙ্গে গ্রহণ করার শিক্ষা পাওয়া যায়। এখানে যে কাজগুলো উল্লেখ আছে, ব্যাখ্যাও সেগুলোর মধ্যেই সীমিত। শিশুর জন্ম পরিবারে আনন্দের বিষয়। সেই আনন্দকে আল্লাহর বরকতের দোয়ার সঙ্গে যুক্ত করা মুমিনের সুন্দর আদব। নবজাতকের জন্য দোয়া করা মানে তার জীবনের শুরুতেই আল্লাহর কল্যাণ কামনা করা।"},"teachings":["নবজাতকের জন্য সুন্দর নাম রাখা গুরুত্বপূর্ণ।","শিশুর জন্য বরকতের দোয়া করা সুন্নতি আদব।","নবজাতককে স্নেহ ও দোয়ার সঙ্গে গ্রহণ করার শিক্ষা আছে।","পরিবারের আনন্দকে আল্লাহর বরকতের সঙ্গে যুক্ত করা উচিত।"],"related_hadiths":[{"id":"2568","book_id":"2","label":"Sahih Muslim"},{"id":"2732","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | বৃষ্টির পানি ও আল্লাহর দান","description":"$book_name$ $hadith_number$ - $chapter_name$. নবীজি বৃষ্টির পানি শরীরে লাগতে দিলেন, কারণ তা সদ্য আল্লাহর পক্ষ থেকে এসেছে—এ হাদিসে তা বলা হয়েছে।"},"heading":{"title":"বৃষ্টির পানি শরীরে লাগানো ও আল্লাহর দানের স্মরণ","description":"মূল বিষয়: বৃষ্টি। এই হাদিসে বলা হয়েছে, রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লামের সঙ্গে থাকা অবস্থায় বৃষ্টি শুরু হলে তিনি শরীরের কিছু অংশ খুলে দিলেন, যাতে সেখানে বৃষ্টির পানি লাগে। সাহাবীরা কারণ জিজ্ঞেস করলে তিনি বললেন, কারণ এটি তার প্রতিপালকের কাছ থেকে সদ্য আগত। এই বর্ণনায় বৃষ্টির পানি সম্পর্কে নবী সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লামের এক সুন্দর অনুভূতি দেখা যায়। তিনি বৃষ্টিকে আল্লাহর দান হিসেবে দেখেছেন এবং সেটির নতুন আগমনকে স্মরণ করেছেন। এখানে কোনো অতিরিক্ত নিয়ম বানানোর কথা নেই; বরং হাদিসে যে কাজ ও কারণ বলা হয়েছে, সেটিই মূল শিক্ষা। বৃষ্টি হলে শুধু বিরক্ত হওয়া নয়, বরং আল্লাহর দান মনে করা—এটিই এই হাদিসের কোমল বার্তা।"},"teachings":["বৃষ্টি আল্লাহর পক্ষ থেকে আসা দান হিসেবে স্মরণ করা উচিত।","রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম বৃষ্টির পানি শরীরে লাগতে দিয়েছেন।","প্রকৃতির নেয়ামত দেখলে আল্লাহর কথা মনে করা মুমিনের আদব।","হাদিসে কাজের সঙ্গে তার কারণও শেখানো হয়েছে।"],"related_hadiths":[{"id":"1032","book_id":"1","label":"Sahih Bukhari"},{"id":"৮৯৯","book_id":"2","label":"Sahih Muslim"},{"id":"272৯","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | বৃষ্টির পানি ও আল্লাহর দান","description":"$book_name$ $hadith_number$ - $chapter_name$. নবীজি বৃষ্টির পানি শরীরে লাগতে দিলেন, কারণ তা সদ্য আল্লাহর পক্ষ থেকে এসেছে—এ হাদিসে তা বলা হয়েছে।"},"heading":{"title":"বৃষ্টির পানি শরীরে লাগানো ও আল্লাহর দানের স্মরণ","description":"মূল বিষয়: বৃষ্টি। এই হাদিসে বলা হয়েছে, রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লামের সঙ্গে থাকা অবস্থায় বৃষ্টি শুরু হলে তিনি শরীরের কিছু অংশ খুলে দিলেন, যাতে সেখানে বৃষ্টির পানি লাগে। সাহাবীরা কারণ জিজ্ঞেস করলে তিনি বললেন, কারণ এটি তার প্রতিপালকের কাছ থেকে সদ্য আগত। এই বর্ণনায় বৃষ্টির পানি সম্পর্কে নবী সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লামের এক সুন্দর অনুভূতি দেখা যায়। তিনি বৃষ্টিকে আল্লাহর দান হিসেবে দেখেছেন এবং সেটির নতুন আগমনকে স্মরণ করেছেন। এখানে কোনো অতিরিক্ত নিয়ম বানানোর কথা নেই; বরং হাদিসে যে কাজ ও কারণ বলা হয়েছে, সেটিই মূল শিক্ষা। বৃষ্টি হলে শুধু বিরক্ত হওয়া নয়, বরং আল্লাহর দান মনে করা—এটিই এই হাদিসের কোমল বার্তা।"},"teachings":["বৃষ্টি আল্লাহর পক্ষ থেকে আসা দান হিসেবে স্মরণ করা উচিত।","রাসূলুল্লাহ সাল্লাল্লাহু ‘আলাইহি ওয়া সাল্লাম বৃষ্টির পানি শরীরে লাগতে দিয়েছেন।","প্রকৃতির নেয়ামত দেখলে আল্লাহর কথা মনে করা মুমিনের আদব।","হাদিসে কাজের সঙ্গে তার কারণও শেখানো হয়েছে।"],"related_hadiths":[{"id":"1032","book_id":"1","label":"Sahih Bukhari"},{"id":"899","book_id":"2","label":"Sahih Muslim"},{"id":"2729","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2164,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ওজুর পর শাহাদাত পড়ার ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. সুন্দরভাবে ওজুর পর শাহাদাত পড়লে জান্নাতের আট দরজা খুলে দেওয়ার সুসংবাদ।"},"heading":{"title":"ওজুর পর দোয়া: শাহাদাত পড়ার মহান ফজিলত","description":"এই হাদিসে ওজুর পর শাহাদাত পড়ার ফজিলত এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, তোমাদের মধ্যে যে কেউ সুন্দর করে ওজু করে বলে, “আশহাদু আনলা ইলাহা ইল্লাল্লাহু ওয়া আন্না মুহাম্মাদান আবদুহু ওয়া রাসূলুহ”, তার জন্য জান্নাতের আটটি দরজা খুলে দেওয়া হবে। সে যেটি দিয়ে ইচ্ছা প্রবেশ করবে। এখানে প্রথমে সুন্দরভাবে ওজু করার কথা বলা হয়েছে, তারপর তাওহীদ ও রাসূলের রিসালাতের সাক্ষ্য দেওয়ার কথা এসেছে। তাই ওজুর পর দোয়া শুধু মুখের কথা নয়; এটি ঈমানের ঘোষণা। ওজুর ফজিলত, ওজুর পর কালিমা এবং জান্নাতের দরজা সম্পর্কিত হাদিস খোঁজেন যারা, তাদের জন্য এই বর্ণনা খুব গুরুত্বপূর্ণ।"},"teachings":["সুন্দরভাবে ওজু করা হাদিসে বিশেষভাবে বলা হয়েছে।","ওজুর পর শাহাদাত পড়া নবী صلى الله عليه وسلم-এর শেখানো আমল।","তাওহীদ ও রিসালাতের সাক্ষ্য ওজুর পরের দোয়ার মূল কথা।","হাদিসে জান্নাতের আট দরজার সুসংবাদ এসেছে।"],"related_hadiths":[{"id":"15৯","book_id":"1","label":"Sahih Bukhari"},{"id":"251","book_id":"2","label":"Sahih Muslim"},{"id":"201","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ওজুর পর শাহাদাত পড়ার ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. সুন্দরভাবে ওজুর পর শাহাদাত পড়লে জান্নাতের আট দরজা খুলে দেওয়ার সুসংবাদ।"},"heading":{"title":"ওজুর পর দোয়া: শাহাদাত পড়ার মহান ফজিলত","description":"এই হাদিসে ওজুর পর শাহাদাত পড়ার ফজিলত এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম বলেছেন, তোমাদের মধ্যে যে কেউ সুন্দর করে ওজু করে বলে, “আশহাদু আনলা ইলাহা ইল্লাল্লাহু ওয়া আন্না মুহাম্মাদান আবদুহু ওয়া রাসূলুহ”, তার জন্য জান্নাতের আটটি দরজা খুলে দেওয়া হবে। সে যেটি দিয়ে ইচ্ছা প্রবেশ করবে। এখানে প্রথমে সুন্দরভাবে ওজু করার কথা বলা হয়েছে, তারপর তাওহীদ ও রাসূলের রিসালাতের সাক্ষ্য দেওয়ার কথা এসেছে। তাই ওজুর পর দোয়া শুধু মুখের কথা নয়; এটি ঈমানের ঘোষণা। ওজুর ফজিলত, ওজুর পর কালিমা এবং জান্নাতের দরজা সম্পর্কিত হাদিস খোঁজেন যারা, তাদের জন্য এই বর্ণনা খুব গুরুত্বপূর্ণ।"},"teachings":["সুন্দরভাবে ওজু করা হাদিসে বিশেষভাবে বলা হয়েছে।","ওজুর পর শাহাদাত পড়া নবী صلى الله عليه وسلم-এর শেখানো আমল।","তাওহীদ ও রিসালাতের সাক্ষ্য ওজুর পরের দোয়ার মূল কথা।","হাদিসে জান্নাতের আট দরজার সুসংবাদ এসেছে।"],"related_hadiths":[{"id":"159","book_id":"1","label":"Sahih Bukhari"},{"id":"251","book_id":"2","label":"Sahih Muslim"},{"id":"201","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -2252,7 +2252,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | হাই তোলা ও শয়তানের হাসি","description":"$book_name$ $hadith_number$ - $chapter_name$. হাই শয়তানের পক্ষ থেকে আসে; তাই হাই এলে সাধ্যানুসারে তা রোধ করার শিক্ষা এই হাদিসে এসেছে।"},"heading":{"title":"হাই তোলা থেকে বিরত থাকা: নববী আদবের সহজ শিক্ষা","description":"এই হাদিসে হাই তোলার আদব শেখানো হয়েছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, হাই শয়তানের পক্ষ থেকে আসে। তাই কারও হাই এলে সে যেন সাধ্যানুসারে তা রোধ করে। হাদিসে আরও বলা হয়েছে, কেউ হাই তুললে শয়তান হাসে। এখানে মূল শিক্ষা হলো, মানুষের সাধারণ আচরণেও ইসলামের সুন্দর শিষ্টাচার আছে। হাই আসা স্বাভাবিক ব্যাপার হতে পারে, কিন্তু একজন মুসলিম সেটিকে নিয়ন্ত্রণের চেষ্টা করবে। বিশেষ করে নামাজ, মজলিস বা মানুষের সামনে আদব বজায় রাখা জরুরি। হাই তোলা হাদিস, হাই রোধ করা এবং ইসলামী আদব—এই বিষয়গুলো এই বর্ণনার কেন্দ্রীয় শিক্ষা। এতে নিজেকে সামলে রাখা এবং শয়তানের পছন্দনীয় ভঙ্গি থেকে দূরে থাকার কথা বোঝা যায়।"},"teachings":["হাই এলে সাধ্যানুসারে তা রোধ করার চেষ্টা করা উচিত।","সাধারণ আচরণেও ইসলামী আদব মানার শিক্ষা আছে।","হাই তোলাকে অবহেলা না করে নিজেকে সামলে রাখা ভালো।","শয়তানের হাসির কারণ হয় এমন ভঙ্গি থেকে দূরে থাকা দরকার।"],"related_hadiths":[{"id":"6226","book_id":"1","label":"Sahih Bukhari"},{"id":"2৯৯4","book_id":"2","label":"Sahih Muslim"},{"id":"502৮","book_id":"4","label":"Sunan Abu Dawud"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | হাই তোলা ও শয়তানের হাসি","description":"$book_name$ $hadith_number$ - $chapter_name$. হাই শয়তানের পক্ষ থেকে আসে; তাই হাই এলে সাধ্যানুসারে তা রোধ করার শিক্ষা এই হাদিসে এসেছে।"},"heading":{"title":"হাই তোলা থেকে বিরত থাকা: নববী আদবের সহজ শিক্ষা","description":"এই হাদিসে হাই তোলার আদব শেখানো হয়েছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, হাই শয়তানের পক্ষ থেকে আসে। তাই কারও হাই এলে সে যেন সাধ্যানুসারে তা রোধ করে। হাদিসে আরও বলা হয়েছে, কেউ হাই তুললে শয়তান হাসে। এখানে মূল শিক্ষা হলো, মানুষের সাধারণ আচরণেও ইসলামের সুন্দর শিষ্টাচার আছে। হাই আসা স্বাভাবিক ব্যাপার হতে পারে, কিন্তু একজন মুসলিম সেটিকে নিয়ন্ত্রণের চেষ্টা করবে। বিশেষ করে নামাজ, মজলিস বা মানুষের সামনে আদব বজায় রাখা জরুরি। হাই তোলা হাদিস, হাই রোধ করা এবং ইসলামী আদব—এই বিষয়গুলো এই বর্ণনার কেন্দ্রীয় শিক্ষা। এতে নিজেকে সামলে রাখা এবং শয়তানের পছন্দনীয় ভঙ্গি থেকে দূরে থাকার কথা বোঝা যায়।"},"teachings":["হাই এলে সাধ্যানুসারে তা রোধ করার চেষ্টা করা উচিত।","সাধারণ আচরণেও ইসলামী আদব মানার শিক্ষা আছে।","হাই তোলাকে অবহেলা না করে নিজেকে সামলে রাখা ভালো।","শয়তানের হাসির কারণ হয় এমন ভঙ্গি থেকে দূরে থাকা দরকার।"],"related_hadiths":[{"id":"6226","book_id":"1","label":"Sahih Bukhari"},{"id":"2994","book_id":"2","label":"Sahih Muslim"},{"id":"5028","book_id":"4","label":"Sunan Abu Dawud"}]}</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পরিবারের কাজে রাসূলের সহযোগিতা","description":"$book_name$ $hadith_number$ - $chapter_name$. রাসূলুল্লাহ ঘরে পরিবারের কাজে সাহায্য করতেন এবং নামাজের সময় হলে নামাজে বেরিয়ে যেতেন।"},"heading":{"title":"পরিবারের কাজে সহযোগিতা: রাসূলের ঘরোয়া জীবনের শিক্ষা","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামের ঘরের জীবন সম্পর্কে একটি সরল কিন্তু গভীর শিক্ষা এসেছে। আয়েশা রাদিয়াল্লাহু আনহাকে জিজ্ঞেস করা হলে তিনি জানান, নবীজি ঘরে পরিবারের কাজে সহযোগিতা করতেন। আর নামাজের সময় হলে নামাজের জন্য বেরিয়ে যেতেন। এই হাদিস আমাদের শেখায়, ঘরের কাজকে ছোট ভাবা ঠিক নয়। পরিবারের কাজে সাহায্য করা ভালো চরিত্রের অংশ। একই সঙ্গে নামাজের সময় হলে ইবাদতকে অগ্রাধিকার দেওয়াও জরুরি। পরিবারের কাজে সহযোগিতা হাদিস, রাসূলের পারিবারিক জীবন এবং নামাজের গুরুত্ব—এই তিনটি বিষয় এখানে একসঙ্গে এসেছে। একজন মুসলিম ঘরে কোমল, সাহায্যকারী এবং দায়িত্বশীল হবে; আবার ইবাদতের সময় হলে আল্লাহর ডাকে সাড়া দেবে।"},"teachings":["পরিবারের কাজে সহযোগিতা করা নবীজির সুন্দর আদর্শ।","ঘরের কাজকে অবহেলা না করে দায়িত্ব হিসেবে দেখা উচিত।","নামাজের সময় হলে নামাজকে অগ্রাধিকার দিতে হবে।","ভালো চরিত্র ঘরের মানুষের সঙ্গেও প্রকাশ পায়।"],"related_hadiths":[{"id":"3৮৯5","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"5363","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পরিবারের কাজে রাসূলের সহযোগিতা","description":"$book_name$ $hadith_number$ - $chapter_name$. রাসূলুল্লাহ ঘরে পরিবারের কাজে সাহায্য করতেন এবং নামাজের সময় হলে নামাজে বেরিয়ে যেতেন।"},"heading":{"title":"পরিবারের কাজে সহযোগিতা: রাসূলের ঘরোয়া জীবনের শিক্ষা","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামের ঘরের জীবন সম্পর্কে একটি সরল কিন্তু গভীর শিক্ষা এসেছে। আয়েশা রাদিয়াল্লাহু আনহাকে জিজ্ঞেস করা হলে তিনি জানান, নবীজি ঘরে পরিবারের কাজে সহযোগিতা করতেন। আর নামাজের সময় হলে নামাজের জন্য বেরিয়ে যেতেন। এই হাদিস আমাদের শেখায়, ঘরের কাজকে ছোট ভাবা ঠিক নয়। পরিবারের কাজে সাহায্য করা ভালো চরিত্রের অংশ। একই সঙ্গে নামাজের সময় হলে ইবাদতকে অগ্রাধিকার দেওয়াও জরুরি। পরিবারের কাজে সহযোগিতা হাদিস, রাসূলের পারিবারিক জীবন এবং নামাজের গুরুত্ব—এই তিনটি বিষয় এখানে একসঙ্গে এসেছে। একজন মুসলিম ঘরে কোমল, সাহায্যকারী এবং দায়িত্বশীল হবে; আবার ইবাদতের সময় হলে আল্লাহর ডাকে সাড়া দেবে।"},"teachings":["পরিবারের কাজে সহযোগিতা করা নবীজির সুন্দর আদর্শ।","ঘরের কাজকে অবহেলা না করে দায়িত্ব হিসেবে দেখা উচিত।","নামাজের সময় হলে নামাজকে অগ্রাধিকার দিতে হবে।","ভালো চরিত্র ঘরের মানুষের সঙ্গেও প্রকাশ পায়।"],"related_hadiths":[{"id":"3895","book_id":"5","label":"Jami at-Tirmidhi"},{"id":"5363","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -2318,7 +2318,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | স্বভাবগত পরিচ্ছন্নতার পাঁচ আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. খাতনা, লোম পরিষ্কার, নখ কাটা ও মোচ খাটো করা—স্বভাবগত পরিচ্ছন্নতার পাঁচটি কাজের শিক্ষা।"},"heading":{"title":"স্বভাবগত পরিচ্ছন্নতা: পাঁচটি সহজ আমলের হাদিস","description":"এই হাদিসে স্বভাবগত অভ্যাস বা ফিতরতের পাঁচটি কাজের কথা বলা হয়েছে। এগুলো হলো খাতনা করা, নাভীর নিচের লোম পরিষ্কার করা, বগলের চুল ছিঁড়ে ফেলা, নখ কাটা এবং মোচ খাটো করা। এই কাজগুলো শরীরের পরিচ্ছন্নতা ও সুন্দর অভ্যাসের সঙ্গে জড়িত। ইসলাম শুধু বড় বড় ইবাদতের কথা বলে না; মানুষের দৈনন্দিন পরিচ্ছন্নতার বিষয়ও শেখায়। স্বভাবগত পরিচ্ছন্নতা হাদিস, নখ কাটা, মোচ খাটো করা এবং শরীর পরিষ্কার রাখা—এসব বিষয় এই হাদিসের মূল আলোচ্য। এখানে অতিরিক্ত কোনো দাবি করা দরকার নেই; বর্ণনাটিই পরিষ্কারভাবে জানিয়ে দেয় যে পরিচ্ছন্নতা একজন মুসলিমের জীবনের অংশ। নিজের শরীর ও অভ্যাসকে গোছানো রাখাও ইসলামী আদবের মধ্যে পড়ে।"},"teachings":["শরীরের পরিচ্ছন্নতা ইসলামের গুরুত্বপূর্ণ শিক্ষা।","নখ কাটা, লোম পরিষ্কার ও মোচ খাটো করা স্বভাবগত অভ্যাসের অংশ।","দৈনন্দিন পরিচ্ছন্নতাকেও মুসলিম জীবনে গুরুত্ব দেওয়া হয়েছে।","নিজের শরীরের পরিচর্যা সুন্দর চরিত্রের প্রকাশ হতে পারে।"],"related_hadiths":[{"id":"5৮৯1","book_id":"1","label":"Sahih Bukhari"},{"id":"25৮","book_id":"2","label":"Sahih Muslim"},{"id":"2756","book_id":"5","label":"Jami at-Tirmidhi"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | স্বভাবগত পরিচ্ছন্নতার পাঁচ আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. খাতনা, লোম পরিষ্কার, নখ কাটা ও মোচ খাটো করা—স্বভাবগত পরিচ্ছন্নতার পাঁচটি কাজের শিক্ষা।"},"heading":{"title":"স্বভাবগত পরিচ্ছন্নতা: পাঁচটি সহজ আমলের হাদিস","description":"এই হাদিসে স্বভাবগত অভ্যাস বা ফিতরতের পাঁচটি কাজের কথা বলা হয়েছে। এগুলো হলো খাতনা করা, নাভীর নিচের লোম পরিষ্কার করা, বগলের চুল ছিঁড়ে ফেলা, নখ কাটা এবং মোচ খাটো করা। এই কাজগুলো শরীরের পরিচ্ছন্নতা ও সুন্দর অভ্যাসের সঙ্গে জড়িত। ইসলাম শুধু বড় বড় ইবাদতের কথা বলে না; মানুষের দৈনন্দিন পরিচ্ছন্নতার বিষয়ও শেখায়। স্বভাবগত পরিচ্ছন্নতা হাদিস, নখ কাটা, মোচ খাটো করা এবং শরীর পরিষ্কার রাখা—এসব বিষয় এই হাদিসের মূল আলোচ্য। এখানে অতিরিক্ত কোনো দাবি করা দরকার নেই; বর্ণনাটিই পরিষ্কারভাবে জানিয়ে দেয় যে পরিচ্ছন্নতা একজন মুসলিমের জীবনের অংশ। নিজের শরীর ও অভ্যাসকে গোছানো রাখাও ইসলামী আদবের মধ্যে পড়ে।"},"teachings":["শরীরের পরিচ্ছন্নতা ইসলামের গুরুত্বপূর্ণ শিক্ষা।","নখ কাটা, লোম পরিষ্কার ও মোচ খাটো করা স্বভাবগত অভ্যাসের অংশ।","দৈনন্দিন পরিচ্ছন্নতাকেও মুসলিম জীবনে গুরুত্ব দেওয়া হয়েছে।","নিজের শরীরের পরিচর্যা সুন্দর চরিত্রের প্রকাশ হতে পারে।"],"related_hadiths":[{"id":"5891","book_id":"1","label":"Sahih Bukhari"},{"id":"258","book_id":"2","label":"Sahih Muslim"},{"id":"2756","book_id":"5","label":"Jami at-Tirmidhi"}]}</t>
         </is>
       </c>
     </row>
@@ -2362,7 +2362,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রাগ না করার সংক্ষিপ্ত উপদেশ","description":"$book_name$ $hadith_number$ - $chapter_name$. এক ব্যক্তি উপদেশ চাইলে রাসূলুল্লাহ বারবার বললেন, রাগ করো না—এতে রাগ নিয়ন্ত্রণের শিক্ষা আছে।"},"heading":{"title":"রাগ করো না: চরিত্র গঠনের সংক্ষিপ্ত কিন্তু শক্তিশালী হাদিস","description":"এই হাদিসে একজন ব্যক্তি রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামের কাছে উপদেশ চান। নবীজি তাকে বলেন, রাগ করো না। লোকটি কয়েকবার একইভাবে উপদেশ চাইলে তিনি আবারও একই কথা বলেন। এর মাধ্যমে বোঝা যায়, রাগ নিয়ন্ত্রণ করা মানুষের চরিত্রের জন্য খুব গুরুত্বপূর্ণ। রাগের সময় মানুষ ভুল কথা বলে, অন্যায় আচরণ করে এবং পরে অনুতপ্ত হয়। তাই নবীজির এই ছোট উপদেশ জীবনের অনেক ক্ষেত্রে কাজে লাগে। রাগ না করার হাদিস, রাগ নিয়ন্ত্রণ এবং ভালো চরিত্র—এই হাদিসের প্রধান বিষয়। এখানে শিক্ষা হলো, রাগ পুরোপুরি আসবে না এমন দাবি নয়; বরং রাগের সময় নিজেকে সামলানো দরকার। সংক্ষিপ্ত উপদেশ হলেও এতে পরিবার, সমাজ ও ব্যক্তিগত জীবনের বড় কল্যাণ আছে।"},"teachings":["রাগ নিয়ন্ত্রণ করা ভালো চরিত্রের গুরুত্বপূর্ণ অংশ।","কম কথা হলেও গভীর উপদেশ জীবনে বড় প্রভাব ফেলতে পারে।","রাগের সময় নিজেকে সামলানোর চেষ্টা করা দরকার।","একই উপদেশ বারবার বলার মাধ্যমে তার গুরুত্ব বোঝানো হয়েছে।"],"related_hadiths":[{"id":"6114","book_id":"1","label":"Sahih Bukhari"},{"id":"260৯","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রাগ না করার সংক্ষিপ্ত উপদেশ","description":"$book_name$ $hadith_number$ - $chapter_name$. এক ব্যক্তি উপদেশ চাইলে রাসূলুল্লাহ বারবার বললেন, রাগ করো না—এতে রাগ নিয়ন্ত্রণের শিক্ষা আছে।"},"heading":{"title":"রাগ করো না: চরিত্র গঠনের সংক্ষিপ্ত কিন্তু শক্তিশালী হাদিস","description":"এই হাদিসে একজন ব্যক্তি রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামের কাছে উপদেশ চান। নবীজি তাকে বলেন, রাগ করো না। লোকটি কয়েকবার একইভাবে উপদেশ চাইলে তিনি আবারও একই কথা বলেন। এর মাধ্যমে বোঝা যায়, রাগ নিয়ন্ত্রণ করা মানুষের চরিত্রের জন্য খুব গুরুত্বপূর্ণ। রাগের সময় মানুষ ভুল কথা বলে, অন্যায় আচরণ করে এবং পরে অনুতপ্ত হয়। তাই নবীজির এই ছোট উপদেশ জীবনের অনেক ক্ষেত্রে কাজে লাগে। রাগ না করার হাদিস, রাগ নিয়ন্ত্রণ এবং ভালো চরিত্র—এই হাদিসের প্রধান বিষয়। এখানে শিক্ষা হলো, রাগ পুরোপুরি আসবে না এমন দাবি নয়; বরং রাগের সময় নিজেকে সামলানো দরকার। সংক্ষিপ্ত উপদেশ হলেও এতে পরিবার, সমাজ ও ব্যক্তিগত জীবনের বড় কল্যাণ আছে।"},"teachings":["রাগ নিয়ন্ত্রণ করা ভালো চরিত্রের গুরুত্বপূর্ণ অংশ।","কম কথা হলেও গভীর উপদেশ জীবনে বড় প্রভাব ফেলতে পারে।","রাগের সময় নিজেকে সামলানোর চেষ্টা করা দরকার।","একই উপদেশ বারবার বলার মাধ্যমে তার গুরুত্ব বোঝানো হয়েছে।"],"related_hadiths":[{"id":"6114","book_id":"1","label":"Sahih Bukhari"},{"id":"2609","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>
@@ -2406,7 +2406,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ওজু ও গোসলে পানির পরিমিত ব্যবহার","description":"$book_name$ $hadith_number$ - $chapter_name$. নবী صلى الله عليه وسلم গোসল ও ওজুতে নির্দিষ্ট পরিমাণ পানি ব্যবহার করতেন; এতে পরিমিতির শিক্ষা আছে।"},"heading":{"title":"ওজু ও গোসলে পানি: নবী صلى الله عليه وسلم-এর পরিমিত ব্যবহারের শিক্ষা","description":"এই হাদিসে নবী করীম সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর ওজু ও গোসলে পানির পরিমাণ বর্ণিত হয়েছে। তিনি এক সা’ থেকে পাঁচ মুদ পর্যন্ত পানি দিয়ে গোসল করতেন এবং এক মুদ পানি দিয়ে ওজু করতেন। হাদিসে কমবেশি পরিমাণও উল্লেখ আছে, যাতে বোঝা যায় তিনি পানির ব্যবহারে পরিমিত ছিলেন। এখানে মূল শিক্ষা হলো, পবিত্রতা অর্জন করতে গিয়ে অযথা পানি বেশি ব্যবহার করা দরকার নয়। ওজু ও গোসলের উদ্দেশ্য হলো শরিয়তসম্মতভাবে পবিত্র হওয়া, অপচয় করা নয়। নবীজির ওজু পদ্ধতি, গোসলের পানি এবং পানির অপচয় থেকে বাঁচার শিক্ষা এই হাদিসে সহজভাবে দেখা যায়। এটি দৈনন্দিন জীবনে খুব প্রয়োগযোগ্য একটি হাদিস।"},"teachings":["নবী صلى الله عليه وسلم ওজুতে এক মুদ পরিমাণ পানি ব্যবহার করতেন।","গোসলের জন্য এক সা’ থেকে পাঁচ মুদ পর্যন্ত পানি ব্যবহারের বর্ণনা আছে।","পবিত্রতার কাজে পানির পরিমিত ব্যবহার শেখা যায়।","ওজু ও গোসল সহজ এবং অপচয়মুক্ত হওয়া উচিত।"],"related_hadiths":[{"id":"234","book_id":"1","label":"Sahih Bukhari"},{"id":"555","book_id":"2","label":"Sahih Muslim"},{"id":"15৯","book_id":"1","label":"Sahih Bukhari"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ওজু ও গোসলে পানির পরিমিত ব্যবহার","description":"$book_name$ $hadith_number$ - $chapter_name$. নবী صلى الله عليه وسلم গোসল ও ওজুতে নির্দিষ্ট পরিমাণ পানি ব্যবহার করতেন; এতে পরিমিতির শিক্ষা আছে।"},"heading":{"title":"ওজু ও গোসলে পানি: নবী صلى الله عليه وسلم-এর পরিমিত ব্যবহারের শিক্ষা","description":"এই হাদিসে নবী করীম সাল্লাল্লাহু আলাইহি ওয়া সাল্লাম-এর ওজু ও গোসলে পানির পরিমাণ বর্ণিত হয়েছে। তিনি এক সা’ থেকে পাঁচ মুদ পর্যন্ত পানি দিয়ে গোসল করতেন এবং এক মুদ পানি দিয়ে ওজু করতেন। হাদিসে কমবেশি পরিমাণও উল্লেখ আছে, যাতে বোঝা যায় তিনি পানির ব্যবহারে পরিমিত ছিলেন। এখানে মূল শিক্ষা হলো, পবিত্রতা অর্জন করতে গিয়ে অযথা পানি বেশি ব্যবহার করা দরকার নয়। ওজু ও গোসলের উদ্দেশ্য হলো শরিয়তসম্মতভাবে পবিত্র হওয়া, অপচয় করা নয়। নবীজির ওজু পদ্ধতি, গোসলের পানি এবং পানির অপচয় থেকে বাঁচার শিক্ষা এই হাদিসে সহজভাবে দেখা যায়। এটি দৈনন্দিন জীবনে খুব প্রয়োগযোগ্য একটি হাদিস।"},"teachings":["নবী صلى الله عليه وسلم ওজুতে এক মুদ পরিমাণ পানি ব্যবহার করতেন।","গোসলের জন্য এক সা’ থেকে পাঁচ মুদ পর্যন্ত পানি ব্যবহারের বর্ণনা আছে।","পবিত্রতার কাজে পানির পরিমিত ব্যবহার শেখা যায়।","ওজু ও গোসল সহজ এবং অপচয়মুক্ত হওয়া উচিত।"],"related_hadiths":[{"id":"234","book_id":"1","label":"Sahih Bukhari"},{"id":"555","book_id":"2","label":"Sahih Muslim"},{"id":"159","book_id":"1","label":"Sahih Bukhari"}]}</t>
         </is>
       </c>
     </row>
@@ -2428,7 +2428,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মৃত্যুর পর চলমান তিন আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. মানুষ মারা গেলে আমল বন্ধ হয়, তবে সাদকায়ে জারিয়া, উপকারী জ্ঞান ও দোয়া করা সন্তান চলমান থাকে।"},"heading":{"title":"সাদকায়ে জারিয়া: মৃত্যুর পরও নেকী জারী থাকার হাদিস","description":"এই হাদিসে মৃত্যুর পর মানুষের আমল সম্পর্কে গুরুত্বপূর্ণ শিক্ষা এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, মানুষ মারা গেলে তার সব আমল বন্ধ হয়ে যায়। তবে তিনটি আমলের নেকী জারী থাকে—সাদকায়ে জারিয়া, ফলপ্রসূ ইলম এবং এমন সুসন্তান যে তার জন্য দোয়া করে। এখানে জীবনের দীর্ঘমেয়াদি প্রস্তুতির কথা বোঝা যায়। শুধু নিজের জন্য আমল করাই নয়, এমন কাজও করা দরকার যার উপকার মৃত্যুর পরও চলতে পারে। সাদকায়ে জারিয়া হাদিস, উপকারী জ্ঞান এবং সন্তানের দোয়া—এই তিনটি বিষয় মূল। এই হাদিস অতিরিক্ত আশা নয়; বরং দায়িত্ব শেখায়। মানুষকে এমন কাজের দিকে ডাকছে, যা অন্যের উপকারে আসে এবং নিজের জন্য নেকীর কারণ হতে পারে।"},"teachings":["মৃত্যুর পর সাধারণ আমল বন্ধ হয়ে যায়।","সাদকায়ে জারিয়া নেকী জারী থাকার একটি কারণ।","উপকারী জ্ঞান মানুষের জন্য চলমান কল্যাণ হতে পারে।","সুসন্তানের দোয়া মৃত ব্যক্তির জন্য উপকারী হতে পারে।"],"related_hadiths":[{"id":"2770","book_id":"1","label":"Sahih Bukhari"},{"id":"2৮৮0","book_id":"4","label":"Sunan Abu Dawud"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মৃত্যুর পর চলমান তিন আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. মানুষ মারা গেলে আমল বন্ধ হয়, তবে সাদকায়ে জারিয়া, উপকারী জ্ঞান ও দোয়া করা সন্তান চলমান থাকে।"},"heading":{"title":"সাদকায়ে জারিয়া: মৃত্যুর পরও নেকী জারী থাকার হাদিস","description":"এই হাদিসে মৃত্যুর পর মানুষের আমল সম্পর্কে গুরুত্বপূর্ণ শিক্ষা এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, মানুষ মারা গেলে তার সব আমল বন্ধ হয়ে যায়। তবে তিনটি আমলের নেকী জারী থাকে—সাদকায়ে জারিয়া, ফলপ্রসূ ইলম এবং এমন সুসন্তান যে তার জন্য দোয়া করে। এখানে জীবনের দীর্ঘমেয়াদি প্রস্তুতির কথা বোঝা যায়। শুধু নিজের জন্য আমল করাই নয়, এমন কাজও করা দরকার যার উপকার মৃত্যুর পরও চলতে পারে। সাদকায়ে জারিয়া হাদিস, উপকারী জ্ঞান এবং সন্তানের দোয়া—এই তিনটি বিষয় মূল। এই হাদিস অতিরিক্ত আশা নয়; বরং দায়িত্ব শেখায়। মানুষকে এমন কাজের দিকে ডাকছে, যা অন্যের উপকারে আসে এবং নিজের জন্য নেকীর কারণ হতে পারে।"},"teachings":["মৃত্যুর পর সাধারণ আমল বন্ধ হয়ে যায়।","সাদকায়ে জারিয়া নেকী জারী থাকার একটি কারণ।","উপকারী জ্ঞান মানুষের জন্য চলমান কল্যাণ হতে পারে।","সুসন্তানের দোয়া মৃত ব্যক্তির জন্য উপকারী হতে পারে।"],"related_hadiths":[{"id":"2770","book_id":"1","label":"Sahih Bukhari"},{"id":"2880","book_id":"4","label":"Sunan Abu Dawud"}]}</t>
         </is>
       </c>
     </row>
@@ -2538,7 +2538,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | যিলহজ্জের প্রথম দশকের আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. যিলহজ্জের প্রথম দশকে নেক আমলের বিশেষ মর্যাদা এবং জিহাদের প্রসঙ্গে ব্যতিক্রমী অবস্থার কথা এসেছে।"},"heading":{"title":"যিলহজ্জের প্রথম দশকের আমল: নেক কাজের বিশেষ সময়","description":"এই হাদিসে যিলহজ্জ মাসের প্রথম দশকের আমলের মর্যাদা এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, এই দিনগুলোতে যে আমল করা হয় তার চেয়ে উত্তম আর কোনো আমল নেই। সাহাবারা জিজ্ঞেস করলেন, জিহাদও কি উত্তম নয়? তিনি বললেন, জিহাদও উত্তম নয়। তবে সেই ব্যক্তির কথা আলাদা, যে নিজের জান ও মাল নিয়ে বের হয় এবং কিছুই নিয়ে ফিরে আসে না। এখানে যিলহজ্জের প্রথম দশক, নেক আমল এবং আমলের গুরুত্ব—এই তিনটি বিষয় প্রধান। এই হাদিস মানুষকে বিশেষ সময়ে বেশি ইবাদত ও ভালো কাজের প্রতি উৎসাহ দেয়। তবে বর্ণনায় যে ব্যতিক্রম এসেছে, সেটিও সতর্কভাবে বুঝতে হবে। মূল কথা হলো, এই দিনগুলো নেক কাজের জন্য বিশেষ সুযোগ।"},"teachings":["যিলহজ্জের প্রথম দশকে নেক আমলের বিশেষ মর্যাদা আছে।","সাহাবারা আমলের মর্যাদা বুঝতে প্রশ্ন করতেন।","জিহাদের প্রসঙ্গে হাদিসে একটি ব্যতিক্রমী অবস্থার কথা এসেছে।","বিশেষ সময়ে ভালো কাজের প্রতি বেশি মনোযোগ দেওয়া উচিত।"],"related_hadiths":[{"id":"1162","book_id":"2","label":"Sahih Muslim"},{"id":"243৮","book_id":"4","label":"Sunan Abu Dawud"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | যিলহজ্জের প্রথম দশকের আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. যিলহজ্জের প্রথম দশকে নেক আমলের বিশেষ মর্যাদা এবং জিহাদের প্রসঙ্গে ব্যতিক্রমী অবস্থার কথা এসেছে।"},"heading":{"title":"যিলহজ্জের প্রথম দশকের আমল: নেক কাজের বিশেষ সময়","description":"এই হাদিসে যিলহজ্জ মাসের প্রথম দশকের আমলের মর্যাদা এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, এই দিনগুলোতে যে আমল করা হয় তার চেয়ে উত্তম আর কোনো আমল নেই। সাহাবারা জিজ্ঞেস করলেন, জিহাদও কি উত্তম নয়? তিনি বললেন, জিহাদও উত্তম নয়। তবে সেই ব্যক্তির কথা আলাদা, যে নিজের জান ও মাল নিয়ে বের হয় এবং কিছুই নিয়ে ফিরে আসে না। এখানে যিলহজ্জের প্রথম দশক, নেক আমল এবং আমলের গুরুত্ব—এই তিনটি বিষয় প্রধান। এই হাদিস মানুষকে বিশেষ সময়ে বেশি ইবাদত ও ভালো কাজের প্রতি উৎসাহ দেয়। তবে বর্ণনায় যে ব্যতিক্রম এসেছে, সেটিও সতর্কভাবে বুঝতে হবে। মূল কথা হলো, এই দিনগুলো নেক কাজের জন্য বিশেষ সুযোগ।"},"teachings":["যিলহজ্জের প্রথম দশকে নেক আমলের বিশেষ মর্যাদা আছে।","সাহাবারা আমলের মর্যাদা বুঝতে প্রশ্ন করতেন।","জিহাদের প্রসঙ্গে হাদিসে একটি ব্যতিক্রমী অবস্থার কথা এসেছে।","বিশেষ সময়ে ভালো কাজের প্রতি বেশি মনোযোগ দেওয়া উচিত।"],"related_hadiths":[{"id":"1162","book_id":"2","label":"Sahih Muslim"},{"id":"2438","book_id":"4","label":"Sunan Abu Dawud"}]}</t>
         </is>
       </c>
     </row>
@@ -2582,7 +2582,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শোনা কথা ছড়ানোর সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. সব শোনা কথা বলে বেড়ানো মানুষকে মিথ্যাবাদী হওয়ার দিকে নিয়ে যেতে পারে—এ সতর্কতা এসেছে।"},"heading":{"title":"সব শোনা কথা বলা নয়: কথাবার্তায় সতর্কতার হাদিস","description":"এই হাদিসে কথাবার্তায় সতর্ক থাকার শিক্ষা এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, কোনো মানুষের মিথ্যাবাদী হওয়ার জন্য এতটুকুই যথেষ্ট যে, সে সব শোনা কথা বলে বেড়ায়। মানুষ অনেক সময় কোনো খবর যাচাই না করেই অন্যের কাছে বলে দেয়। এতে ভুল কথা ছড়িয়ে পড়ে এবং মিথ্যার দায় তৈরি হতে পারে। শোনা কথা বলা হাদিস, মিথ্যা থেকে বাঁচা এবং খবর যাচাই—এই বিষয়গুলো এখানে খুব গুরুত্বপূর্ণ। হাদিসটি আমাদের শেখায়, মুখের কথা হালকা বিষয় নয়। সব কথা বলা বুদ্ধিমানের কাজ নয়; বরং কোন কথা বলা উচিত আর কোন কথা থামিয়ে রাখা উচিত, তা বুঝতে হবে। একজন মুসলিমের কথায় সততা ও দায়িত্ব থাকা দরকার।"},"teachings":["যাচাই ছাড়া সব শোনা কথা বলা ঠিক নয়।","শোনা কথা ছড়ানো মিথ্যার কারণ হতে পারে।","কথাবার্তায় দায়িত্বশীল হওয়া জরুরি।","মুসলিমের জিহ্বা সততা ও সাবধানতার সঙ্গে ব্যবহার করা উচিত।"],"related_hadiths":[{"id":"60৯4","book_id":"1","label":"Sahih Bukhari"},{"id":"2607","book_id":"2","label":"Sahih Muslim"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শোনা কথা ছড়ানোর সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. সব শোনা কথা বলে বেড়ানো মানুষকে মিথ্যাবাদী হওয়ার দিকে নিয়ে যেতে পারে—এ সতর্কতা এসেছে।"},"heading":{"title":"সব শোনা কথা বলা নয়: কথাবার্তায় সতর্কতার হাদিস","description":"এই হাদিসে কথাবার্তায় সতর্ক থাকার শিক্ষা এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, কোনো মানুষের মিথ্যাবাদী হওয়ার জন্য এতটুকুই যথেষ্ট যে, সে সব শোনা কথা বলে বেড়ায়। মানুষ অনেক সময় কোনো খবর যাচাই না করেই অন্যের কাছে বলে দেয়। এতে ভুল কথা ছড়িয়ে পড়ে এবং মিথ্যার দায় তৈরি হতে পারে। শোনা কথা বলা হাদিস, মিথ্যা থেকে বাঁচা এবং খবর যাচাই—এই বিষয়গুলো এখানে খুব গুরুত্বপূর্ণ। হাদিসটি আমাদের শেখায়, মুখের কথা হালকা বিষয় নয়। সব কথা বলা বুদ্ধিমানের কাজ নয়; বরং কোন কথা বলা উচিত আর কোন কথা থামিয়ে রাখা উচিত, তা বুঝতে হবে। একজন মুসলিমের কথায় সততা ও দায়িত্ব থাকা দরকার।"},"teachings":["যাচাই ছাড়া সব শোনা কথা বলা ঠিক নয়।","শোনা কথা ছড়ানো মিথ্যার কারণ হতে পারে।","কথাবার্তায় দায়িত্বশীল হওয়া জরুরি।","মুসলিমের জিহ্বা সততা ও সাবধানতার সঙ্গে ব্যবহার করা উচিত।"],"related_hadiths":[{"id":"6094","book_id":"1","label":"Sahih Bukhari"},{"id":"2607","book_id":"2","label":"Sahih Muslim"}]}</t>
         </is>
       </c>
     </row>

</xml_diff>